<commit_message>
update: update XRO & cv
</commit_message>
<xml_diff>
--- a/content/climate/XRO/XRO_ENSO_fcst.xlsx
+++ b/content/climate/XRO/XRO_ENSO_fcst.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>init</t>
   </si>
@@ -117,6 +117,9 @@
   </si>
   <si>
     <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
   </si>
   <si>
     <t>Readme</t>
@@ -493,7 +496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U34"/>
+  <dimension ref="A1:U35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="21" width="10.7109375" style="1" customWidth="1"/>
@@ -501,7 +504,7 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B1" s="2">
         <v>0</v>
@@ -575,52 +578,52 @@
         <v>-0.731</v>
       </c>
       <c r="D2" s="1">
-        <v>-0.711</v>
+        <v>-0.712</v>
       </c>
       <c r="E2" s="1">
-        <v>-0.51</v>
+        <v>-0.511</v>
       </c>
       <c r="F2" s="1">
         <v>-0.148</v>
       </c>
       <c r="G2" s="1">
-        <v>0.258</v>
+        <v>0.26</v>
       </c>
       <c r="H2" s="1">
-        <v>0.5679999999999999</v>
+        <v>0.57</v>
       </c>
       <c r="I2" s="1">
-        <v>0.763</v>
+        <v>0.766</v>
       </c>
       <c r="J2" s="1">
-        <v>0.9409999999999999</v>
+        <v>0.945</v>
       </c>
       <c r="K2" s="1">
-        <v>1.213</v>
+        <v>1.217</v>
       </c>
       <c r="L2" s="1">
-        <v>1.564</v>
+        <v>1.569</v>
       </c>
       <c r="M2" s="1">
-        <v>1.829</v>
+        <v>1.834</v>
       </c>
       <c r="N2" s="1">
-        <v>1.885</v>
+        <v>1.889</v>
       </c>
       <c r="O2" s="1">
-        <v>1.755</v>
+        <v>1.759</v>
       </c>
       <c r="P2" s="1">
-        <v>1.507</v>
+        <v>1.51</v>
       </c>
       <c r="Q2" s="1">
-        <v>1.202</v>
+        <v>1.205</v>
       </c>
       <c r="R2" s="1">
-        <v>0.885</v>
+        <v>0.887</v>
       </c>
       <c r="S2" s="1">
-        <v>0.593</v>
+        <v>0.594</v>
       </c>
       <c r="T2" s="1">
         <v>0.356</v>
@@ -637,52 +640,52 @@
         <v>-0.473</v>
       </c>
       <c r="C3" s="1">
-        <v>-0.458</v>
+        <v>-0.459</v>
       </c>
       <c r="D3" s="1">
         <v>-0.314</v>
       </c>
       <c r="E3" s="1">
-        <v>-0.023</v>
+        <v>-0.022</v>
       </c>
       <c r="F3" s="1">
-        <v>0.292</v>
+        <v>0.294</v>
       </c>
       <c r="G3" s="1">
-        <v>0.522</v>
+        <v>0.526</v>
       </c>
       <c r="H3" s="1">
-        <v>0.661</v>
+        <v>0.665</v>
       </c>
       <c r="I3" s="1">
-        <v>0.781</v>
+        <v>0.785</v>
       </c>
       <c r="J3" s="1">
-        <v>0.954</v>
+        <v>0.959</v>
       </c>
       <c r="K3" s="1">
-        <v>1.171</v>
+        <v>1.177</v>
       </c>
       <c r="L3" s="1">
-        <v>1.326</v>
+        <v>1.332</v>
       </c>
       <c r="M3" s="1">
-        <v>1.336</v>
+        <v>1.342</v>
       </c>
       <c r="N3" s="1">
-        <v>1.215</v>
+        <v>1.221</v>
       </c>
       <c r="O3" s="1">
-        <v>1.027</v>
+        <v>1.032</v>
       </c>
       <c r="P3" s="1">
-        <v>0.8169999999999999</v>
+        <v>0.821</v>
       </c>
       <c r="Q3" s="1">
-        <v>0.593</v>
+        <v>0.596</v>
       </c>
       <c r="R3" s="1">
-        <v>0.373</v>
+        <v>0.374</v>
       </c>
       <c r="S3" s="1">
         <v>0.185</v>
@@ -691,7 +694,7 @@
         <v>0.047</v>
       </c>
       <c r="U3" s="1">
-        <v>-0.046</v>
+        <v>-0.047</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -702,52 +705,52 @@
         <v>-0.02</v>
       </c>
       <c r="C4" s="1">
-        <v>0.07000000000000001</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="D4" s="1">
-        <v>0.275</v>
+        <v>0.276</v>
       </c>
       <c r="E4" s="1">
-        <v>0.482</v>
+        <v>0.484</v>
       </c>
       <c r="F4" s="1">
-        <v>0.607</v>
+        <v>0.609</v>
       </c>
       <c r="G4" s="1">
-        <v>0.662</v>
+        <v>0.665</v>
       </c>
       <c r="H4" s="1">
-        <v>0.717</v>
+        <v>0.72</v>
       </c>
       <c r="I4" s="1">
-        <v>0.826</v>
+        <v>0.83</v>
       </c>
       <c r="J4" s="1">
-        <v>0.972</v>
+        <v>0.977</v>
       </c>
       <c r="K4" s="1">
-        <v>1.073</v>
+        <v>1.078</v>
       </c>
       <c r="L4" s="1">
-        <v>1.057</v>
+        <v>1.062</v>
       </c>
       <c r="M4" s="1">
-        <v>0.9379999999999999</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="N4" s="1">
-        <v>0.783</v>
+        <v>0.787</v>
       </c>
       <c r="O4" s="1">
-        <v>0.623</v>
+        <v>0.627</v>
       </c>
       <c r="P4" s="1">
-        <v>0.446</v>
+        <v>0.448</v>
       </c>
       <c r="Q4" s="1">
-        <v>0.253</v>
+        <v>0.255</v>
       </c>
       <c r="R4" s="1">
-        <v>0.078</v>
+        <v>0.079</v>
       </c>
       <c r="S4" s="1">
         <v>-0.055</v>
@@ -770,52 +773,52 @@
         <v>0.334</v>
       </c>
       <c r="D5" s="1">
-        <v>0.571</v>
+        <v>0.572</v>
       </c>
       <c r="E5" s="1">
-        <v>0.741</v>
+        <v>0.743</v>
       </c>
       <c r="F5" s="1">
-        <v>0.842</v>
+        <v>0.844</v>
       </c>
       <c r="G5" s="1">
-        <v>0.926</v>
+        <v>0.927</v>
       </c>
       <c r="H5" s="1">
-        <v>1.046</v>
+        <v>1.048</v>
       </c>
       <c r="I5" s="1">
-        <v>1.192</v>
+        <v>1.195</v>
       </c>
       <c r="J5" s="1">
-        <v>1.273</v>
+        <v>1.276</v>
       </c>
       <c r="K5" s="1">
-        <v>1.218</v>
+        <v>1.221</v>
       </c>
       <c r="L5" s="1">
-        <v>1.058</v>
+        <v>1.06</v>
       </c>
       <c r="M5" s="1">
-        <v>0.876</v>
+        <v>0.878</v>
       </c>
       <c r="N5" s="1">
-        <v>0.698</v>
+        <v>0.7</v>
       </c>
       <c r="O5" s="1">
-        <v>0.489</v>
+        <v>0.491</v>
       </c>
       <c r="P5" s="1">
-        <v>0.25</v>
+        <v>0.251</v>
       </c>
       <c r="Q5" s="1">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="R5" s="1">
         <v>-0.153</v>
       </c>
       <c r="S5" s="1">
-        <v>-0.27</v>
+        <v>-0.269</v>
       </c>
       <c r="T5" s="1">
         <v>-0.362</v>
@@ -835,58 +838,58 @@
         <v>0.626</v>
       </c>
       <c r="D6" s="1">
-        <v>0.842</v>
+        <v>0.843</v>
       </c>
       <c r="E6" s="1">
-        <v>0.965</v>
+        <v>0.966</v>
       </c>
       <c r="F6" s="1">
-        <v>1.056</v>
+        <v>1.057</v>
       </c>
       <c r="G6" s="1">
-        <v>1.183</v>
+        <v>1.184</v>
       </c>
       <c r="H6" s="1">
-        <v>1.328</v>
+        <v>1.33</v>
       </c>
       <c r="I6" s="1">
-        <v>1.393</v>
+        <v>1.395</v>
       </c>
       <c r="J6" s="1">
-        <v>1.308</v>
+        <v>1.311</v>
       </c>
       <c r="K6" s="1">
-        <v>1.118</v>
+        <v>1.12</v>
       </c>
       <c r="L6" s="1">
-        <v>0.916</v>
+        <v>0.918</v>
       </c>
       <c r="M6" s="1">
-        <v>0.725</v>
+        <v>0.727</v>
       </c>
       <c r="N6" s="1">
-        <v>0.501</v>
+        <v>0.502</v>
       </c>
       <c r="O6" s="1">
-        <v>0.241</v>
+        <v>0.242</v>
       </c>
       <c r="P6" s="1">
-        <v>-0.008</v>
+        <v>-0.007</v>
       </c>
       <c r="Q6" s="1">
-        <v>-0.201</v>
+        <v>-0.2</v>
       </c>
       <c r="R6" s="1">
-        <v>-0.327</v>
+        <v>-0.326</v>
       </c>
       <c r="S6" s="1">
-        <v>-0.427</v>
+        <v>-0.426</v>
       </c>
       <c r="T6" s="1">
-        <v>-0.537</v>
+        <v>-0.536</v>
       </c>
       <c r="U6" s="1">
-        <v>-0.639</v>
+        <v>-0.638</v>
       </c>
     </row>
     <row r="7" spans="1:21">
@@ -903,52 +906,52 @@
         <v>1.129</v>
       </c>
       <c r="E7" s="1">
-        <v>1.223</v>
+        <v>1.224</v>
       </c>
       <c r="F7" s="1">
-        <v>1.344</v>
+        <v>1.346</v>
       </c>
       <c r="G7" s="1">
-        <v>1.461</v>
+        <v>1.464</v>
       </c>
       <c r="H7" s="1">
-        <v>1.481</v>
+        <v>1.484</v>
       </c>
       <c r="I7" s="1">
-        <v>1.357</v>
+        <v>1.36</v>
       </c>
       <c r="J7" s="1">
-        <v>1.141</v>
+        <v>1.145</v>
       </c>
       <c r="K7" s="1">
-        <v>0.926</v>
+        <v>0.929</v>
       </c>
       <c r="L7" s="1">
-        <v>0.717</v>
+        <v>0.72</v>
       </c>
       <c r="M7" s="1">
-        <v>0.457</v>
+        <v>0.459</v>
       </c>
       <c r="N7" s="1">
-        <v>0.151</v>
+        <v>0.152</v>
       </c>
       <c r="O7" s="1">
-        <v>-0.139</v>
+        <v>-0.138</v>
       </c>
       <c r="P7" s="1">
-        <v>-0.352</v>
+        <v>-0.351</v>
       </c>
       <c r="Q7" s="1">
-        <v>-0.478</v>
+        <v>-0.477</v>
       </c>
       <c r="R7" s="1">
-        <v>-0.582</v>
+        <v>-0.581</v>
       </c>
       <c r="S7" s="1">
-        <v>-0.712</v>
+        <v>-0.711</v>
       </c>
       <c r="T7" s="1">
-        <v>-0.841</v>
+        <v>-0.84</v>
       </c>
       <c r="U7" s="1">
         <v>-0.895</v>
@@ -962,52 +965,52 @@
         <v>1.051</v>
       </c>
       <c r="C8" s="1">
-        <v>1.163</v>
+        <v>1.164</v>
       </c>
       <c r="D8" s="1">
-        <v>1.331</v>
+        <v>1.332</v>
       </c>
       <c r="E8" s="1">
-        <v>1.482</v>
+        <v>1.484</v>
       </c>
       <c r="F8" s="1">
-        <v>1.574</v>
+        <v>1.578</v>
       </c>
       <c r="G8" s="1">
-        <v>1.534</v>
+        <v>1.538</v>
       </c>
       <c r="H8" s="1">
-        <v>1.347</v>
+        <v>1.351</v>
       </c>
       <c r="I8" s="1">
-        <v>1.093</v>
+        <v>1.097</v>
       </c>
       <c r="J8" s="1">
-        <v>0.868</v>
+        <v>0.872</v>
       </c>
       <c r="K8" s="1">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="L8" s="1">
-        <v>0.387</v>
+        <v>0.389</v>
       </c>
       <c r="M8" s="1">
-        <v>0.055</v>
+        <v>0.057</v>
       </c>
       <c r="N8" s="1">
-        <v>-0.259</v>
+        <v>-0.258</v>
       </c>
       <c r="O8" s="1">
-        <v>-0.479</v>
+        <v>-0.478</v>
       </c>
       <c r="P8" s="1">
-        <v>-0.599</v>
+        <v>-0.598</v>
       </c>
       <c r="Q8" s="1">
-        <v>-0.703</v>
+        <v>-0.702</v>
       </c>
       <c r="R8" s="1">
-        <v>-0.85</v>
+        <v>-0.849</v>
       </c>
       <c r="S8" s="1">
         <v>-1.004</v>
@@ -1030,40 +1033,40 @@
         <v>1.447</v>
       </c>
       <c r="D9" s="1">
-        <v>1.66</v>
+        <v>1.661</v>
       </c>
       <c r="E9" s="1">
-        <v>1.759</v>
+        <v>1.762</v>
       </c>
       <c r="F9" s="1">
-        <v>1.683</v>
+        <v>1.687</v>
       </c>
       <c r="G9" s="1">
-        <v>1.462</v>
+        <v>1.466</v>
       </c>
       <c r="H9" s="1">
-        <v>1.192</v>
+        <v>1.196</v>
       </c>
       <c r="I9" s="1">
-        <v>0.955</v>
+        <v>0.958</v>
       </c>
       <c r="J9" s="1">
-        <v>0.715</v>
+        <v>0.718</v>
       </c>
       <c r="K9" s="1">
-        <v>0.393</v>
+        <v>0.395</v>
       </c>
       <c r="L9" s="1">
-        <v>0.008999999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="M9" s="1">
-        <v>-0.346</v>
+        <v>-0.345</v>
       </c>
       <c r="N9" s="1">
         <v>-0.584</v>
       </c>
       <c r="O9" s="1">
-        <v>-0.703</v>
+        <v>-0.702</v>
       </c>
       <c r="P9" s="1">
         <v>-0.8070000000000001</v>
@@ -1075,13 +1078,13 @@
         <v>-1.144</v>
       </c>
       <c r="S9" s="1">
-        <v>-1.217</v>
+        <v>-1.218</v>
       </c>
       <c r="T9" s="1">
-        <v>-1.122</v>
+        <v>-1.123</v>
       </c>
       <c r="U9" s="1">
-        <v>-0.9330000000000001</v>
+        <v>-0.9340000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:21">
@@ -1092,43 +1095,43 @@
         <v>1.555</v>
       </c>
       <c r="C10" s="1">
-        <v>1.696</v>
+        <v>1.697</v>
       </c>
       <c r="D10" s="1">
-        <v>1.857</v>
+        <v>1.859</v>
       </c>
       <c r="E10" s="1">
-        <v>1.822</v>
+        <v>1.824</v>
       </c>
       <c r="F10" s="1">
-        <v>1.61</v>
+        <v>1.613</v>
       </c>
       <c r="G10" s="1">
-        <v>1.332</v>
+        <v>1.335</v>
       </c>
       <c r="H10" s="1">
-        <v>1.075</v>
+        <v>1.078</v>
       </c>
       <c r="I10" s="1">
-        <v>0.8149999999999999</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="J10" s="1">
-        <v>0.481</v>
+        <v>0.483</v>
       </c>
       <c r="K10" s="1">
-        <v>0.093</v>
+        <v>0.095</v>
       </c>
       <c r="L10" s="1">
-        <v>-0.263</v>
+        <v>-0.262</v>
       </c>
       <c r="M10" s="1">
-        <v>-0.507</v>
+        <v>-0.506</v>
       </c>
       <c r="N10" s="1">
-        <v>-0.636</v>
+        <v>-0.635</v>
       </c>
       <c r="O10" s="1">
-        <v>-0.743</v>
+        <v>-0.742</v>
       </c>
       <c r="P10" s="1">
         <v>-0.896</v>
@@ -1157,58 +1160,58 @@
         <v>1.596</v>
       </c>
       <c r="C11" s="1">
-        <v>1.722</v>
+        <v>1.723</v>
       </c>
       <c r="D11" s="1">
-        <v>1.797</v>
+        <v>1.798</v>
       </c>
       <c r="E11" s="1">
-        <v>1.647</v>
+        <v>1.649</v>
       </c>
       <c r="F11" s="1">
-        <v>1.392</v>
+        <v>1.393</v>
       </c>
       <c r="G11" s="1">
-        <v>1.132</v>
+        <v>1.134</v>
       </c>
       <c r="H11" s="1">
-        <v>0.865</v>
+        <v>0.866</v>
       </c>
       <c r="I11" s="1">
-        <v>0.539</v>
+        <v>0.54</v>
       </c>
       <c r="J11" s="1">
-        <v>0.175</v>
+        <v>0.176</v>
       </c>
       <c r="K11" s="1">
-        <v>-0.155</v>
+        <v>-0.154</v>
       </c>
       <c r="L11" s="1">
-        <v>-0.385</v>
+        <v>-0.383</v>
       </c>
       <c r="M11" s="1">
-        <v>-0.514</v>
+        <v>-0.512</v>
       </c>
       <c r="N11" s="1">
-        <v>-0.618</v>
+        <v>-0.616</v>
       </c>
       <c r="O11" s="1">
-        <v>-0.751</v>
+        <v>-0.749</v>
       </c>
       <c r="P11" s="1">
-        <v>-0.886</v>
+        <v>-0.884</v>
       </c>
       <c r="Q11" s="1">
-        <v>-0.9409999999999999</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="R11" s="1">
-        <v>-0.867</v>
+        <v>-0.866</v>
       </c>
       <c r="S11" s="1">
         <v>-0.718</v>
       </c>
       <c r="T11" s="1">
-        <v>-0.582</v>
+        <v>-0.581</v>
       </c>
       <c r="U11" s="1">
         <v>-0.49</v>
@@ -1225,49 +1228,49 @@
         <v>1.843</v>
       </c>
       <c r="D12" s="1">
-        <v>1.666</v>
+        <v>1.667</v>
       </c>
       <c r="E12" s="1">
-        <v>1.418</v>
+        <v>1.419</v>
       </c>
       <c r="F12" s="1">
-        <v>1.159</v>
+        <v>1.16</v>
       </c>
       <c r="G12" s="1">
-        <v>0.863</v>
+        <v>0.864</v>
       </c>
       <c r="H12" s="1">
-        <v>0.489</v>
+        <v>0.49</v>
       </c>
       <c r="I12" s="1">
-        <v>0.075</v>
+        <v>0.076</v>
       </c>
       <c r="J12" s="1">
-        <v>-0.292</v>
+        <v>-0.291</v>
       </c>
       <c r="K12" s="1">
-        <v>-0.537</v>
+        <v>-0.535</v>
       </c>
       <c r="L12" s="1">
-        <v>-0.666</v>
+        <v>-0.664</v>
       </c>
       <c r="M12" s="1">
-        <v>-0.775</v>
+        <v>-0.773</v>
       </c>
       <c r="N12" s="1">
-        <v>-0.929</v>
+        <v>-0.927</v>
       </c>
       <c r="O12" s="1">
-        <v>-1.09</v>
+        <v>-1.089</v>
       </c>
       <c r="P12" s="1">
-        <v>-1.155</v>
+        <v>-1.154</v>
       </c>
       <c r="Q12" s="1">
         <v>-1.061</v>
       </c>
       <c r="R12" s="1">
-        <v>-0.88</v>
+        <v>-0.879</v>
       </c>
       <c r="S12" s="1">
         <v>-0.715</v>
@@ -1276,7 +1279,7 @@
         <v>-0.603</v>
       </c>
       <c r="U12" s="1">
-        <v>-0.53</v>
+        <v>-0.529</v>
       </c>
     </row>
     <row r="13" spans="1:21">
@@ -1290,34 +1293,34 @@
         <v>1.859</v>
       </c>
       <c r="D13" s="1">
-        <v>1.592</v>
+        <v>1.593</v>
       </c>
       <c r="E13" s="1">
-        <v>1.295</v>
+        <v>1.296</v>
       </c>
       <c r="F13" s="1">
-        <v>0.956</v>
+        <v>0.957</v>
       </c>
       <c r="G13" s="1">
-        <v>0.534</v>
+        <v>0.535</v>
       </c>
       <c r="H13" s="1">
-        <v>0.067</v>
+        <v>0.068</v>
       </c>
       <c r="I13" s="1">
-        <v>-0.353</v>
+        <v>-0.352</v>
       </c>
       <c r="J13" s="1">
-        <v>-0.642</v>
+        <v>-0.641</v>
       </c>
       <c r="K13" s="1">
-        <v>-0.794</v>
+        <v>-0.793</v>
       </c>
       <c r="L13" s="1">
-        <v>-0.917</v>
+        <v>-0.916</v>
       </c>
       <c r="M13" s="1">
-        <v>-1.089</v>
+        <v>-1.088</v>
       </c>
       <c r="N13" s="1">
         <v>-1.271</v>
@@ -1329,19 +1332,19 @@
         <v>-1.244</v>
       </c>
       <c r="Q13" s="1">
-        <v>-1.036</v>
+        <v>-1.037</v>
       </c>
       <c r="R13" s="1">
-        <v>-0.841</v>
+        <v>-0.842</v>
       </c>
       <c r="S13" s="1">
-        <v>-0.702</v>
+        <v>-0.703</v>
       </c>
       <c r="T13" s="1">
         <v>-0.609</v>
       </c>
       <c r="U13" s="1">
-        <v>-0.548</v>
+        <v>-0.547</v>
       </c>
     </row>
     <row r="14" spans="1:21">
@@ -1358,28 +1361,28 @@
         <v>1.389</v>
       </c>
       <c r="E14" s="1">
-        <v>0.989</v>
+        <v>0.99</v>
       </c>
       <c r="F14" s="1">
-        <v>0.472</v>
+        <v>0.473</v>
       </c>
       <c r="G14" s="1">
-        <v>-0.08500000000000001</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="H14" s="1">
-        <v>-0.5679999999999999</v>
+        <v>-0.5659999999999999</v>
       </c>
       <c r="I14" s="1">
-        <v>-0.863</v>
+        <v>-0.861</v>
       </c>
       <c r="J14" s="1">
-        <v>-0.982</v>
+        <v>-0.98</v>
       </c>
       <c r="K14" s="1">
-        <v>-1.081</v>
+        <v>-1.08</v>
       </c>
       <c r="L14" s="1">
-        <v>-1.261</v>
+        <v>-1.26</v>
       </c>
       <c r="M14" s="1">
         <v>-1.467</v>
@@ -1391,10 +1394,10 @@
         <v>-1.408</v>
       </c>
       <c r="P14" s="1">
-        <v>-1.159</v>
+        <v>-1.16</v>
       </c>
       <c r="Q14" s="1">
-        <v>-0.948</v>
+        <v>-0.949</v>
       </c>
       <c r="R14" s="1">
         <v>-0.8139999999999999</v>
@@ -1406,7 +1409,7 @@
         <v>-0.672</v>
       </c>
       <c r="U14" s="1">
-        <v>-0.621</v>
+        <v>-0.62</v>
       </c>
     </row>
     <row r="15" spans="1:21">
@@ -1417,10 +1420,10 @@
         <v>1.537</v>
       </c>
       <c r="C15" s="1">
-        <v>1.358</v>
+        <v>1.359</v>
       </c>
       <c r="D15" s="1">
-        <v>0.986</v>
+        <v>0.987</v>
       </c>
       <c r="E15" s="1">
         <v>0.498</v>
@@ -1429,49 +1432,49 @@
         <v>-0.057</v>
       </c>
       <c r="G15" s="1">
-        <v>-0.5629999999999999</v>
+        <v>-0.5620000000000001</v>
       </c>
       <c r="H15" s="1">
-        <v>-0.889</v>
+        <v>-0.888</v>
       </c>
       <c r="I15" s="1">
-        <v>-1.024</v>
+        <v>-1.023</v>
       </c>
       <c r="J15" s="1">
-        <v>-1.13</v>
+        <v>-1.129</v>
       </c>
       <c r="K15" s="1">
         <v>-1.319</v>
       </c>
       <c r="L15" s="1">
-        <v>-1.54</v>
+        <v>-1.541</v>
       </c>
       <c r="M15" s="1">
-        <v>-1.632</v>
+        <v>-1.634</v>
       </c>
       <c r="N15" s="1">
-        <v>-1.499</v>
+        <v>-1.501</v>
       </c>
       <c r="O15" s="1">
-        <v>-1.241</v>
+        <v>-1.242</v>
       </c>
       <c r="P15" s="1">
-        <v>-1.014</v>
+        <v>-1.016</v>
       </c>
       <c r="Q15" s="1">
-        <v>-0.871</v>
+        <v>-0.873</v>
       </c>
       <c r="R15" s="1">
-        <v>-0.789</v>
+        <v>-0.79</v>
       </c>
       <c r="S15" s="1">
-        <v>-0.738</v>
+        <v>-0.737</v>
       </c>
       <c r="T15" s="1">
-        <v>-0.694</v>
+        <v>-0.6929999999999999</v>
       </c>
       <c r="U15" s="1">
-        <v>-0.656</v>
+        <v>-0.655</v>
       </c>
     </row>
     <row r="16" spans="1:21">
@@ -1485,22 +1488,22 @@
         <v>0.996</v>
       </c>
       <c r="D16" s="1">
-        <v>0.534</v>
+        <v>0.535</v>
       </c>
       <c r="E16" s="1">
-        <v>0.018</v>
+        <v>0.019</v>
       </c>
       <c r="F16" s="1">
-        <v>-0.453</v>
+        <v>-0.452</v>
       </c>
       <c r="G16" s="1">
-        <v>-0.765</v>
+        <v>-0.764</v>
       </c>
       <c r="H16" s="1">
-        <v>-0.903</v>
+        <v>-0.902</v>
       </c>
       <c r="I16" s="1">
-        <v>-1.004</v>
+        <v>-1.003</v>
       </c>
       <c r="J16" s="1">
         <v>-1.171</v>
@@ -1509,34 +1512,34 @@
         <v>-1.368</v>
       </c>
       <c r="L16" s="1">
-        <v>-1.46</v>
+        <v>-1.461</v>
       </c>
       <c r="M16" s="1">
-        <v>-1.353</v>
+        <v>-1.355</v>
       </c>
       <c r="N16" s="1">
-        <v>-1.126</v>
+        <v>-1.127</v>
       </c>
       <c r="O16" s="1">
-        <v>-0.915</v>
+        <v>-0.916</v>
       </c>
       <c r="P16" s="1">
-        <v>-0.773</v>
+        <v>-0.774</v>
       </c>
       <c r="Q16" s="1">
         <v>-0.6889999999999999</v>
       </c>
       <c r="R16" s="1">
-        <v>-0.64</v>
+        <v>-0.639</v>
       </c>
       <c r="S16" s="1">
-        <v>-0.605</v>
+        <v>-0.603</v>
       </c>
       <c r="T16" s="1">
-        <v>-0.576</v>
+        <v>-0.575</v>
       </c>
       <c r="U16" s="1">
-        <v>-0.574</v>
+        <v>-0.573</v>
       </c>
     </row>
     <row r="17" spans="1:21">
@@ -1553,55 +1556,55 @@
         <v>0.075</v>
       </c>
       <c r="E17" s="1">
-        <v>-0.385</v>
+        <v>-0.384</v>
       </c>
       <c r="F17" s="1">
-        <v>-0.697</v>
+        <v>-0.696</v>
       </c>
       <c r="G17" s="1">
-        <v>-0.847</v>
+        <v>-0.846</v>
       </c>
       <c r="H17" s="1">
-        <v>-0.959</v>
+        <v>-0.958</v>
       </c>
       <c r="I17" s="1">
         <v>-1.127</v>
       </c>
       <c r="J17" s="1">
-        <v>-1.319</v>
+        <v>-1.32</v>
       </c>
       <c r="K17" s="1">
-        <v>-1.411</v>
+        <v>-1.413</v>
       </c>
       <c r="L17" s="1">
-        <v>-1.313</v>
+        <v>-1.314</v>
       </c>
       <c r="M17" s="1">
-        <v>-1.093</v>
+        <v>-1.095</v>
       </c>
       <c r="N17" s="1">
-        <v>-0.884</v>
+        <v>-0.886</v>
       </c>
       <c r="O17" s="1">
-        <v>-0.74</v>
+        <v>-0.741</v>
       </c>
       <c r="P17" s="1">
         <v>-0.654</v>
       </c>
       <c r="Q17" s="1">
-        <v>-0.607</v>
+        <v>-0.606</v>
       </c>
       <c r="R17" s="1">
-        <v>-0.578</v>
+        <v>-0.577</v>
       </c>
       <c r="S17" s="1">
-        <v>-0.5570000000000001</v>
+        <v>-0.555</v>
       </c>
       <c r="T17" s="1">
-        <v>-0.5570000000000001</v>
+        <v>-0.555</v>
       </c>
       <c r="U17" s="1">
-        <v>-0.585</v>
+        <v>-0.583</v>
       </c>
     </row>
     <row r="18" spans="1:21">
@@ -1615,13 +1618,13 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="D18" s="1">
-        <v>-0.469</v>
+        <v>-0.468</v>
       </c>
       <c r="E18" s="1">
-        <v>-0.789</v>
+        <v>-0.787</v>
       </c>
       <c r="F18" s="1">
-        <v>-0.9370000000000001</v>
+        <v>-0.9360000000000001</v>
       </c>
       <c r="G18" s="1">
         <v>-1.042</v>
@@ -1630,22 +1633,22 @@
         <v>-1.204</v>
       </c>
       <c r="I18" s="1">
-        <v>-1.384</v>
+        <v>-1.385</v>
       </c>
       <c r="J18" s="1">
-        <v>-1.463</v>
+        <v>-1.464</v>
       </c>
       <c r="K18" s="1">
-        <v>-1.358</v>
+        <v>-1.359</v>
       </c>
       <c r="L18" s="1">
-        <v>-1.139</v>
+        <v>-1.14</v>
       </c>
       <c r="M18" s="1">
-        <v>-0.925</v>
+        <v>-0.926</v>
       </c>
       <c r="N18" s="1">
-        <v>-0.761</v>
+        <v>-0.762</v>
       </c>
       <c r="O18" s="1">
         <v>-0.642</v>
@@ -1654,19 +1657,19 @@
         <v>-0.5639999999999999</v>
       </c>
       <c r="Q18" s="1">
-        <v>-0.519</v>
+        <v>-0.518</v>
       </c>
       <c r="R18" s="1">
-        <v>-0.49</v>
+        <v>-0.488</v>
       </c>
       <c r="S18" s="1">
-        <v>-0.48</v>
+        <v>-0.478</v>
       </c>
       <c r="T18" s="1">
+        <v>-0.487</v>
+      </c>
+      <c r="U18" s="1">
         <v>-0.489</v>
-      </c>
-      <c r="U18" s="1">
-        <v>-0.492</v>
       </c>
     </row>
     <row r="19" spans="1:21">
@@ -1677,22 +1680,22 @@
         <v>0.252</v>
       </c>
       <c r="C19" s="1">
-        <v>0.023</v>
+        <v>0.024</v>
       </c>
       <c r="D19" s="1">
-        <v>-0.302</v>
+        <v>-0.301</v>
       </c>
       <c r="E19" s="1">
-        <v>-0.497</v>
+        <v>-0.496</v>
       </c>
       <c r="F19" s="1">
-        <v>-0.649</v>
+        <v>-0.648</v>
       </c>
       <c r="G19" s="1">
-        <v>-0.823</v>
+        <v>-0.822</v>
       </c>
       <c r="H19" s="1">
-        <v>-0.99</v>
+        <v>-0.989</v>
       </c>
       <c r="I19" s="1">
         <v>-1.064</v>
@@ -1710,28 +1713,28 @@
         <v>-0.569</v>
       </c>
       <c r="N19" s="1">
-        <v>-0.549</v>
+        <v>-0.548</v>
       </c>
       <c r="O19" s="1">
-        <v>-0.5610000000000001</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="P19" s="1">
-        <v>-0.569</v>
+        <v>-0.5679999999999999</v>
       </c>
       <c r="Q19" s="1">
-        <v>-0.5659999999999999</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="R19" s="1">
-        <v>-0.581</v>
+        <v>-0.579</v>
       </c>
       <c r="S19" s="1">
-        <v>-0.629</v>
+        <v>-0.627</v>
       </c>
       <c r="T19" s="1">
-        <v>-0.676</v>
+        <v>-0.673</v>
       </c>
       <c r="U19" s="1">
-        <v>-0.6820000000000001</v>
+        <v>-0.679</v>
       </c>
     </row>
     <row r="20" spans="1:21">
@@ -1745,58 +1748,58 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="D20" s="1">
-        <v>-0.116</v>
+        <v>-0.115</v>
       </c>
       <c r="E20" s="1">
-        <v>-0.285</v>
+        <v>-0.284</v>
       </c>
       <c r="F20" s="1">
-        <v>-0.452</v>
+        <v>-0.451</v>
       </c>
       <c r="G20" s="1">
-        <v>-0.588</v>
+        <v>-0.586</v>
       </c>
       <c r="H20" s="1">
-        <v>-0.646</v>
+        <v>-0.645</v>
       </c>
       <c r="I20" s="1">
-        <v>-0.598</v>
+        <v>-0.596</v>
       </c>
       <c r="J20" s="1">
-        <v>-0.482</v>
+        <v>-0.481</v>
       </c>
       <c r="K20" s="1">
         <v>-0.382</v>
       </c>
       <c r="L20" s="1">
-        <v>-0.351</v>
+        <v>-0.35</v>
       </c>
       <c r="M20" s="1">
-        <v>-0.382</v>
+        <v>-0.381</v>
       </c>
       <c r="N20" s="1">
-        <v>-0.44</v>
+        <v>-0.438</v>
       </c>
       <c r="O20" s="1">
-        <v>-0.483</v>
+        <v>-0.481</v>
       </c>
       <c r="P20" s="1">
-        <v>-0.504</v>
+        <v>-0.502</v>
       </c>
       <c r="Q20" s="1">
-        <v>-0.535</v>
+        <v>-0.532</v>
       </c>
       <c r="R20" s="1">
-        <v>-0.592</v>
+        <v>-0.589</v>
       </c>
       <c r="S20" s="1">
-        <v>-0.646</v>
+        <v>-0.643</v>
       </c>
       <c r="T20" s="1">
-        <v>-0.659</v>
+        <v>-0.656</v>
       </c>
       <c r="U20" s="1">
-        <v>-0.622</v>
+        <v>-0.619</v>
       </c>
     </row>
     <row r="21" spans="1:21">
@@ -1813,55 +1816,55 @@
         <v>-0.241</v>
       </c>
       <c r="E21" s="1">
-        <v>-0.395</v>
+        <v>-0.394</v>
       </c>
       <c r="F21" s="1">
-        <v>-0.541</v>
+        <v>-0.54</v>
       </c>
       <c r="G21" s="1">
-        <v>-0.619</v>
+        <v>-0.618</v>
       </c>
       <c r="H21" s="1">
-        <v>-0.584</v>
+        <v>-0.583</v>
       </c>
       <c r="I21" s="1">
         <v>-0.471</v>
       </c>
       <c r="J21" s="1">
-        <v>-0.376</v>
+        <v>-0.375</v>
       </c>
       <c r="K21" s="1">
-        <v>-0.359</v>
+        <v>-0.358</v>
       </c>
       <c r="L21" s="1">
-        <v>-0.412</v>
+        <v>-0.411</v>
       </c>
       <c r="M21" s="1">
-        <v>-0.489</v>
+        <v>-0.488</v>
       </c>
       <c r="N21" s="1">
-        <v>-0.543</v>
+        <v>-0.541</v>
       </c>
       <c r="O21" s="1">
-        <v>-0.5679999999999999</v>
+        <v>-0.5659999999999999</v>
       </c>
       <c r="P21" s="1">
-        <v>-0.605</v>
+        <v>-0.603</v>
       </c>
       <c r="Q21" s="1">
-        <v>-0.677</v>
+        <v>-0.674</v>
       </c>
       <c r="R21" s="1">
-        <v>-0.748</v>
+        <v>-0.745</v>
       </c>
       <c r="S21" s="1">
-        <v>-0.769</v>
+        <v>-0.766</v>
       </c>
       <c r="T21" s="1">
-        <v>-0.724</v>
+        <v>-0.722</v>
       </c>
       <c r="U21" s="1">
-        <v>-0.632</v>
+        <v>-0.63</v>
       </c>
     </row>
     <row r="22" spans="1:21">
@@ -1872,7 +1875,7 @@
         <v>-0.217</v>
       </c>
       <c r="C22" s="1">
-        <v>-0.287</v>
+        <v>-0.286</v>
       </c>
       <c r="D22" s="1">
         <v>-0.433</v>
@@ -1884,49 +1887,49 @@
         <v>-0.676</v>
       </c>
       <c r="G22" s="1">
-        <v>-0.647</v>
+        <v>-0.646</v>
       </c>
       <c r="H22" s="1">
         <v>-0.526</v>
       </c>
       <c r="I22" s="1">
-        <v>-0.419</v>
+        <v>-0.42</v>
       </c>
       <c r="J22" s="1">
         <v>-0.396</v>
       </c>
       <c r="K22" s="1">
-        <v>-0.451</v>
+        <v>-0.45</v>
       </c>
       <c r="L22" s="1">
-        <v>-0.531</v>
+        <v>-0.53</v>
       </c>
       <c r="M22" s="1">
-        <v>-0.587</v>
+        <v>-0.585</v>
       </c>
       <c r="N22" s="1">
-        <v>-0.611</v>
+        <v>-0.609</v>
       </c>
       <c r="O22" s="1">
-        <v>-0.649</v>
+        <v>-0.647</v>
       </c>
       <c r="P22" s="1">
-        <v>-0.726</v>
+        <v>-0.724</v>
       </c>
       <c r="Q22" s="1">
-        <v>-0.803</v>
+        <v>-0.801</v>
       </c>
       <c r="R22" s="1">
-        <v>-0.826</v>
+        <v>-0.823</v>
       </c>
       <c r="S22" s="1">
-        <v>-0.778</v>
+        <v>-0.775</v>
       </c>
       <c r="T22" s="1">
-        <v>-0.679</v>
+        <v>-0.677</v>
       </c>
       <c r="U22" s="1">
-        <v>-0.549</v>
+        <v>-0.548</v>
       </c>
     </row>
     <row r="23" spans="1:21">
@@ -1940,7 +1943,7 @@
         <v>-0.412</v>
       </c>
       <c r="D23" s="1">
-        <v>-0.586</v>
+        <v>-0.585</v>
       </c>
       <c r="E23" s="1">
         <v>-0.646</v>
@@ -1958,40 +1961,40 @@
         <v>-0.343</v>
       </c>
       <c r="J23" s="1">
-        <v>-0.426</v>
+        <v>-0.425</v>
       </c>
       <c r="K23" s="1">
-        <v>-0.524</v>
+        <v>-0.523</v>
       </c>
       <c r="L23" s="1">
-        <v>-0.584</v>
+        <v>-0.582</v>
       </c>
       <c r="M23" s="1">
-        <v>-0.606</v>
+        <v>-0.604</v>
       </c>
       <c r="N23" s="1">
-        <v>-0.641</v>
+        <v>-0.639</v>
       </c>
       <c r="O23" s="1">
-        <v>-0.715</v>
+        <v>-0.712</v>
       </c>
       <c r="P23" s="1">
-        <v>-0.788</v>
+        <v>-0.785</v>
       </c>
       <c r="Q23" s="1">
-        <v>-0.806</v>
+        <v>-0.803</v>
       </c>
       <c r="R23" s="1">
-        <v>-0.752</v>
+        <v>-0.75</v>
       </c>
       <c r="S23" s="1">
-        <v>-0.651</v>
+        <v>-0.649</v>
       </c>
       <c r="T23" s="1">
-        <v>-0.525</v>
+        <v>-0.523</v>
       </c>
       <c r="U23" s="1">
-        <v>-0.376</v>
+        <v>-0.375</v>
       </c>
     </row>
     <row r="24" spans="1:21">
@@ -2005,58 +2008,58 @@
         <v>-0.183</v>
       </c>
       <c r="D24" s="1">
-        <v>-0.277</v>
+        <v>-0.276</v>
       </c>
       <c r="E24" s="1">
-        <v>-0.266</v>
+        <v>-0.265</v>
       </c>
       <c r="F24" s="1">
         <v>-0.192</v>
       </c>
       <c r="G24" s="1">
-        <v>-0.147</v>
+        <v>-0.146</v>
       </c>
       <c r="H24" s="1">
-        <v>-0.187</v>
+        <v>-0.186</v>
       </c>
       <c r="I24" s="1">
-        <v>-0.297</v>
+        <v>-0.295</v>
       </c>
       <c r="J24" s="1">
-        <v>-0.42</v>
+        <v>-0.417</v>
       </c>
       <c r="K24" s="1">
-        <v>-0.501</v>
+        <v>-0.498</v>
       </c>
       <c r="L24" s="1">
-        <v>-0.539</v>
+        <v>-0.536</v>
       </c>
       <c r="M24" s="1">
-        <v>-0.584</v>
+        <v>-0.581</v>
       </c>
       <c r="N24" s="1">
-        <v>-0.665</v>
+        <v>-0.662</v>
       </c>
       <c r="O24" s="1">
-        <v>-0.747</v>
+        <v>-0.743</v>
       </c>
       <c r="P24" s="1">
-        <v>-0.77</v>
+        <v>-0.766</v>
       </c>
       <c r="Q24" s="1">
-        <v>-0.717</v>
+        <v>-0.713</v>
       </c>
       <c r="R24" s="1">
-        <v>-0.615</v>
+        <v>-0.612</v>
       </c>
       <c r="S24" s="1">
-        <v>-0.497</v>
+        <v>-0.495</v>
       </c>
       <c r="T24" s="1">
-        <v>-0.372</v>
+        <v>-0.37</v>
       </c>
       <c r="U24" s="1">
-        <v>-0.247</v>
+        <v>-0.245</v>
       </c>
     </row>
     <row r="25" spans="1:21">
@@ -2082,46 +2085,46 @@
         <v>-0.282</v>
       </c>
       <c r="H25" s="1">
-        <v>-0.321</v>
+        <v>-0.32</v>
       </c>
       <c r="I25" s="1">
-        <v>-0.382</v>
+        <v>-0.38</v>
       </c>
       <c r="J25" s="1">
-        <v>-0.43</v>
+        <v>-0.427</v>
       </c>
       <c r="K25" s="1">
-        <v>-0.454</v>
+        <v>-0.451</v>
       </c>
       <c r="L25" s="1">
-        <v>-0.479</v>
+        <v>-0.476</v>
       </c>
       <c r="M25" s="1">
-        <v>-0.516</v>
+        <v>-0.513</v>
       </c>
       <c r="N25" s="1">
-        <v>-0.546</v>
+        <v>-0.541</v>
       </c>
       <c r="O25" s="1">
-        <v>-0.545</v>
+        <v>-0.54</v>
       </c>
       <c r="P25" s="1">
-        <v>-0.51</v>
+        <v>-0.506</v>
       </c>
       <c r="Q25" s="1">
-        <v>-0.446</v>
+        <v>-0.443</v>
       </c>
       <c r="R25" s="1">
-        <v>-0.35</v>
+        <v>-0.347</v>
       </c>
       <c r="S25" s="1">
-        <v>-0.22</v>
+        <v>-0.218</v>
       </c>
       <c r="T25" s="1">
-        <v>-0.08</v>
+        <v>-0.078</v>
       </c>
       <c r="U25" s="1">
-        <v>0.029</v>
+        <v>0.031</v>
       </c>
     </row>
     <row r="26" spans="1:21">
@@ -2135,58 +2138,58 @@
         <v>-0.635</v>
       </c>
       <c r="D26" s="1">
-        <v>-0.474</v>
+        <v>-0.475</v>
       </c>
       <c r="E26" s="1">
-        <v>-0.373</v>
+        <v>-0.374</v>
       </c>
       <c r="F26" s="1">
         <v>-0.376</v>
       </c>
       <c r="G26" s="1">
-        <v>-0.458</v>
+        <v>-0.457</v>
       </c>
       <c r="H26" s="1">
-        <v>-0.5610000000000001</v>
+        <v>-0.5590000000000001</v>
       </c>
       <c r="I26" s="1">
-        <v>-0.624</v>
+        <v>-0.621</v>
       </c>
       <c r="J26" s="1">
-        <v>-0.642</v>
+        <v>-0.64</v>
       </c>
       <c r="K26" s="1">
-        <v>-0.669</v>
+        <v>-0.666</v>
       </c>
       <c r="L26" s="1">
-        <v>-0.732</v>
+        <v>-0.728</v>
       </c>
       <c r="M26" s="1">
-        <v>-0.794</v>
+        <v>-0.79</v>
       </c>
       <c r="N26" s="1">
-        <v>-0.803</v>
+        <v>-0.798</v>
       </c>
       <c r="O26" s="1">
-        <v>-0.745</v>
+        <v>-0.742</v>
       </c>
       <c r="P26" s="1">
-        <v>-0.646</v>
+        <v>-0.643</v>
       </c>
       <c r="Q26" s="1">
-        <v>-0.52</v>
+        <v>-0.517</v>
       </c>
       <c r="R26" s="1">
-        <v>-0.363</v>
+        <v>-0.361</v>
       </c>
       <c r="S26" s="1">
-        <v>-0.192</v>
+        <v>-0.19</v>
       </c>
       <c r="T26" s="1">
-        <v>-0.052</v>
+        <v>-0.049</v>
       </c>
       <c r="U26" s="1">
-        <v>0.034</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="27" spans="1:21">
@@ -2200,58 +2203,58 @@
         <v>-0.24</v>
       </c>
       <c r="D27" s="1">
-        <v>-0.138</v>
+        <v>-0.139</v>
       </c>
       <c r="E27" s="1">
         <v>-0.166</v>
       </c>
       <c r="F27" s="1">
-        <v>-0.283</v>
+        <v>-0.282</v>
       </c>
       <c r="G27" s="1">
-        <v>-0.408</v>
+        <v>-0.407</v>
       </c>
       <c r="H27" s="1">
-        <v>-0.48</v>
+        <v>-0.477</v>
       </c>
       <c r="I27" s="1">
-        <v>-0.504</v>
+        <v>-0.501</v>
       </c>
       <c r="J27" s="1">
-        <v>-0.531</v>
+        <v>-0.528</v>
       </c>
       <c r="K27" s="1">
-        <v>-0.584</v>
+        <v>-0.581</v>
       </c>
       <c r="L27" s="1">
-        <v>-0.637</v>
+        <v>-0.633</v>
       </c>
       <c r="M27" s="1">
-        <v>-0.649</v>
+        <v>-0.645</v>
       </c>
       <c r="N27" s="1">
-        <v>-0.602</v>
+        <v>-0.598</v>
       </c>
       <c r="O27" s="1">
-        <v>-0.512</v>
+        <v>-0.51</v>
       </c>
       <c r="P27" s="1">
-        <v>-0.401</v>
+        <v>-0.399</v>
       </c>
       <c r="Q27" s="1">
-        <v>-0.275</v>
+        <v>-0.273</v>
       </c>
       <c r="R27" s="1">
-        <v>-0.151</v>
+        <v>-0.149</v>
       </c>
       <c r="S27" s="1">
-        <v>-0.059</v>
+        <v>-0.057</v>
       </c>
       <c r="T27" s="1">
-        <v>-0.008</v>
+        <v>-0.006</v>
       </c>
       <c r="U27" s="1">
-        <v>0.022</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="28" spans="1:21">
@@ -2265,58 +2268,58 @@
         <v>0.129</v>
       </c>
       <c r="D28" s="1">
-        <v>0.08</v>
+        <v>0.081</v>
       </c>
       <c r="E28" s="1">
-        <v>-0.029</v>
+        <v>-0.027</v>
       </c>
       <c r="F28" s="1">
-        <v>-0.146</v>
+        <v>-0.143</v>
       </c>
       <c r="G28" s="1">
-        <v>-0.225</v>
+        <v>-0.222</v>
       </c>
       <c r="H28" s="1">
-        <v>-0.266</v>
+        <v>-0.263</v>
       </c>
       <c r="I28" s="1">
-        <v>-0.3</v>
+        <v>-0.296</v>
       </c>
       <c r="J28" s="1">
-        <v>-0.342</v>
+        <v>-0.337</v>
       </c>
       <c r="K28" s="1">
-        <v>-0.382</v>
+        <v>-0.377</v>
       </c>
       <c r="L28" s="1">
-        <v>-0.397</v>
+        <v>-0.392</v>
       </c>
       <c r="M28" s="1">
-        <v>-0.372</v>
+        <v>-0.368</v>
       </c>
       <c r="N28" s="1">
-        <v>-0.315</v>
+        <v>-0.311</v>
       </c>
       <c r="O28" s="1">
-        <v>-0.244</v>
+        <v>-0.241</v>
       </c>
       <c r="P28" s="1">
-        <v>-0.175</v>
+        <v>-0.172</v>
       </c>
       <c r="Q28" s="1">
-        <v>-0.117</v>
+        <v>-0.115</v>
       </c>
       <c r="R28" s="1">
-        <v>-0.081</v>
+        <v>-0.079</v>
       </c>
       <c r="S28" s="1">
-        <v>-0.065</v>
+        <v>-0.063</v>
       </c>
       <c r="T28" s="1">
-        <v>-0.058</v>
+        <v>-0.056</v>
       </c>
       <c r="U28" s="1">
-        <v>-0.047</v>
+        <v>-0.046</v>
       </c>
     </row>
     <row r="29" spans="1:21">
@@ -2330,58 +2333,58 @@
         <v>-0.105</v>
       </c>
       <c r="D29" s="1">
-        <v>-0.115</v>
+        <v>-0.114</v>
       </c>
       <c r="E29" s="1">
-        <v>-0.143</v>
+        <v>-0.141</v>
       </c>
       <c r="F29" s="1">
-        <v>-0.156</v>
+        <v>-0.153</v>
       </c>
       <c r="G29" s="1">
-        <v>-0.157</v>
+        <v>-0.154</v>
       </c>
       <c r="H29" s="1">
-        <v>-0.158</v>
+        <v>-0.154</v>
       </c>
       <c r="I29" s="1">
-        <v>-0.154</v>
+        <v>-0.15</v>
       </c>
       <c r="J29" s="1">
-        <v>-0.146</v>
+        <v>-0.142</v>
       </c>
       <c r="K29" s="1">
-        <v>-0.139</v>
+        <v>-0.134</v>
       </c>
       <c r="L29" s="1">
-        <v>-0.13</v>
+        <v>-0.125</v>
       </c>
       <c r="M29" s="1">
-        <v>-0.107</v>
+        <v>-0.104</v>
       </c>
       <c r="N29" s="1">
-        <v>-0.067</v>
+        <v>-0.064</v>
       </c>
       <c r="O29" s="1">
-        <v>-0.017</v>
+        <v>-0.014</v>
       </c>
       <c r="P29" s="1">
-        <v>0.026</v>
+        <v>0.029</v>
       </c>
       <c r="Q29" s="1">
+        <v>0.051</v>
+      </c>
+      <c r="R29" s="1">
+        <v>0.052</v>
+      </c>
+      <c r="S29" s="1">
         <v>0.049</v>
       </c>
-      <c r="R29" s="1">
-        <v>0.051</v>
-      </c>
-      <c r="S29" s="1">
-        <v>0.048</v>
-      </c>
       <c r="T29" s="1">
-        <v>0.056</v>
+        <v>0.058</v>
       </c>
       <c r="U29" s="1">
-        <v>0.08</v>
+        <v>0.081</v>
       </c>
     </row>
     <row r="30" spans="1:21">
@@ -2392,61 +2395,61 @@
         <v>-0.025</v>
       </c>
       <c r="C30" s="1">
-        <v>-0.046</v>
+        <v>-0.045</v>
       </c>
       <c r="D30" s="1">
-        <v>-0.081</v>
+        <v>-0.079</v>
       </c>
       <c r="E30" s="1">
-        <v>-0.102</v>
+        <v>-0.099</v>
       </c>
       <c r="F30" s="1">
-        <v>-0.118</v>
+        <v>-0.114</v>
       </c>
       <c r="G30" s="1">
-        <v>-0.144</v>
+        <v>-0.14</v>
       </c>
       <c r="H30" s="1">
+        <v>-0.176</v>
+      </c>
+      <c r="I30" s="1">
+        <v>-0.209</v>
+      </c>
+      <c r="J30" s="1">
+        <v>-0.226</v>
+      </c>
+      <c r="K30" s="1">
+        <v>-0.215</v>
+      </c>
+      <c r="L30" s="1">
         <v>-0.18</v>
       </c>
-      <c r="I30" s="1">
-        <v>-0.214</v>
-      </c>
-      <c r="J30" s="1">
-        <v>-0.231</v>
-      </c>
-      <c r="K30" s="1">
-        <v>-0.22</v>
-      </c>
-      <c r="L30" s="1">
-        <v>-0.183</v>
-      </c>
       <c r="M30" s="1">
-        <v>-0.142</v>
+        <v>-0.139</v>
       </c>
       <c r="N30" s="1">
-        <v>-0.115</v>
+        <v>-0.112</v>
       </c>
       <c r="O30" s="1">
-        <v>-0.105</v>
+        <v>-0.103</v>
       </c>
       <c r="P30" s="1">
-        <v>-0.108</v>
+        <v>-0.106</v>
       </c>
       <c r="Q30" s="1">
-        <v>-0.116</v>
+        <v>-0.114</v>
       </c>
       <c r="R30" s="1">
-        <v>-0.123</v>
+        <v>-0.121</v>
       </c>
       <c r="S30" s="1">
-        <v>-0.131</v>
+        <v>-0.129</v>
       </c>
       <c r="T30" s="1">
-        <v>-0.142</v>
+        <v>-0.14</v>
       </c>
       <c r="U30" s="1">
-        <v>-0.151</v>
+        <v>-0.149</v>
       </c>
     </row>
     <row r="31" spans="1:21">
@@ -2457,61 +2460,61 @@
         <v>0.024</v>
       </c>
       <c r="C31" s="1">
-        <v>-0.001</v>
+        <v>-0</v>
       </c>
       <c r="D31" s="1">
-        <v>-0.037</v>
+        <v>-0.035</v>
       </c>
       <c r="E31" s="1">
-        <v>-0.061</v>
+        <v>-0.058</v>
       </c>
       <c r="F31" s="1">
-        <v>-0.106</v>
+        <v>-0.102</v>
       </c>
       <c r="G31" s="1">
-        <v>-0.185</v>
+        <v>-0.181</v>
       </c>
       <c r="H31" s="1">
-        <v>-0.266</v>
+        <v>-0.26</v>
       </c>
       <c r="I31" s="1">
+        <v>-0.294</v>
+      </c>
+      <c r="J31" s="1">
+        <v>-0.272</v>
+      </c>
+      <c r="K31" s="1">
+        <v>-0.222</v>
+      </c>
+      <c r="L31" s="1">
+        <v>-0.196</v>
+      </c>
+      <c r="M31" s="1">
+        <v>-0.215</v>
+      </c>
+      <c r="N31" s="1">
+        <v>-0.261</v>
+      </c>
+      <c r="O31" s="1">
         <v>-0.301</v>
       </c>
-      <c r="J31" s="1">
-        <v>-0.277</v>
-      </c>
-      <c r="K31" s="1">
-        <v>-0.227</v>
-      </c>
-      <c r="L31" s="1">
-        <v>-0.199</v>
-      </c>
-      <c r="M31" s="1">
-        <v>-0.218</v>
-      </c>
-      <c r="N31" s="1">
-        <v>-0.264</v>
-      </c>
-      <c r="O31" s="1">
-        <v>-0.303</v>
-      </c>
       <c r="P31" s="1">
-        <v>-0.318</v>
+        <v>-0.315</v>
       </c>
       <c r="Q31" s="1">
-        <v>-0.319</v>
+        <v>-0.316</v>
       </c>
       <c r="R31" s="1">
-        <v>-0.339</v>
+        <v>-0.337</v>
       </c>
       <c r="S31" s="1">
-        <v>-0.392</v>
+        <v>-0.39</v>
       </c>
       <c r="T31" s="1">
-        <v>-0.448</v>
+        <v>-0.446</v>
       </c>
       <c r="U31" s="1">
-        <v>-0.463</v>
+        <v>-0.46</v>
       </c>
     </row>
     <row r="32" spans="1:21">
@@ -2531,7 +2534,7 @@
         <v>-0.246</v>
       </c>
       <c r="F32" s="1">
-        <v>-0.364</v>
+        <v>-0.363</v>
       </c>
       <c r="G32" s="1">
         <v>-0.467</v>
@@ -2543,10 +2546,10 @@
         <v>-0.472</v>
       </c>
       <c r="J32" s="1">
-        <v>-0.395</v>
+        <v>-0.394</v>
       </c>
       <c r="K32" s="1">
-        <v>-0.331</v>
+        <v>-0.33</v>
       </c>
       <c r="L32" s="1">
         <v>-0.311</v>
@@ -2555,28 +2558,28 @@
         <v>-0.325</v>
       </c>
       <c r="N32" s="1">
-        <v>-0.346</v>
+        <v>-0.345</v>
       </c>
       <c r="O32" s="1">
-        <v>-0.354</v>
+        <v>-0.353</v>
       </c>
       <c r="P32" s="1">
         <v>-0.353</v>
       </c>
       <c r="Q32" s="1">
-        <v>-0.372</v>
+        <v>-0.371</v>
       </c>
       <c r="R32" s="1">
-        <v>-0.421</v>
+        <v>-0.42</v>
       </c>
       <c r="S32" s="1">
-        <v>-0.471</v>
+        <v>-0.47</v>
       </c>
       <c r="T32" s="1">
-        <v>-0.484</v>
+        <v>-0.483</v>
       </c>
       <c r="U32" s="1">
-        <v>-0.454</v>
+        <v>-0.453</v>
       </c>
     </row>
     <row r="33" spans="1:21">
@@ -2596,7 +2599,7 @@
         <v>-0.548</v>
       </c>
       <c r="F33" s="1">
-        <v>-0.652</v>
+        <v>-0.651</v>
       </c>
       <c r="G33" s="1">
         <v>-0.669</v>
@@ -2611,37 +2614,37 @@
         <v>-0.412</v>
       </c>
       <c r="K33" s="1">
-        <v>-0.346</v>
+        <v>-0.345</v>
       </c>
       <c r="L33" s="1">
         <v>-0.301</v>
       </c>
       <c r="M33" s="1">
-        <v>-0.275</v>
+        <v>-0.274</v>
       </c>
       <c r="N33" s="1">
         <v>-0.258</v>
       </c>
       <c r="O33" s="1">
-        <v>-0.247</v>
+        <v>-0.246</v>
       </c>
       <c r="P33" s="1">
-        <v>-0.249</v>
+        <v>-0.248</v>
       </c>
       <c r="Q33" s="1">
-        <v>-0.269</v>
+        <v>-0.268</v>
       </c>
       <c r="R33" s="1">
-        <v>-0.288</v>
+        <v>-0.287</v>
       </c>
       <c r="S33" s="1">
-        <v>-0.291</v>
+        <v>-0.29</v>
       </c>
       <c r="T33" s="1">
-        <v>-0.281</v>
+        <v>-0.28</v>
       </c>
       <c r="U33" s="1">
-        <v>-0.254</v>
+        <v>-0.253</v>
       </c>
     </row>
     <row r="34" spans="1:21">
@@ -2649,64 +2652,129 @@
         <v>33</v>
       </c>
       <c r="B34" s="1">
-        <v>-0.42</v>
+        <v>-0.396</v>
       </c>
       <c r="C34" s="1">
+        <v>-0.46</v>
+      </c>
+      <c r="D34" s="1">
+        <v>-0.588</v>
+      </c>
+      <c r="E34" s="1">
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="F34" s="1">
+        <v>-0.715</v>
+      </c>
+      <c r="G34" s="1">
+        <v>-0.656</v>
+      </c>
+      <c r="H34" s="1">
+        <v>-0.55</v>
+      </c>
+      <c r="I34" s="1">
+        <v>-0.443</v>
+      </c>
+      <c r="J34" s="1">
+        <v>-0.359</v>
+      </c>
+      <c r="K34" s="1">
+        <v>-0.299</v>
+      </c>
+      <c r="L34" s="1">
+        <v>-0.263</v>
+      </c>
+      <c r="M34" s="1">
+        <v>-0.244</v>
+      </c>
+      <c r="N34" s="1">
+        <v>-0.232</v>
+      </c>
+      <c r="O34" s="1">
+        <v>-0.23</v>
+      </c>
+      <c r="P34" s="1">
+        <v>-0.242</v>
+      </c>
+      <c r="Q34" s="1">
+        <v>-0.252</v>
+      </c>
+      <c r="R34" s="1">
+        <v>-0.252</v>
+      </c>
+      <c r="S34" s="1">
+        <v>-0.247</v>
+      </c>
+      <c r="T34" s="1">
+        <v>-0.226</v>
+      </c>
+      <c r="U34" s="1">
+        <v>-0.177</v>
+      </c>
+    </row>
+    <row r="35" spans="1:21">
+      <c r="A35" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1">
         <v>-0.478</v>
       </c>
-      <c r="D34" s="1">
-        <v>-0.599</v>
-      </c>
-      <c r="E34" s="1">
-        <v>-0.7</v>
-      </c>
-      <c r="F34" s="1">
-        <v>-0.725</v>
-      </c>
-      <c r="G34" s="1">
-        <v>-0.666</v>
-      </c>
-      <c r="H34" s="1">
-        <v>-0.5600000000000001</v>
-      </c>
-      <c r="I34" s="1">
-        <v>-0.451</v>
-      </c>
-      <c r="J34" s="1">
-        <v>-0.366</v>
-      </c>
-      <c r="K34" s="1">
-        <v>-0.305</v>
-      </c>
-      <c r="L34" s="1">
-        <v>-0.269</v>
-      </c>
-      <c r="M34" s="1">
-        <v>-0.25</v>
-      </c>
-      <c r="N34" s="1">
-        <v>-0.238</v>
-      </c>
-      <c r="O34" s="1">
-        <v>-0.237</v>
-      </c>
-      <c r="P34" s="1">
-        <v>-0.25</v>
-      </c>
-      <c r="Q34" s="1">
-        <v>-0.262</v>
-      </c>
-      <c r="R34" s="1">
-        <v>-0.264</v>
-      </c>
-      <c r="S34" s="1">
-        <v>-0.258</v>
-      </c>
-      <c r="T34" s="1">
-        <v>-0.236</v>
-      </c>
-      <c r="U34" s="1">
-        <v>-0.186</v>
+      <c r="C35" s="1">
+        <v>-0.55</v>
+      </c>
+      <c r="D35" s="1">
+        <v>-0.635</v>
+      </c>
+      <c r="E35" s="1">
+        <v>-0.646</v>
+      </c>
+      <c r="F35" s="1">
+        <v>-0.591</v>
+      </c>
+      <c r="G35" s="1">
+        <v>-0.496</v>
+      </c>
+      <c r="H35" s="1">
+        <v>-0.386</v>
+      </c>
+      <c r="I35" s="1">
+        <v>-0.276</v>
+      </c>
+      <c r="J35" s="1">
+        <v>-0.179</v>
+      </c>
+      <c r="K35" s="1">
+        <v>-0.115</v>
+      </c>
+      <c r="L35" s="1">
+        <v>-0.08400000000000001</v>
+      </c>
+      <c r="M35" s="1">
+        <v>-0.065</v>
+      </c>
+      <c r="N35" s="1">
+        <v>-0.045</v>
+      </c>
+      <c r="O35" s="1">
+        <v>-0.021</v>
+      </c>
+      <c r="P35" s="1">
+        <v>0.005</v>
+      </c>
+      <c r="Q35" s="1">
+        <v>0.014</v>
+      </c>
+      <c r="R35" s="1">
+        <v>0</v>
+      </c>
+      <c r="S35" s="1">
+        <v>-0.013</v>
+      </c>
+      <c r="T35" s="1">
+        <v>-0.001</v>
+      </c>
+      <c r="U35" s="1">
+        <v>0.035</v>
       </c>
     </row>
   </sheetData>
@@ -2721,22 +2789,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update: update XRO forecast
</commit_message>
<xml_diff>
--- a/content/climate/XRO/XRO_ENSO_fcst.xlsx
+++ b/content/climate/XRO/XRO_ENSO_fcst.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>init</t>
   </si>
@@ -123,6 +123,9 @@
   </si>
   <si>
     <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
   </si>
   <si>
     <t>Readme</t>
@@ -499,7 +502,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U36"/>
+  <dimension ref="A1:U37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="21" width="10.7109375" style="1" customWidth="1"/>
@@ -507,7 +510,7 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B1" s="2">
         <v>0</v>
@@ -2531,13 +2534,13 @@
         <v>-0.096</v>
       </c>
       <c r="D32" s="1">
-        <v>-0.158</v>
+        <v>-0.159</v>
       </c>
       <c r="E32" s="1">
-        <v>-0.245</v>
+        <v>-0.246</v>
       </c>
       <c r="F32" s="1">
-        <v>-0.362</v>
+        <v>-0.363</v>
       </c>
       <c r="G32" s="1">
         <v>-0.466</v>
@@ -2549,7 +2552,7 @@
         <v>-0.471</v>
       </c>
       <c r="J32" s="1">
-        <v>-0.393</v>
+        <v>-0.394</v>
       </c>
       <c r="K32" s="1">
         <v>-0.33</v>
@@ -2561,7 +2564,7 @@
         <v>-0.324</v>
       </c>
       <c r="N32" s="1">
-        <v>-0.344</v>
+        <v>-0.345</v>
       </c>
       <c r="O32" s="1">
         <v>-0.353</v>
@@ -2579,7 +2582,7 @@
         <v>-0.469</v>
       </c>
       <c r="T32" s="1">
-        <v>-0.482</v>
+        <v>-0.483</v>
       </c>
       <c r="U32" s="1">
         <v>-0.452</v>
@@ -2608,13 +2611,13 @@
         <v>-0.668</v>
       </c>
       <c r="H33" s="1">
-        <v>-0.604</v>
+        <v>-0.605</v>
       </c>
       <c r="I33" s="1">
         <v>-0.504</v>
       </c>
       <c r="J33" s="1">
-        <v>-0.411</v>
+        <v>-0.412</v>
       </c>
       <c r="K33" s="1">
         <v>-0.345</v>
@@ -2638,13 +2641,13 @@
         <v>-0.267</v>
       </c>
       <c r="R33" s="1">
-        <v>-0.285</v>
+        <v>-0.286</v>
       </c>
       <c r="S33" s="1">
         <v>-0.289</v>
       </c>
       <c r="T33" s="1">
-        <v>-0.279</v>
+        <v>-0.28</v>
       </c>
       <c r="U33" s="1">
         <v>-0.252</v>
@@ -2697,10 +2700,10 @@
         <v>-0.229</v>
       </c>
       <c r="P34" s="1">
-        <v>-0.24</v>
+        <v>-0.241</v>
       </c>
       <c r="Q34" s="1">
-        <v>-0.25</v>
+        <v>-0.251</v>
       </c>
       <c r="R34" s="1">
         <v>-0.251</v>
@@ -2712,7 +2715,7 @@
         <v>-0.225</v>
       </c>
       <c r="U34" s="1">
-        <v>-0.176</v>
+        <v>-0.177</v>
       </c>
     </row>
     <row r="35" spans="1:21">
@@ -2756,7 +2759,7 @@
         <v>-0.067</v>
       </c>
       <c r="N35" s="1">
-        <v>-0.047</v>
+        <v>-0.048</v>
       </c>
       <c r="O35" s="1">
         <v>-0.023</v>
@@ -2765,7 +2768,7 @@
         <v>0.002</v>
       </c>
       <c r="Q35" s="1">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="R35" s="1">
         <v>-0.002</v>
@@ -2777,7 +2780,7 @@
         <v>-0.002</v>
       </c>
       <c r="U35" s="1">
-        <v>0.035</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="36" spans="1:21">
@@ -2785,64 +2788,129 @@
         <v>35</v>
       </c>
       <c r="B36" s="1">
-        <v>-0.6879999999999999</v>
+        <v>-0.6929999999999999</v>
       </c>
       <c r="C36" s="1">
-        <v>-0.707</v>
+        <v>-0.713</v>
       </c>
       <c r="D36" s="1">
-        <v>-0.694</v>
+        <v>-0.701</v>
       </c>
       <c r="E36" s="1">
-        <v>-0.626</v>
+        <v>-0.633</v>
       </c>
       <c r="F36" s="1">
-        <v>-0.526</v>
+        <v>-0.532</v>
       </c>
       <c r="G36" s="1">
-        <v>-0.408</v>
+        <v>-0.412</v>
       </c>
       <c r="H36" s="1">
-        <v>-0.279</v>
+        <v>-0.28</v>
       </c>
       <c r="I36" s="1">
-        <v>-0.158</v>
+        <v>-0.157</v>
       </c>
       <c r="J36" s="1">
-        <v>-0.074</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="K36" s="1">
-        <v>-0.029</v>
+        <v>-0.025</v>
       </c>
       <c r="L36" s="1">
-        <v>0.001</v>
+        <v>0.005</v>
       </c>
       <c r="M36" s="1">
-        <v>0.038</v>
+        <v>0.044</v>
       </c>
       <c r="N36" s="1">
-        <v>0.089</v>
+        <v>0.097</v>
       </c>
       <c r="O36" s="1">
-        <v>0.139</v>
+        <v>0.149</v>
       </c>
       <c r="P36" s="1">
-        <v>0.159</v>
+        <v>0.169</v>
       </c>
       <c r="Q36" s="1">
-        <v>0.137</v>
+        <v>0.147</v>
       </c>
       <c r="R36" s="1">
-        <v>0.106</v>
+        <v>0.114</v>
       </c>
       <c r="S36" s="1">
-        <v>0.098</v>
+        <v>0.105</v>
       </c>
       <c r="T36" s="1">
-        <v>0.116</v>
+        <v>0.122</v>
       </c>
       <c r="U36" s="1">
-        <v>0.139</v>
+        <v>0.145</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21">
+      <c r="A37" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1">
+        <v>-0.601</v>
+      </c>
+      <c r="C37" s="1">
+        <v>-0.5580000000000001</v>
+      </c>
+      <c r="D37" s="1">
+        <v>-0.456</v>
+      </c>
+      <c r="E37" s="1">
+        <v>-0.344</v>
+      </c>
+      <c r="F37" s="1">
+        <v>-0.23</v>
+      </c>
+      <c r="G37" s="1">
+        <v>-0.094</v>
+      </c>
+      <c r="H37" s="1">
+        <v>0.045</v>
+      </c>
+      <c r="I37" s="1">
+        <v>0.152</v>
+      </c>
+      <c r="J37" s="1">
+        <v>0.216</v>
+      </c>
+      <c r="K37" s="1">
+        <v>0.262</v>
+      </c>
+      <c r="L37" s="1">
+        <v>0.334</v>
+      </c>
+      <c r="M37" s="1">
+        <v>0.441</v>
+      </c>
+      <c r="N37" s="1">
+        <v>0.541</v>
+      </c>
+      <c r="O37" s="1">
+        <v>0.574</v>
+      </c>
+      <c r="P37" s="1">
+        <v>0.531</v>
+      </c>
+      <c r="Q37" s="1">
+        <v>0.452</v>
+      </c>
+      <c r="R37" s="1">
+        <v>0.38</v>
+      </c>
+      <c r="S37" s="1">
+        <v>0.321</v>
+      </c>
+      <c r="T37" s="1">
+        <v>0.267</v>
+      </c>
+      <c r="U37" s="1">
+        <v>0.215</v>
       </c>
     </row>
   </sheetData>
@@ -2857,22 +2925,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update XRO forecast (trend correction)
</commit_message>
<xml_diff>
--- a/content/climate/XRO/XRO_ENSO_fcst.xlsx
+++ b/content/climate/XRO/XRO_ENSO_fcst.xlsx
@@ -15,10 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
-  <si>
-    <t>init</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>2023-01</t>
   </si>
@@ -140,7 +137,7 @@
     <t>Extended nonlinear recharge oscillator (XRO) ENSO forecast (Zhao et al. 2024)</t>
   </si>
   <si>
-    <t>Reference: Zhao, S., F.-F. Jin, M. F. Stuecker, P. R. Thompson, J.-S. Kug, M. J. McPhaden, M. A. Cane, A. T. Wittenberg, and W. Cai, 2024: Explainable El Niño predictability from climate mode interactions. Nature, 630, 891–898, https://doi.org/10.1038/s41586-024-07534-6</t>
+    <t>Reference: Zhao et al. (2024), Nature</t>
   </si>
   <si>
     <t>Webpage: https://senzhao.netlify.app/climate/xro/</t>
@@ -516,7 +513,7 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B1" s="2">
         <v>0</v>
@@ -581,2472 +578,2472 @@
     </row>
     <row r="2" spans="1:21">
       <c r="A2" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>-0.68</v>
+        <v>-0.696</v>
       </c>
       <c r="C2" s="1">
-        <v>-0.731</v>
+        <v>-0.733</v>
       </c>
       <c r="D2" s="1">
-        <v>-0.712</v>
+        <v>-0.71</v>
       </c>
       <c r="E2" s="1">
-        <v>-0.511</v>
+        <v>-0.539</v>
       </c>
       <c r="F2" s="1">
-        <v>-0.148</v>
+        <v>-0.219</v>
       </c>
       <c r="G2" s="1">
-        <v>0.26</v>
+        <v>0.172</v>
       </c>
       <c r="H2" s="1">
-        <v>0.57</v>
+        <v>0.528</v>
       </c>
       <c r="I2" s="1">
-        <v>0.766</v>
+        <v>0.8080000000000001</v>
       </c>
       <c r="J2" s="1">
-        <v>0.945</v>
+        <v>1.066</v>
       </c>
       <c r="K2" s="1">
-        <v>1.217</v>
+        <v>1.386</v>
       </c>
       <c r="L2" s="1">
-        <v>1.569</v>
+        <v>1.739</v>
       </c>
       <c r="M2" s="1">
-        <v>1.834</v>
+        <v>1.972</v>
       </c>
       <c r="N2" s="1">
-        <v>1.889</v>
+        <v>2.029</v>
       </c>
       <c r="O2" s="1">
-        <v>1.759</v>
+        <v>1.929</v>
       </c>
       <c r="P2" s="1">
-        <v>1.51</v>
+        <v>1.649</v>
       </c>
       <c r="Q2" s="1">
-        <v>1.205</v>
+        <v>1.249</v>
       </c>
       <c r="R2" s="1">
-        <v>0.887</v>
+        <v>0.839</v>
       </c>
       <c r="S2" s="1">
-        <v>0.594</v>
+        <v>0.486</v>
       </c>
       <c r="T2" s="1">
-        <v>0.356</v>
+        <v>0.243</v>
       </c>
       <c r="U2" s="1">
-        <v>0.183</v>
+        <v>0.118</v>
       </c>
     </row>
     <row r="3" spans="1:21">
       <c r="A3" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="1">
-        <v>-0.473</v>
+        <v>-0.489</v>
       </c>
       <c r="C3" s="1">
-        <v>-0.459</v>
+        <v>-0.476</v>
       </c>
       <c r="D3" s="1">
-        <v>-0.314</v>
+        <v>-0.34</v>
       </c>
       <c r="E3" s="1">
-        <v>-0.022</v>
+        <v>-0.064</v>
       </c>
       <c r="F3" s="1">
-        <v>0.294</v>
+        <v>0.266</v>
       </c>
       <c r="G3" s="1">
-        <v>0.526</v>
+        <v>0.556</v>
       </c>
       <c r="H3" s="1">
-        <v>0.665</v>
+        <v>0.771</v>
       </c>
       <c r="I3" s="1">
-        <v>0.785</v>
+        <v>0.971</v>
       </c>
       <c r="J3" s="1">
-        <v>0.959</v>
+        <v>1.207</v>
       </c>
       <c r="K3" s="1">
-        <v>1.177</v>
+        <v>1.431</v>
       </c>
       <c r="L3" s="1">
-        <v>1.332</v>
+        <v>1.572</v>
       </c>
       <c r="M3" s="1">
-        <v>1.342</v>
+        <v>1.586</v>
       </c>
       <c r="N3" s="1">
-        <v>1.221</v>
+        <v>1.481</v>
       </c>
       <c r="O3" s="1">
-        <v>1.032</v>
+        <v>1.261</v>
       </c>
       <c r="P3" s="1">
-        <v>0.821</v>
+        <v>0.951</v>
       </c>
       <c r="Q3" s="1">
-        <v>0.596</v>
+        <v>0.622</v>
       </c>
       <c r="R3" s="1">
-        <v>0.374</v>
+        <v>0.323</v>
       </c>
       <c r="S3" s="1">
-        <v>0.185</v>
+        <v>0.111</v>
       </c>
       <c r="T3" s="1">
-        <v>0.047</v>
+        <v>-0.004</v>
       </c>
       <c r="U3" s="1">
-        <v>-0.047</v>
+        <v>-0.052</v>
       </c>
     </row>
     <row r="4" spans="1:21">
       <c r="A4" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="1">
-        <v>-0.02</v>
+        <v>-0.036</v>
       </c>
       <c r="C4" s="1">
-        <v>0.07099999999999999</v>
+        <v>0.026</v>
       </c>
       <c r="D4" s="1">
-        <v>0.276</v>
+        <v>0.199</v>
       </c>
       <c r="E4" s="1">
-        <v>0.484</v>
+        <v>0.421</v>
       </c>
       <c r="F4" s="1">
-        <v>0.609</v>
+        <v>0.62</v>
       </c>
       <c r="G4" s="1">
-        <v>0.665</v>
+        <v>0.774</v>
       </c>
       <c r="H4" s="1">
-        <v>0.72</v>
+        <v>0.911</v>
       </c>
       <c r="I4" s="1">
-        <v>0.83</v>
+        <v>1.079</v>
       </c>
       <c r="J4" s="1">
-        <v>0.977</v>
+        <v>1.238</v>
       </c>
       <c r="K4" s="1">
-        <v>1.078</v>
+        <v>1.338</v>
       </c>
       <c r="L4" s="1">
-        <v>1.062</v>
+        <v>1.332</v>
       </c>
       <c r="M4" s="1">
-        <v>0.9429999999999999</v>
+        <v>1.225</v>
       </c>
       <c r="N4" s="1">
-        <v>0.787</v>
+        <v>1.036</v>
       </c>
       <c r="O4" s="1">
-        <v>0.627</v>
+        <v>0.769</v>
       </c>
       <c r="P4" s="1">
-        <v>0.448</v>
+        <v>0.479</v>
       </c>
       <c r="Q4" s="1">
-        <v>0.255</v>
+        <v>0.213</v>
       </c>
       <c r="R4" s="1">
-        <v>0.079</v>
+        <v>0.01</v>
       </c>
       <c r="S4" s="1">
-        <v>-0.055</v>
+        <v>-0.1</v>
       </c>
       <c r="T4" s="1">
-        <v>-0.144</v>
+        <v>-0.139</v>
       </c>
       <c r="U4" s="1">
-        <v>-0.215</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="5" spans="1:21">
       <c r="A5" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="1">
-        <v>0.182</v>
+        <v>0.165</v>
       </c>
       <c r="C5" s="1">
-        <v>0.334</v>
+        <v>0.263</v>
       </c>
       <c r="D5" s="1">
-        <v>0.572</v>
+        <v>0.458</v>
       </c>
       <c r="E5" s="1">
-        <v>0.743</v>
+        <v>0.671</v>
       </c>
       <c r="F5" s="1">
-        <v>0.844</v>
+        <v>0.868</v>
       </c>
       <c r="G5" s="1">
-        <v>0.927</v>
+        <v>1.043</v>
       </c>
       <c r="H5" s="1">
-        <v>1.048</v>
+        <v>1.205</v>
       </c>
       <c r="I5" s="1">
-        <v>1.195</v>
+        <v>1.323</v>
       </c>
       <c r="J5" s="1">
-        <v>1.276</v>
+        <v>1.36</v>
       </c>
       <c r="K5" s="1">
-        <v>1.221</v>
+        <v>1.325</v>
       </c>
       <c r="L5" s="1">
-        <v>1.06</v>
+        <v>1.222</v>
       </c>
       <c r="M5" s="1">
-        <v>0.878</v>
+        <v>1.024</v>
       </c>
       <c r="N5" s="1">
-        <v>0.7</v>
+        <v>0.742</v>
       </c>
       <c r="O5" s="1">
-        <v>0.491</v>
+        <v>0.423</v>
       </c>
       <c r="P5" s="1">
-        <v>0.251</v>
+        <v>0.112</v>
       </c>
       <c r="Q5" s="1">
-        <v>0.023</v>
+        <v>-0.131</v>
       </c>
       <c r="R5" s="1">
-        <v>-0.153</v>
+        <v>-0.253</v>
       </c>
       <c r="S5" s="1">
-        <v>-0.269</v>
+        <v>-0.289</v>
       </c>
       <c r="T5" s="1">
-        <v>-0.362</v>
+        <v>-0.325</v>
       </c>
       <c r="U5" s="1">
-        <v>-0.46</v>
+        <v>-0.409</v>
       </c>
     </row>
     <row r="6" spans="1:21">
       <c r="A6" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="1">
-        <v>0.464</v>
+        <v>0.447</v>
       </c>
       <c r="C6" s="1">
-        <v>0.626</v>
+        <v>0.605</v>
       </c>
       <c r="D6" s="1">
-        <v>0.843</v>
+        <v>0.864</v>
       </c>
       <c r="E6" s="1">
-        <v>0.966</v>
+        <v>1.102</v>
       </c>
       <c r="F6" s="1">
-        <v>1.057</v>
+        <v>1.313</v>
       </c>
       <c r="G6" s="1">
-        <v>1.184</v>
+        <v>1.494</v>
       </c>
       <c r="H6" s="1">
-        <v>1.33</v>
+        <v>1.625</v>
       </c>
       <c r="I6" s="1">
-        <v>1.395</v>
+        <v>1.645</v>
       </c>
       <c r="J6" s="1">
-        <v>1.311</v>
+        <v>1.564</v>
       </c>
       <c r="K6" s="1">
-        <v>1.12</v>
+        <v>1.419</v>
       </c>
       <c r="L6" s="1">
-        <v>0.918</v>
+        <v>1.198</v>
       </c>
       <c r="M6" s="1">
-        <v>0.727</v>
+        <v>0.867</v>
       </c>
       <c r="N6" s="1">
-        <v>0.502</v>
+        <v>0.474</v>
       </c>
       <c r="O6" s="1">
-        <v>0.242</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="P6" s="1">
-        <v>-0.007</v>
+        <v>-0.212</v>
       </c>
       <c r="Q6" s="1">
-        <v>-0.2</v>
+        <v>-0.357</v>
       </c>
       <c r="R6" s="1">
-        <v>-0.326</v>
+        <v>-0.399</v>
       </c>
       <c r="S6" s="1">
-        <v>-0.426</v>
+        <v>-0.451</v>
       </c>
       <c r="T6" s="1">
-        <v>-0.536</v>
+        <v>-0.5649999999999999</v>
       </c>
       <c r="U6" s="1">
-        <v>-0.638</v>
+        <v>-0.695</v>
       </c>
     </row>
     <row r="7" spans="1:21">
       <c r="A7" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="1">
-        <v>0.904</v>
+        <v>0.887</v>
       </c>
       <c r="C7" s="1">
-        <v>1.007</v>
+        <v>1.057</v>
       </c>
       <c r="D7" s="1">
-        <v>1.129</v>
+        <v>1.308</v>
       </c>
       <c r="E7" s="1">
-        <v>1.224</v>
+        <v>1.526</v>
       </c>
       <c r="F7" s="1">
-        <v>1.346</v>
+        <v>1.692</v>
       </c>
       <c r="G7" s="1">
-        <v>1.464</v>
+        <v>1.767</v>
       </c>
       <c r="H7" s="1">
-        <v>1.484</v>
+        <v>1.748</v>
       </c>
       <c r="I7" s="1">
-        <v>1.36</v>
+        <v>1.648</v>
       </c>
       <c r="J7" s="1">
-        <v>1.145</v>
+        <v>1.48</v>
       </c>
       <c r="K7" s="1">
-        <v>0.929</v>
+        <v>1.22</v>
       </c>
       <c r="L7" s="1">
-        <v>0.72</v>
+        <v>0.861</v>
       </c>
       <c r="M7" s="1">
-        <v>0.459</v>
+        <v>0.434</v>
       </c>
       <c r="N7" s="1">
-        <v>0.152</v>
+        <v>-0.012</v>
       </c>
       <c r="O7" s="1">
-        <v>-0.138</v>
+        <v>-0.368</v>
       </c>
       <c r="P7" s="1">
-        <v>-0.351</v>
+        <v>-0.529</v>
       </c>
       <c r="Q7" s="1">
-        <v>-0.477</v>
+        <v>-0.5610000000000001</v>
       </c>
       <c r="R7" s="1">
-        <v>-0.581</v>
+        <v>-0.614</v>
       </c>
       <c r="S7" s="1">
-        <v>-0.711</v>
+        <v>-0.757</v>
       </c>
       <c r="T7" s="1">
-        <v>-0.84</v>
+        <v>-0.919</v>
       </c>
       <c r="U7" s="1">
-        <v>-0.895</v>
+        <v>-0.964</v>
       </c>
     </row>
     <row r="8" spans="1:21">
       <c r="A8" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="1">
-        <v>1.051</v>
+        <v>1.033</v>
       </c>
       <c r="C8" s="1">
-        <v>1.164</v>
+        <v>1.216</v>
       </c>
       <c r="D8" s="1">
-        <v>1.332</v>
+        <v>1.497</v>
       </c>
       <c r="E8" s="1">
-        <v>1.484</v>
+        <v>1.706</v>
       </c>
       <c r="F8" s="1">
-        <v>1.578</v>
+        <v>1.792</v>
       </c>
       <c r="G8" s="1">
-        <v>1.538</v>
+        <v>1.735</v>
       </c>
       <c r="H8" s="1">
-        <v>1.351</v>
+        <v>1.588</v>
       </c>
       <c r="I8" s="1">
-        <v>1.097</v>
+        <v>1.408</v>
       </c>
       <c r="J8" s="1">
-        <v>0.872</v>
+        <v>1.157</v>
       </c>
       <c r="K8" s="1">
-        <v>0.662</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="L8" s="1">
-        <v>0.389</v>
+        <v>0.383</v>
       </c>
       <c r="M8" s="1">
-        <v>0.057</v>
+        <v>-0.054</v>
       </c>
       <c r="N8" s="1">
-        <v>-0.258</v>
+        <v>-0.4</v>
       </c>
       <c r="O8" s="1">
-        <v>-0.478</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="P8" s="1">
-        <v>-0.598</v>
+        <v>-0.606</v>
       </c>
       <c r="Q8" s="1">
-        <v>-0.702</v>
+        <v>-0.668</v>
       </c>
       <c r="R8" s="1">
-        <v>-0.849</v>
+        <v>-0.8120000000000001</v>
       </c>
       <c r="S8" s="1">
-        <v>-1.004</v>
+        <v>-0.985</v>
       </c>
       <c r="T8" s="1">
-        <v>-1.068</v>
+        <v>-1.037</v>
       </c>
       <c r="U8" s="1">
-        <v>-0.989</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="9" spans="1:21">
       <c r="A9" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="1">
-        <v>1.304</v>
+        <v>1.286</v>
       </c>
       <c r="C9" s="1">
-        <v>1.447</v>
+        <v>1.483</v>
       </c>
       <c r="D9" s="1">
-        <v>1.661</v>
+        <v>1.762</v>
       </c>
       <c r="E9" s="1">
-        <v>1.762</v>
+        <v>1.882</v>
       </c>
       <c r="F9" s="1">
-        <v>1.687</v>
+        <v>1.82</v>
       </c>
       <c r="G9" s="1">
-        <v>1.466</v>
+        <v>1.663</v>
       </c>
       <c r="H9" s="1">
-        <v>1.196</v>
+        <v>1.462</v>
       </c>
       <c r="I9" s="1">
-        <v>0.958</v>
+        <v>1.195</v>
       </c>
       <c r="J9" s="1">
-        <v>0.718</v>
+        <v>0.838</v>
       </c>
       <c r="K9" s="1">
-        <v>0.395</v>
+        <v>0.385</v>
       </c>
       <c r="L9" s="1">
-        <v>0.01</v>
+        <v>-0.097</v>
       </c>
       <c r="M9" s="1">
-        <v>-0.345</v>
+        <v>-0.475</v>
       </c>
       <c r="N9" s="1">
-        <v>-0.584</v>
+        <v>-0.641</v>
       </c>
       <c r="O9" s="1">
-        <v>-0.702</v>
+        <v>-0.678</v>
       </c>
       <c r="P9" s="1">
-        <v>-0.8070000000000001</v>
+        <v>-0.737</v>
       </c>
       <c r="Q9" s="1">
-        <v>-0.969</v>
+        <v>-0.889</v>
       </c>
       <c r="R9" s="1">
-        <v>-1.144</v>
+        <v>-1.078</v>
       </c>
       <c r="S9" s="1">
-        <v>-1.218</v>
+        <v>-1.141</v>
       </c>
       <c r="T9" s="1">
-        <v>-1.123</v>
+        <v>-1.015</v>
       </c>
       <c r="U9" s="1">
-        <v>-0.9340000000000001</v>
+        <v>-0.826</v>
       </c>
     </row>
     <row r="10" spans="1:21">
       <c r="A10" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="1">
-        <v>1.555</v>
+        <v>1.537</v>
       </c>
       <c r="C10" s="1">
-        <v>1.697</v>
+        <v>1.691</v>
       </c>
       <c r="D10" s="1">
-        <v>1.859</v>
+        <v>1.866</v>
       </c>
       <c r="E10" s="1">
-        <v>1.824</v>
+        <v>1.853</v>
       </c>
       <c r="F10" s="1">
-        <v>1.613</v>
+        <v>1.706</v>
       </c>
       <c r="G10" s="1">
-        <v>1.335</v>
+        <v>1.5</v>
       </c>
       <c r="H10" s="1">
-        <v>1.078</v>
+        <v>1.235</v>
       </c>
       <c r="I10" s="1">
-        <v>0.8169999999999999</v>
+        <v>0.873</v>
       </c>
       <c r="J10" s="1">
-        <v>0.483</v>
+        <v>0.427</v>
       </c>
       <c r="K10" s="1">
-        <v>0.095</v>
+        <v>-0.027</v>
       </c>
       <c r="L10" s="1">
-        <v>-0.262</v>
+        <v>-0.379</v>
       </c>
       <c r="M10" s="1">
-        <v>-0.506</v>
+        <v>-0.552</v>
       </c>
       <c r="N10" s="1">
-        <v>-0.635</v>
+        <v>-0.597</v>
       </c>
       <c r="O10" s="1">
-        <v>-0.742</v>
+        <v>-0.662</v>
       </c>
       <c r="P10" s="1">
-        <v>-0.896</v>
+        <v>-0.8110000000000001</v>
       </c>
       <c r="Q10" s="1">
-        <v>-1.059</v>
+        <v>-0.979</v>
       </c>
       <c r="R10" s="1">
-        <v>-1.128</v>
+        <v>-1.034</v>
       </c>
       <c r="S10" s="1">
-        <v>-1.041</v>
+        <v>-0.916</v>
       </c>
       <c r="T10" s="1">
-        <v>-0.865</v>
+        <v>-0.74</v>
       </c>
       <c r="U10" s="1">
-        <v>-0.704</v>
+        <v>-0.621</v>
       </c>
     </row>
     <row r="11" spans="1:21">
       <c r="A11" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="1">
-        <v>1.596</v>
+        <v>1.577</v>
       </c>
       <c r="C11" s="1">
-        <v>1.723</v>
+        <v>1.701</v>
       </c>
       <c r="D11" s="1">
-        <v>1.798</v>
+        <v>1.796</v>
       </c>
       <c r="E11" s="1">
-        <v>1.649</v>
+        <v>1.708</v>
       </c>
       <c r="F11" s="1">
-        <v>1.393</v>
+        <v>1.52</v>
       </c>
       <c r="G11" s="1">
-        <v>1.134</v>
+        <v>1.261</v>
       </c>
       <c r="H11" s="1">
-        <v>0.866</v>
+        <v>0.91</v>
       </c>
       <c r="I11" s="1">
-        <v>0.54</v>
+        <v>0.497</v>
       </c>
       <c r="J11" s="1">
-        <v>0.176</v>
+        <v>0.078</v>
       </c>
       <c r="K11" s="1">
-        <v>-0.154</v>
+        <v>-0.258</v>
       </c>
       <c r="L11" s="1">
-        <v>-0.383</v>
+        <v>-0.435</v>
       </c>
       <c r="M11" s="1">
-        <v>-0.512</v>
+        <v>-0.499</v>
       </c>
       <c r="N11" s="1">
-        <v>-0.616</v>
+        <v>-0.578</v>
       </c>
       <c r="O11" s="1">
-        <v>-0.749</v>
+        <v>-0.713</v>
       </c>
       <c r="P11" s="1">
-        <v>-0.884</v>
+        <v>-0.852</v>
       </c>
       <c r="Q11" s="1">
-        <v>-0.9399999999999999</v>
+        <v>-0.89</v>
       </c>
       <c r="R11" s="1">
-        <v>-0.866</v>
+        <v>-0.787</v>
       </c>
       <c r="S11" s="1">
-        <v>-0.718</v>
+        <v>-0.637</v>
       </c>
       <c r="T11" s="1">
-        <v>-0.581</v>
+        <v>-0.534</v>
       </c>
       <c r="U11" s="1">
-        <v>-0.49</v>
+        <v>-0.491</v>
       </c>
     </row>
     <row r="12" spans="1:21">
       <c r="A12" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="1">
-        <v>1.889</v>
+        <v>1.87</v>
       </c>
       <c r="C12" s="1">
-        <v>1.843</v>
+        <v>1.853</v>
       </c>
       <c r="D12" s="1">
-        <v>1.667</v>
+        <v>1.724</v>
       </c>
       <c r="E12" s="1">
-        <v>1.419</v>
+        <v>1.521</v>
       </c>
       <c r="F12" s="1">
-        <v>1.16</v>
+        <v>1.249</v>
       </c>
       <c r="G12" s="1">
-        <v>0.864</v>
+        <v>0.885</v>
       </c>
       <c r="H12" s="1">
-        <v>0.49</v>
+        <v>0.441</v>
       </c>
       <c r="I12" s="1">
-        <v>0.076</v>
+        <v>-0.022</v>
       </c>
       <c r="J12" s="1">
-        <v>-0.291</v>
+        <v>-0.387</v>
       </c>
       <c r="K12" s="1">
-        <v>-0.535</v>
+        <v>-0.5669999999999999</v>
       </c>
       <c r="L12" s="1">
-        <v>-0.664</v>
+        <v>-0.615</v>
       </c>
       <c r="M12" s="1">
-        <v>-0.773</v>
+        <v>-0.675</v>
       </c>
       <c r="N12" s="1">
-        <v>-0.927</v>
+        <v>-0.821</v>
       </c>
       <c r="O12" s="1">
-        <v>-1.089</v>
+        <v>-0.995</v>
       </c>
       <c r="P12" s="1">
-        <v>-1.154</v>
+        <v>-1.049</v>
       </c>
       <c r="Q12" s="1">
-        <v>-1.061</v>
+        <v>-0.929</v>
       </c>
       <c r="R12" s="1">
-        <v>-0.879</v>
+        <v>-0.75</v>
       </c>
       <c r="S12" s="1">
-        <v>-0.715</v>
+        <v>-0.622</v>
       </c>
       <c r="T12" s="1">
-        <v>-0.603</v>
+        <v>-0.571</v>
       </c>
       <c r="U12" s="1">
-        <v>-0.529</v>
+        <v>-0.5620000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:21">
       <c r="A13" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="1">
-        <v>1.975</v>
+        <v>1.955</v>
       </c>
       <c r="C13" s="1">
-        <v>1.859</v>
+        <v>1.871</v>
       </c>
       <c r="D13" s="1">
-        <v>1.593</v>
+        <v>1.641</v>
       </c>
       <c r="E13" s="1">
-        <v>1.296</v>
+        <v>1.311</v>
       </c>
       <c r="F13" s="1">
-        <v>0.957</v>
+        <v>0.888</v>
       </c>
       <c r="G13" s="1">
-        <v>0.535</v>
+        <v>0.396</v>
       </c>
       <c r="H13" s="1">
-        <v>0.068</v>
+        <v>-0.107</v>
       </c>
       <c r="I13" s="1">
-        <v>-0.352</v>
+        <v>-0.517</v>
       </c>
       <c r="J13" s="1">
-        <v>-0.641</v>
+        <v>-0.713</v>
       </c>
       <c r="K13" s="1">
-        <v>-0.793</v>
+        <v>-0.762</v>
       </c>
       <c r="L13" s="1">
-        <v>-0.916</v>
+        <v>-0.839</v>
       </c>
       <c r="M13" s="1">
-        <v>-1.088</v>
+        <v>-1.01</v>
       </c>
       <c r="N13" s="1">
-        <v>-1.271</v>
+        <v>-1.209</v>
       </c>
       <c r="O13" s="1">
-        <v>-1.347</v>
+        <v>-1.269</v>
       </c>
       <c r="P13" s="1">
-        <v>-1.244</v>
+        <v>-1.131</v>
       </c>
       <c r="Q13" s="1">
-        <v>-1.037</v>
+        <v>-0.926</v>
       </c>
       <c r="R13" s="1">
-        <v>-0.842</v>
+        <v>-0.772</v>
       </c>
       <c r="S13" s="1">
-        <v>-0.703</v>
+        <v>-0.694</v>
       </c>
       <c r="T13" s="1">
-        <v>-0.609</v>
+        <v>-0.656</v>
       </c>
       <c r="U13" s="1">
-        <v>-0.547</v>
+        <v>-0.61</v>
       </c>
     </row>
     <row r="14" spans="1:21">
       <c r="A14" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" s="1">
-        <v>1.78</v>
+        <v>1.76</v>
       </c>
       <c r="C14" s="1">
-        <v>1.668</v>
+        <v>1.646</v>
       </c>
       <c r="D14" s="1">
-        <v>1.389</v>
+        <v>1.346</v>
       </c>
       <c r="E14" s="1">
-        <v>0.99</v>
+        <v>0.9</v>
       </c>
       <c r="F14" s="1">
-        <v>0.473</v>
+        <v>0.355</v>
       </c>
       <c r="G14" s="1">
-        <v>-0.08400000000000001</v>
+        <v>-0.201</v>
       </c>
       <c r="H14" s="1">
-        <v>-0.5659999999999999</v>
+        <v>-0.639</v>
       </c>
       <c r="I14" s="1">
-        <v>-0.861</v>
+        <v>-0.836</v>
       </c>
       <c r="J14" s="1">
-        <v>-0.98</v>
+        <v>-0.871</v>
       </c>
       <c r="K14" s="1">
-        <v>-1.08</v>
+        <v>-0.9330000000000001</v>
       </c>
       <c r="L14" s="1">
-        <v>-1.26</v>
+        <v>-1.105</v>
       </c>
       <c r="M14" s="1">
-        <v>-1.467</v>
+        <v>-1.313</v>
       </c>
       <c r="N14" s="1">
-        <v>-1.546</v>
+        <v>-1.373</v>
       </c>
       <c r="O14" s="1">
-        <v>-1.408</v>
+        <v>-1.219</v>
       </c>
       <c r="P14" s="1">
-        <v>-1.16</v>
+        <v>-0.99</v>
       </c>
       <c r="Q14" s="1">
-        <v>-0.949</v>
+        <v>-0.821</v>
       </c>
       <c r="R14" s="1">
-        <v>-0.8139999999999999</v>
+        <v>-0.732</v>
       </c>
       <c r="S14" s="1">
-        <v>-0.731</v>
+        <v>-0.6870000000000001</v>
       </c>
       <c r="T14" s="1">
-        <v>-0.672</v>
+        <v>-0.644</v>
       </c>
       <c r="U14" s="1">
-        <v>-0.62</v>
+        <v>-0.574</v>
       </c>
     </row>
     <row r="15" spans="1:21">
       <c r="A15" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" s="1">
-        <v>1.537</v>
+        <v>1.517</v>
       </c>
       <c r="C15" s="1">
-        <v>1.359</v>
+        <v>1.31</v>
       </c>
       <c r="D15" s="1">
-        <v>0.987</v>
+        <v>0.877</v>
       </c>
       <c r="E15" s="1">
-        <v>0.498</v>
+        <v>0.346</v>
       </c>
       <c r="F15" s="1">
-        <v>-0.057</v>
+        <v>-0.217</v>
       </c>
       <c r="G15" s="1">
-        <v>-0.5620000000000001</v>
+        <v>-0.671</v>
       </c>
       <c r="H15" s="1">
-        <v>-0.888</v>
+        <v>-0.872</v>
       </c>
       <c r="I15" s="1">
-        <v>-1.023</v>
+        <v>-0.896</v>
       </c>
       <c r="J15" s="1">
-        <v>-1.129</v>
+        <v>-0.959</v>
       </c>
       <c r="K15" s="1">
-        <v>-1.319</v>
+        <v>-1.149</v>
       </c>
       <c r="L15" s="1">
-        <v>-1.541</v>
+        <v>-1.37</v>
       </c>
       <c r="M15" s="1">
-        <v>-1.634</v>
+        <v>-1.43</v>
       </c>
       <c r="N15" s="1">
-        <v>-1.501</v>
+        <v>-1.273</v>
       </c>
       <c r="O15" s="1">
-        <v>-1.242</v>
+        <v>-1.042</v>
       </c>
       <c r="P15" s="1">
-        <v>-1.016</v>
+        <v>-0.872</v>
       </c>
       <c r="Q15" s="1">
-        <v>-0.873</v>
+        <v>-0.794</v>
       </c>
       <c r="R15" s="1">
-        <v>-0.79</v>
+        <v>-0.763</v>
       </c>
       <c r="S15" s="1">
-        <v>-0.737</v>
+        <v>-0.73</v>
       </c>
       <c r="T15" s="1">
-        <v>-0.6929999999999999</v>
+        <v>-0.662</v>
       </c>
       <c r="U15" s="1">
-        <v>-0.655</v>
+        <v>-0.58</v>
       </c>
     </row>
     <row r="16" spans="1:21">
       <c r="A16" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" s="1">
-        <v>1.227</v>
+        <v>1.207</v>
       </c>
       <c r="C16" s="1">
-        <v>0.996</v>
+        <v>0.928</v>
       </c>
       <c r="D16" s="1">
-        <v>0.535</v>
+        <v>0.405</v>
       </c>
       <c r="E16" s="1">
-        <v>0.019</v>
+        <v>-0.138</v>
       </c>
       <c r="F16" s="1">
-        <v>-0.452</v>
+        <v>-0.5679999999999999</v>
       </c>
       <c r="G16" s="1">
-        <v>-0.764</v>
+        <v>-0.757</v>
       </c>
       <c r="H16" s="1">
-        <v>-0.902</v>
+        <v>-0.792</v>
       </c>
       <c r="I16" s="1">
-        <v>-1.003</v>
+        <v>-0.852</v>
       </c>
       <c r="J16" s="1">
-        <v>-1.171</v>
+        <v>-1.012</v>
       </c>
       <c r="K16" s="1">
-        <v>-1.368</v>
+        <v>-1.203</v>
       </c>
       <c r="L16" s="1">
-        <v>-1.461</v>
+        <v>-1.26</v>
       </c>
       <c r="M16" s="1">
-        <v>-1.355</v>
+        <v>-1.125</v>
       </c>
       <c r="N16" s="1">
-        <v>-1.127</v>
+        <v>-0.924</v>
       </c>
       <c r="O16" s="1">
-        <v>-0.916</v>
+        <v>-0.771</v>
       </c>
       <c r="P16" s="1">
-        <v>-0.774</v>
+        <v>-0.695</v>
       </c>
       <c r="Q16" s="1">
-        <v>-0.6889999999999999</v>
+        <v>-0.66</v>
       </c>
       <c r="R16" s="1">
-        <v>-0.639</v>
+        <v>-0.622</v>
       </c>
       <c r="S16" s="1">
-        <v>-0.603</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="T16" s="1">
-        <v>-0.575</v>
+        <v>-0.49</v>
       </c>
       <c r="U16" s="1">
-        <v>-0.573</v>
+        <v>-0.455</v>
       </c>
     </row>
     <row r="17" spans="1:21">
       <c r="A17" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" s="1">
-        <v>0.847</v>
+        <v>0.826</v>
       </c>
       <c r="C17" s="1">
-        <v>0.572</v>
+        <v>0.509</v>
       </c>
       <c r="D17" s="1">
-        <v>0.075</v>
+        <v>-0.039</v>
       </c>
       <c r="E17" s="1">
-        <v>-0.384</v>
+        <v>-0.473</v>
       </c>
       <c r="F17" s="1">
-        <v>-0.696</v>
+        <v>-0.672</v>
       </c>
       <c r="G17" s="1">
-        <v>-0.846</v>
+        <v>-0.717</v>
       </c>
       <c r="H17" s="1">
-        <v>-0.958</v>
+        <v>-0.789</v>
       </c>
       <c r="I17" s="1">
-        <v>-1.127</v>
+        <v>-0.961</v>
       </c>
       <c r="J17" s="1">
-        <v>-1.32</v>
+        <v>-1.158</v>
       </c>
       <c r="K17" s="1">
-        <v>-1.413</v>
+        <v>-1.213</v>
       </c>
       <c r="L17" s="1">
-        <v>-1.314</v>
+        <v>-1.074</v>
       </c>
       <c r="M17" s="1">
-        <v>-1.095</v>
+        <v>-0.876</v>
       </c>
       <c r="N17" s="1">
-        <v>-0.886</v>
+        <v>-0.738</v>
       </c>
       <c r="O17" s="1">
-        <v>-0.741</v>
+        <v>-0.6830000000000001</v>
       </c>
       <c r="P17" s="1">
-        <v>-0.654</v>
+        <v>-0.673</v>
       </c>
       <c r="Q17" s="1">
-        <v>-0.606</v>
+        <v>-0.658</v>
       </c>
       <c r="R17" s="1">
-        <v>-0.577</v>
+        <v>-0.607</v>
       </c>
       <c r="S17" s="1">
-        <v>-0.555</v>
+        <v>-0.537</v>
       </c>
       <c r="T17" s="1">
-        <v>-0.555</v>
+        <v>-0.5</v>
       </c>
       <c r="U17" s="1">
-        <v>-0.583</v>
+        <v>-0.524</v>
       </c>
     </row>
     <row r="18" spans="1:21">
       <c r="A18" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" s="1">
-        <v>0.315</v>
+        <v>0.293</v>
       </c>
       <c r="C18" s="1">
-        <v>0.008999999999999999</v>
+        <v>-0.01</v>
       </c>
       <c r="D18" s="1">
-        <v>-0.468</v>
+        <v>-0.446</v>
       </c>
       <c r="E18" s="1">
-        <v>-0.787</v>
+        <v>-0.661</v>
       </c>
       <c r="F18" s="1">
-        <v>-0.9360000000000001</v>
+        <v>-0.723</v>
       </c>
       <c r="G18" s="1">
-        <v>-1.042</v>
+        <v>-0.803</v>
       </c>
       <c r="H18" s="1">
-        <v>-1.204</v>
+        <v>-0.97</v>
       </c>
       <c r="I18" s="1">
-        <v>-1.385</v>
+        <v>-1.15</v>
       </c>
       <c r="J18" s="1">
-        <v>-1.464</v>
+        <v>-1.195</v>
       </c>
       <c r="K18" s="1">
-        <v>-1.359</v>
+        <v>-1.059</v>
       </c>
       <c r="L18" s="1">
-        <v>-1.14</v>
+        <v>-0.865</v>
       </c>
       <c r="M18" s="1">
-        <v>-0.926</v>
+        <v>-0.725</v>
       </c>
       <c r="N18" s="1">
-        <v>-0.762</v>
+        <v>-0.651</v>
       </c>
       <c r="O18" s="1">
-        <v>-0.642</v>
+        <v>-0.616</v>
       </c>
       <c r="P18" s="1">
-        <v>-0.5639999999999999</v>
+        <v>-0.582</v>
       </c>
       <c r="Q18" s="1">
-        <v>-0.518</v>
+        <v>-0.523</v>
       </c>
       <c r="R18" s="1">
-        <v>-0.488</v>
+        <v>-0.453</v>
       </c>
       <c r="S18" s="1">
-        <v>-0.478</v>
+        <v>-0.416</v>
       </c>
       <c r="T18" s="1">
-        <v>-0.487</v>
+        <v>-0.429</v>
       </c>
       <c r="U18" s="1">
-        <v>-0.489</v>
+        <v>-0.461</v>
       </c>
     </row>
     <row r="19" spans="1:21">
       <c r="A19" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" s="1">
-        <v>0.252</v>
+        <v>0.231</v>
       </c>
       <c r="C19" s="1">
-        <v>0.024</v>
+        <v>0.042</v>
       </c>
       <c r="D19" s="1">
-        <v>-0.301</v>
+        <v>-0.201</v>
       </c>
       <c r="E19" s="1">
-        <v>-0.496</v>
+        <v>-0.327</v>
       </c>
       <c r="F19" s="1">
-        <v>-0.648</v>
+        <v>-0.453</v>
       </c>
       <c r="G19" s="1">
-        <v>-0.822</v>
+        <v>-0.628</v>
       </c>
       <c r="H19" s="1">
-        <v>-0.989</v>
+        <v>-0.793</v>
       </c>
       <c r="I19" s="1">
-        <v>-1.064</v>
+        <v>-0.834</v>
       </c>
       <c r="J19" s="1">
-        <v>-0.986</v>
+        <v>-0.724</v>
       </c>
       <c r="K19" s="1">
-        <v>-0.8120000000000001</v>
+        <v>-0.571</v>
       </c>
       <c r="L19" s="1">
+        <v>-0.484</v>
+      </c>
+      <c r="M19" s="1">
+        <v>-0.499</v>
+      </c>
+      <c r="N19" s="1">
+        <v>-0.5679999999999999</v>
+      </c>
+      <c r="O19" s="1">
+        <v>-0.613</v>
+      </c>
+      <c r="P19" s="1">
+        <v>-0.59</v>
+      </c>
+      <c r="Q19" s="1">
+        <v>-0.537</v>
+      </c>
+      <c r="R19" s="1">
+        <v>-0.518</v>
+      </c>
+      <c r="S19" s="1">
+        <v>-0.5629999999999999</v>
+      </c>
+      <c r="T19" s="1">
+        <v>-0.634</v>
+      </c>
+      <c r="U19" s="1">
         <v>-0.654</v>
-      </c>
-      <c r="M19" s="1">
-        <v>-0.569</v>
-      </c>
-      <c r="N19" s="1">
-        <v>-0.548</v>
-      </c>
-      <c r="O19" s="1">
-        <v>-0.5600000000000001</v>
-      </c>
-      <c r="P19" s="1">
-        <v>-0.5679999999999999</v>
-      </c>
-      <c r="Q19" s="1">
-        <v>-0.5639999999999999</v>
-      </c>
-      <c r="R19" s="1">
-        <v>-0.579</v>
-      </c>
-      <c r="S19" s="1">
-        <v>-0.627</v>
-      </c>
-      <c r="T19" s="1">
-        <v>-0.673</v>
-      </c>
-      <c r="U19" s="1">
-        <v>-0.679</v>
       </c>
     </row>
     <row r="20" spans="1:21">
       <c r="A20" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="1">
-        <v>0.192</v>
+        <v>0.17</v>
       </c>
       <c r="C20" s="1">
-        <v>0.07199999999999999</v>
+        <v>0.098</v>
       </c>
       <c r="D20" s="1">
-        <v>-0.115</v>
+        <v>-0.014</v>
       </c>
       <c r="E20" s="1">
-        <v>-0.284</v>
+        <v>-0.14</v>
       </c>
       <c r="F20" s="1">
-        <v>-0.451</v>
+        <v>-0.29</v>
       </c>
       <c r="G20" s="1">
-        <v>-0.586</v>
+        <v>-0.416</v>
       </c>
       <c r="H20" s="1">
-        <v>-0.645</v>
+        <v>-0.441</v>
       </c>
       <c r="I20" s="1">
-        <v>-0.596</v>
+        <v>-0.356</v>
       </c>
       <c r="J20" s="1">
-        <v>-0.481</v>
+        <v>-0.26</v>
       </c>
       <c r="K20" s="1">
-        <v>-0.382</v>
+        <v>-0.239</v>
       </c>
       <c r="L20" s="1">
-        <v>-0.35</v>
+        <v>-0.294</v>
       </c>
       <c r="M20" s="1">
-        <v>-0.381</v>
+        <v>-0.393</v>
       </c>
       <c r="N20" s="1">
-        <v>-0.438</v>
+        <v>-0.47</v>
       </c>
       <c r="O20" s="1">
-        <v>-0.481</v>
+        <v>-0.479</v>
       </c>
       <c r="P20" s="1">
-        <v>-0.502</v>
+        <v>-0.455</v>
       </c>
       <c r="Q20" s="1">
-        <v>-0.532</v>
+        <v>-0.462</v>
       </c>
       <c r="R20" s="1">
-        <v>-0.589</v>
+        <v>-0.52</v>
       </c>
       <c r="S20" s="1">
-        <v>-0.643</v>
+        <v>-0.592</v>
       </c>
       <c r="T20" s="1">
-        <v>-0.656</v>
+        <v>-0.612</v>
       </c>
       <c r="U20" s="1">
-        <v>-0.619</v>
+        <v>-0.5600000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:21">
       <c r="A21" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" s="1">
-        <v>-0.051</v>
+        <v>-0.073</v>
       </c>
       <c r="C21" s="1">
-        <v>-0.112</v>
+        <v>-0.092</v>
       </c>
       <c r="D21" s="1">
-        <v>-0.241</v>
+        <v>-0.178</v>
       </c>
       <c r="E21" s="1">
-        <v>-0.394</v>
+        <v>-0.322</v>
       </c>
       <c r="F21" s="1">
-        <v>-0.54</v>
+        <v>-0.44</v>
       </c>
       <c r="G21" s="1">
-        <v>-0.618</v>
+        <v>-0.454</v>
       </c>
       <c r="H21" s="1">
-        <v>-0.583</v>
+        <v>-0.364</v>
       </c>
       <c r="I21" s="1">
-        <v>-0.471</v>
+        <v>-0.271</v>
       </c>
       <c r="J21" s="1">
-        <v>-0.375</v>
+        <v>-0.256</v>
       </c>
       <c r="K21" s="1">
-        <v>-0.358</v>
+        <v>-0.321</v>
       </c>
       <c r="L21" s="1">
-        <v>-0.411</v>
+        <v>-0.43</v>
       </c>
       <c r="M21" s="1">
-        <v>-0.488</v>
+        <v>-0.52</v>
       </c>
       <c r="N21" s="1">
-        <v>-0.541</v>
+        <v>-0.534</v>
       </c>
       <c r="O21" s="1">
-        <v>-0.5659999999999999</v>
+        <v>-0.505</v>
       </c>
       <c r="P21" s="1">
-        <v>-0.603</v>
+        <v>-0.502</v>
       </c>
       <c r="Q21" s="1">
-        <v>-0.674</v>
+        <v>-0.5590000000000001</v>
       </c>
       <c r="R21" s="1">
-        <v>-0.745</v>
+        <v>-0.64</v>
       </c>
       <c r="S21" s="1">
-        <v>-0.766</v>
+        <v>-0.661</v>
       </c>
       <c r="T21" s="1">
-        <v>-0.722</v>
+        <v>-0.598</v>
       </c>
       <c r="U21" s="1">
-        <v>-0.63</v>
+        <v>-0.504</v>
       </c>
     </row>
     <row r="22" spans="1:21">
       <c r="A22" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" s="1">
-        <v>-0.217</v>
+        <v>-0.239</v>
       </c>
       <c r="C22" s="1">
-        <v>-0.286</v>
+        <v>-0.292</v>
       </c>
       <c r="D22" s="1">
-        <v>-0.433</v>
+        <v>-0.415</v>
       </c>
       <c r="E22" s="1">
-        <v>-0.585</v>
+        <v>-0.534</v>
       </c>
       <c r="F22" s="1">
-        <v>-0.676</v>
+        <v>-0.551</v>
       </c>
       <c r="G22" s="1">
-        <v>-0.646</v>
+        <v>-0.459</v>
       </c>
       <c r="H22" s="1">
-        <v>-0.526</v>
+        <v>-0.353</v>
       </c>
       <c r="I22" s="1">
-        <v>-0.42</v>
+        <v>-0.32</v>
       </c>
       <c r="J22" s="1">
-        <v>-0.396</v>
+        <v>-0.378</v>
       </c>
       <c r="K22" s="1">
-        <v>-0.45</v>
+        <v>-0.482</v>
       </c>
       <c r="L22" s="1">
-        <v>-0.53</v>
+        <v>-0.5590000000000001</v>
       </c>
       <c r="M22" s="1">
-        <v>-0.585</v>
+        <v>-0.5659999999999999</v>
       </c>
       <c r="N22" s="1">
-        <v>-0.609</v>
+        <v>-0.535</v>
       </c>
       <c r="O22" s="1">
-        <v>-0.647</v>
+        <v>-0.537</v>
       </c>
       <c r="P22" s="1">
-        <v>-0.724</v>
+        <v>-0.6</v>
       </c>
       <c r="Q22" s="1">
-        <v>-0.801</v>
+        <v>-0.6830000000000001</v>
       </c>
       <c r="R22" s="1">
-        <v>-0.823</v>
+        <v>-0.706</v>
       </c>
       <c r="S22" s="1">
-        <v>-0.775</v>
+        <v>-0.643</v>
       </c>
       <c r="T22" s="1">
-        <v>-0.677</v>
+        <v>-0.543</v>
       </c>
       <c r="U22" s="1">
-        <v>-0.548</v>
+        <v>-0.446</v>
       </c>
     </row>
     <row r="23" spans="1:21">
       <c r="A23" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" s="1">
-        <v>-0.285</v>
+        <v>-0.308</v>
       </c>
       <c r="C23" s="1">
-        <v>-0.412</v>
+        <v>-0.424</v>
       </c>
       <c r="D23" s="1">
-        <v>-0.585</v>
+        <v>-0.5629999999999999</v>
       </c>
       <c r="E23" s="1">
-        <v>-0.646</v>
+        <v>-0.55</v>
       </c>
       <c r="F23" s="1">
-        <v>-0.571</v>
+        <v>-0.409</v>
       </c>
       <c r="G23" s="1">
-        <v>-0.431</v>
+        <v>-0.281</v>
       </c>
       <c r="H23" s="1">
-        <v>-0.337</v>
+        <v>-0.258</v>
       </c>
       <c r="I23" s="1">
-        <v>-0.343</v>
+        <v>-0.333</v>
       </c>
       <c r="J23" s="1">
+        <v>-0.453</v>
+      </c>
+      <c r="K23" s="1">
+        <v>-0.547</v>
+      </c>
+      <c r="L23" s="1">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="M23" s="1">
+        <v>-0.524</v>
+      </c>
+      <c r="N23" s="1">
+        <v>-0.513</v>
+      </c>
+      <c r="O23" s="1">
+        <v>-0.5669999999999999</v>
+      </c>
+      <c r="P23" s="1">
+        <v>-0.649</v>
+      </c>
+      <c r="Q23" s="1">
+        <v>-0.675</v>
+      </c>
+      <c r="R23" s="1">
+        <v>-0.619</v>
+      </c>
+      <c r="S23" s="1">
+        <v>-0.522</v>
+      </c>
+      <c r="T23" s="1">
         <v>-0.425</v>
       </c>
-      <c r="K23" s="1">
-        <v>-0.523</v>
-      </c>
-      <c r="L23" s="1">
-        <v>-0.582</v>
-      </c>
-      <c r="M23" s="1">
-        <v>-0.604</v>
-      </c>
-      <c r="N23" s="1">
-        <v>-0.639</v>
-      </c>
-      <c r="O23" s="1">
-        <v>-0.712</v>
-      </c>
-      <c r="P23" s="1">
-        <v>-0.785</v>
-      </c>
-      <c r="Q23" s="1">
-        <v>-0.803</v>
-      </c>
-      <c r="R23" s="1">
-        <v>-0.75</v>
-      </c>
-      <c r="S23" s="1">
-        <v>-0.649</v>
-      </c>
-      <c r="T23" s="1">
-        <v>-0.523</v>
-      </c>
       <c r="U23" s="1">
-        <v>-0.375</v>
+        <v>-0.335</v>
       </c>
     </row>
     <row r="24" spans="1:21">
       <c r="A24" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" s="1">
-        <v>-0.095</v>
+        <v>-0.118</v>
       </c>
       <c r="C24" s="1">
-        <v>-0.183</v>
+        <v>-0.172</v>
       </c>
       <c r="D24" s="1">
-        <v>-0.276</v>
+        <v>-0.197</v>
       </c>
       <c r="E24" s="1">
-        <v>-0.265</v>
+        <v>-0.139</v>
       </c>
       <c r="F24" s="1">
-        <v>-0.192</v>
+        <v>-0.08</v>
       </c>
       <c r="G24" s="1">
-        <v>-0.146</v>
+        <v>-0.089</v>
       </c>
       <c r="H24" s="1">
-        <v>-0.186</v>
+        <v>-0.181</v>
       </c>
       <c r="I24" s="1">
-        <v>-0.295</v>
+        <v>-0.316</v>
       </c>
       <c r="J24" s="1">
-        <v>-0.417</v>
+        <v>-0.428</v>
       </c>
       <c r="K24" s="1">
-        <v>-0.498</v>
+        <v>-0.466</v>
       </c>
       <c r="L24" s="1">
-        <v>-0.536</v>
+        <v>-0.448</v>
       </c>
       <c r="M24" s="1">
-        <v>-0.581</v>
+        <v>-0.453</v>
       </c>
       <c r="N24" s="1">
-        <v>-0.662</v>
+        <v>-0.521</v>
       </c>
       <c r="O24" s="1">
-        <v>-0.743</v>
+        <v>-0.616</v>
       </c>
       <c r="P24" s="1">
-        <v>-0.766</v>
+        <v>-0.651</v>
       </c>
       <c r="Q24" s="1">
-        <v>-0.713</v>
+        <v>-0.597</v>
       </c>
       <c r="R24" s="1">
-        <v>-0.612</v>
+        <v>-0.504</v>
       </c>
       <c r="S24" s="1">
-        <v>-0.495</v>
+        <v>-0.422</v>
       </c>
       <c r="T24" s="1">
-        <v>-0.37</v>
+        <v>-0.353</v>
       </c>
       <c r="U24" s="1">
-        <v>-0.245</v>
+        <v>-0.282</v>
       </c>
     </row>
     <row r="25" spans="1:21">
       <c r="A25" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" s="1">
-        <v>-0.59</v>
+        <v>-0.613</v>
       </c>
       <c r="C25" s="1">
         <v>-0.588</v>
       </c>
       <c r="D25" s="1">
-        <v>-0.515</v>
+        <v>-0.487</v>
       </c>
       <c r="E25" s="1">
-        <v>-0.389</v>
+        <v>-0.372</v>
       </c>
       <c r="F25" s="1">
-        <v>-0.301</v>
+        <v>-0.318</v>
       </c>
       <c r="G25" s="1">
-        <v>-0.282</v>
+        <v>-0.326</v>
       </c>
       <c r="H25" s="1">
-        <v>-0.32</v>
+        <v>-0.363</v>
       </c>
       <c r="I25" s="1">
-        <v>-0.38</v>
+        <v>-0.391</v>
       </c>
       <c r="J25" s="1">
-        <v>-0.427</v>
+        <v>-0.379</v>
       </c>
       <c r="K25" s="1">
-        <v>-0.451</v>
+        <v>-0.349</v>
       </c>
       <c r="L25" s="1">
-        <v>-0.476</v>
+        <v>-0.333</v>
       </c>
       <c r="M25" s="1">
-        <v>-0.513</v>
+        <v>-0.339</v>
       </c>
       <c r="N25" s="1">
-        <v>-0.541</v>
+        <v>-0.354</v>
       </c>
       <c r="O25" s="1">
-        <v>-0.54</v>
+        <v>-0.344</v>
       </c>
       <c r="P25" s="1">
-        <v>-0.506</v>
+        <v>-0.307</v>
       </c>
       <c r="Q25" s="1">
-        <v>-0.443</v>
+        <v>-0.261</v>
       </c>
       <c r="R25" s="1">
-        <v>-0.347</v>
+        <v>-0.212</v>
       </c>
       <c r="S25" s="1">
-        <v>-0.218</v>
+        <v>-0.145</v>
       </c>
       <c r="T25" s="1">
-        <v>-0.078</v>
+        <v>-0.062</v>
       </c>
       <c r="U25" s="1">
-        <v>0.031</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="26" spans="1:21">
       <c r="A26" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B26" s="1">
-        <v>-0.726</v>
+        <v>-0.749</v>
       </c>
       <c r="C26" s="1">
-        <v>-0.635</v>
+        <v>-0.647</v>
       </c>
       <c r="D26" s="1">
-        <v>-0.475</v>
+        <v>-0.493</v>
       </c>
       <c r="E26" s="1">
-        <v>-0.374</v>
+        <v>-0.414</v>
       </c>
       <c r="F26" s="1">
-        <v>-0.376</v>
+        <v>-0.421</v>
       </c>
       <c r="G26" s="1">
-        <v>-0.457</v>
+        <v>-0.48</v>
       </c>
       <c r="H26" s="1">
-        <v>-0.5590000000000001</v>
+        <v>-0.528</v>
       </c>
       <c r="I26" s="1">
-        <v>-0.621</v>
+        <v>-0.526</v>
       </c>
       <c r="J26" s="1">
-        <v>-0.64</v>
+        <v>-0.496</v>
       </c>
       <c r="K26" s="1">
-        <v>-0.666</v>
+        <v>-0.481</v>
       </c>
       <c r="L26" s="1">
-        <v>-0.728</v>
+        <v>-0.507</v>
       </c>
       <c r="M26" s="1">
-        <v>-0.79</v>
+        <v>-0.5570000000000001</v>
       </c>
       <c r="N26" s="1">
-        <v>-0.798</v>
+        <v>-0.5679999999999999</v>
       </c>
       <c r="O26" s="1">
-        <v>-0.742</v>
+        <v>-0.518</v>
       </c>
       <c r="P26" s="1">
-        <v>-0.643</v>
+        <v>-0.444</v>
       </c>
       <c r="Q26" s="1">
-        <v>-0.517</v>
+        <v>-0.361</v>
       </c>
       <c r="R26" s="1">
-        <v>-0.361</v>
+        <v>-0.262</v>
       </c>
       <c r="S26" s="1">
-        <v>-0.19</v>
+        <v>-0.149</v>
       </c>
       <c r="T26" s="1">
-        <v>-0.049</v>
+        <v>-0.042</v>
       </c>
       <c r="U26" s="1">
-        <v>0.036</v>
+        <v>0.049</v>
       </c>
     </row>
     <row r="27" spans="1:21">
       <c r="A27" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" s="1">
-        <v>-0.344</v>
+        <v>-0.368</v>
       </c>
       <c r="C27" s="1">
-        <v>-0.24</v>
+        <v>-0.28</v>
       </c>
       <c r="D27" s="1">
-        <v>-0.139</v>
+        <v>-0.217</v>
       </c>
       <c r="E27" s="1">
-        <v>-0.166</v>
+        <v>-0.267</v>
       </c>
       <c r="F27" s="1">
-        <v>-0.282</v>
+        <v>-0.368</v>
       </c>
       <c r="G27" s="1">
-        <v>-0.407</v>
+        <v>-0.434</v>
       </c>
       <c r="H27" s="1">
-        <v>-0.477</v>
+        <v>-0.417</v>
       </c>
       <c r="I27" s="1">
-        <v>-0.501</v>
+        <v>-0.37</v>
       </c>
       <c r="J27" s="1">
-        <v>-0.528</v>
+        <v>-0.353</v>
       </c>
       <c r="K27" s="1">
-        <v>-0.581</v>
+        <v>-0.378</v>
       </c>
       <c r="L27" s="1">
-        <v>-0.633</v>
+        <v>-0.412</v>
       </c>
       <c r="M27" s="1">
-        <v>-0.645</v>
+        <v>-0.412</v>
       </c>
       <c r="N27" s="1">
-        <v>-0.598</v>
+        <v>-0.366</v>
       </c>
       <c r="O27" s="1">
-        <v>-0.51</v>
+        <v>-0.303</v>
       </c>
       <c r="P27" s="1">
-        <v>-0.399</v>
+        <v>-0.242</v>
       </c>
       <c r="Q27" s="1">
-        <v>-0.273</v>
+        <v>-0.182</v>
       </c>
       <c r="R27" s="1">
-        <v>-0.149</v>
+        <v>-0.118</v>
       </c>
       <c r="S27" s="1">
-        <v>-0.057</v>
+        <v>-0.053</v>
       </c>
       <c r="T27" s="1">
-        <v>-0.006</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="U27" s="1">
-        <v>0.024</v>
+        <v>0.064</v>
       </c>
     </row>
     <row r="28" spans="1:21">
       <c r="A28" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" s="1">
-        <v>0.128</v>
+        <v>0.104</v>
       </c>
       <c r="C28" s="1">
-        <v>0.129</v>
+        <v>0.082</v>
       </c>
       <c r="D28" s="1">
-        <v>0.081</v>
+        <v>0.02</v>
       </c>
       <c r="E28" s="1">
-        <v>-0.027</v>
+        <v>-0.059</v>
       </c>
       <c r="F28" s="1">
-        <v>-0.143</v>
+        <v>-0.115</v>
       </c>
       <c r="G28" s="1">
-        <v>-0.222</v>
+        <v>-0.12</v>
       </c>
       <c r="H28" s="1">
-        <v>-0.263</v>
+        <v>-0.098</v>
       </c>
       <c r="I28" s="1">
-        <v>-0.296</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="J28" s="1">
-        <v>-0.337</v>
+        <v>-0.098</v>
       </c>
       <c r="K28" s="1">
-        <v>-0.377</v>
+        <v>-0.126</v>
       </c>
       <c r="L28" s="1">
-        <v>-0.392</v>
+        <v>-0.14</v>
       </c>
       <c r="M28" s="1">
-        <v>-0.368</v>
+        <v>-0.12</v>
       </c>
       <c r="N28" s="1">
-        <v>-0.311</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="O28" s="1">
-        <v>-0.241</v>
+        <v>-0.073</v>
       </c>
       <c r="P28" s="1">
-        <v>-0.172</v>
+        <v>-0.081</v>
       </c>
       <c r="Q28" s="1">
-        <v>-0.115</v>
+        <v>-0.08699999999999999</v>
       </c>
       <c r="R28" s="1">
-        <v>-0.079</v>
+        <v>-0.08699999999999999</v>
       </c>
       <c r="S28" s="1">
-        <v>-0.063</v>
+        <v>-0.066</v>
       </c>
       <c r="T28" s="1">
-        <v>-0.056</v>
+        <v>-0.031</v>
       </c>
       <c r="U28" s="1">
-        <v>-0.046</v>
+        <v>-0.001</v>
       </c>
     </row>
     <row r="29" spans="1:21">
       <c r="A29" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" s="1">
-        <v>-0.118</v>
+        <v>-0.142</v>
       </c>
       <c r="C29" s="1">
-        <v>-0.105</v>
+        <v>-0.145</v>
       </c>
       <c r="D29" s="1">
-        <v>-0.114</v>
+        <v>-0.149</v>
       </c>
       <c r="E29" s="1">
-        <v>-0.141</v>
+        <v>-0.123</v>
       </c>
       <c r="F29" s="1">
-        <v>-0.153</v>
+        <v>-0.061</v>
       </c>
       <c r="G29" s="1">
-        <v>-0.154</v>
+        <v>-0.002</v>
       </c>
       <c r="H29" s="1">
-        <v>-0.154</v>
+        <v>0.039</v>
       </c>
       <c r="I29" s="1">
-        <v>-0.15</v>
+        <v>0.067</v>
       </c>
       <c r="J29" s="1">
-        <v>-0.142</v>
+        <v>0.076</v>
       </c>
       <c r="K29" s="1">
-        <v>-0.134</v>
+        <v>0.076</v>
       </c>
       <c r="L29" s="1">
-        <v>-0.125</v>
+        <v>0.081</v>
       </c>
       <c r="M29" s="1">
-        <v>-0.104</v>
+        <v>0.076</v>
       </c>
       <c r="N29" s="1">
-        <v>-0.064</v>
+        <v>0.055</v>
       </c>
       <c r="O29" s="1">
-        <v>-0.014</v>
+        <v>0.031</v>
       </c>
       <c r="P29" s="1">
-        <v>0.029</v>
+        <v>0.018</v>
       </c>
       <c r="Q29" s="1">
-        <v>0.051</v>
+        <v>0.016</v>
       </c>
       <c r="R29" s="1">
-        <v>0.052</v>
+        <v>0.025</v>
       </c>
       <c r="S29" s="1">
         <v>0.049</v>
       </c>
       <c r="T29" s="1">
-        <v>0.058</v>
+        <v>0.08</v>
       </c>
       <c r="U29" s="1">
-        <v>0.081</v>
+        <v>0.096</v>
       </c>
     </row>
     <row r="30" spans="1:21">
       <c r="A30" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" s="1">
-        <v>-0.025</v>
+        <v>-0.05</v>
       </c>
       <c r="C30" s="1">
-        <v>-0.045</v>
+        <v>-0.061</v>
       </c>
       <c r="D30" s="1">
-        <v>-0.079</v>
+        <v>-0.053</v>
       </c>
       <c r="E30" s="1">
-        <v>-0.099</v>
+        <v>-0.017</v>
       </c>
       <c r="F30" s="1">
-        <v>-0.114</v>
+        <v>0.021</v>
       </c>
       <c r="G30" s="1">
-        <v>-0.14</v>
+        <v>0.04</v>
       </c>
       <c r="H30" s="1">
-        <v>-0.176</v>
+        <v>0.031</v>
       </c>
       <c r="I30" s="1">
-        <v>-0.209</v>
+        <v>0.002</v>
       </c>
       <c r="J30" s="1">
-        <v>-0.226</v>
+        <v>-0.02</v>
       </c>
       <c r="K30" s="1">
-        <v>-0.215</v>
+        <v>-0.006</v>
       </c>
       <c r="L30" s="1">
-        <v>-0.18</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="M30" s="1">
-        <v>-0.139</v>
+        <v>-0.01</v>
       </c>
       <c r="N30" s="1">
-        <v>-0.112</v>
+        <v>-0.051</v>
       </c>
       <c r="O30" s="1">
-        <v>-0.103</v>
+        <v>-0.106</v>
       </c>
       <c r="P30" s="1">
-        <v>-0.106</v>
+        <v>-0.149</v>
       </c>
       <c r="Q30" s="1">
-        <v>-0.114</v>
+        <v>-0.154</v>
       </c>
       <c r="R30" s="1">
-        <v>-0.121</v>
+        <v>-0.134</v>
       </c>
       <c r="S30" s="1">
-        <v>-0.129</v>
+        <v>-0.126</v>
       </c>
       <c r="T30" s="1">
-        <v>-0.14</v>
+        <v>-0.147</v>
       </c>
       <c r="U30" s="1">
-        <v>-0.149</v>
+        <v>-0.183</v>
       </c>
     </row>
     <row r="31" spans="1:21">
       <c r="A31" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31" s="1">
-        <v>0.024</v>
+        <v>-0.001</v>
       </c>
       <c r="C31" s="1">
-        <v>-0</v>
+        <v>0.012</v>
       </c>
       <c r="D31" s="1">
-        <v>-0.035</v>
+        <v>0.033</v>
       </c>
       <c r="E31" s="1">
-        <v>-0.058</v>
+        <v>0.055</v>
       </c>
       <c r="F31" s="1">
-        <v>-0.102</v>
+        <v>0.05</v>
       </c>
       <c r="G31" s="1">
-        <v>-0.181</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="H31" s="1">
-        <v>-0.26</v>
+        <v>-0.063</v>
       </c>
       <c r="I31" s="1">
-        <v>-0.294</v>
+        <v>-0.115</v>
       </c>
       <c r="J31" s="1">
-        <v>-0.272</v>
+        <v>-0.114</v>
       </c>
       <c r="K31" s="1">
-        <v>-0.222</v>
+        <v>-0.08799999999999999</v>
       </c>
       <c r="L31" s="1">
-        <v>-0.196</v>
+        <v>-0.093</v>
       </c>
       <c r="M31" s="1">
+        <v>-0.143</v>
+      </c>
+      <c r="N31" s="1">
         <v>-0.215</v>
       </c>
-      <c r="N31" s="1">
-        <v>-0.261</v>
-      </c>
       <c r="O31" s="1">
-        <v>-0.301</v>
+        <v>-0.28</v>
       </c>
       <c r="P31" s="1">
-        <v>-0.315</v>
+        <v>-0.298</v>
       </c>
       <c r="Q31" s="1">
-        <v>-0.316</v>
+        <v>-0.284</v>
       </c>
       <c r="R31" s="1">
-        <v>-0.337</v>
+        <v>-0.278</v>
       </c>
       <c r="S31" s="1">
-        <v>-0.39</v>
+        <v>-0.313</v>
       </c>
       <c r="T31" s="1">
-        <v>-0.446</v>
+        <v>-0.376</v>
       </c>
       <c r="U31" s="1">
-        <v>-0.46</v>
+        <v>-0.399</v>
       </c>
     </row>
     <row r="32" spans="1:21">
       <c r="A32" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B32" s="1">
-        <v>-0.062</v>
+        <v>-0.08799999999999999</v>
       </c>
       <c r="C32" s="1">
-        <v>-0.097</v>
+        <v>-0.083</v>
       </c>
       <c r="D32" s="1">
-        <v>-0.161</v>
+        <v>-0.089</v>
       </c>
       <c r="E32" s="1">
+        <v>-0.118</v>
+      </c>
+      <c r="F32" s="1">
+        <v>-0.196</v>
+      </c>
+      <c r="G32" s="1">
+        <v>-0.286</v>
+      </c>
+      <c r="H32" s="1">
+        <v>-0.32</v>
+      </c>
+      <c r="I32" s="1">
+        <v>-0.284</v>
+      </c>
+      <c r="J32" s="1">
+        <v>-0.221</v>
+      </c>
+      <c r="K32" s="1">
+        <v>-0.184</v>
+      </c>
+      <c r="L32" s="1">
+        <v>-0.2</v>
+      </c>
+      <c r="M32" s="1">
         <v>-0.248</v>
       </c>
-      <c r="F32" s="1">
-        <v>-0.366</v>
-      </c>
-      <c r="G32" s="1">
-        <v>-0.47</v>
-      </c>
-      <c r="H32" s="1">
-        <v>-0.511</v>
-      </c>
-      <c r="I32" s="1">
-        <v>-0.475</v>
-      </c>
-      <c r="J32" s="1">
-        <v>-0.397</v>
-      </c>
-      <c r="K32" s="1">
-        <v>-0.333</v>
-      </c>
-      <c r="L32" s="1">
-        <v>-0.313</v>
-      </c>
-      <c r="M32" s="1">
-        <v>-0.327</v>
-      </c>
       <c r="N32" s="1">
-        <v>-0.348</v>
+        <v>-0.28</v>
       </c>
       <c r="O32" s="1">
-        <v>-0.356</v>
+        <v>-0.274</v>
       </c>
       <c r="P32" s="1">
-        <v>-0.355</v>
+        <v>-0.251</v>
       </c>
       <c r="Q32" s="1">
-        <v>-0.373</v>
+        <v>-0.247</v>
       </c>
       <c r="R32" s="1">
-        <v>-0.423</v>
+        <v>-0.282</v>
       </c>
       <c r="S32" s="1">
-        <v>-0.473</v>
+        <v>-0.33</v>
       </c>
       <c r="T32" s="1">
-        <v>-0.486</v>
+        <v>-0.343</v>
       </c>
       <c r="U32" s="1">
-        <v>-0.456</v>
+        <v>-0.311</v>
       </c>
     </row>
     <row r="33" spans="1:21">
       <c r="A33" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33" s="1">
-        <v>-0.306</v>
+        <v>-0.332</v>
       </c>
       <c r="C33" s="1">
-        <v>-0.331</v>
+        <v>-0.324</v>
       </c>
       <c r="D33" s="1">
-        <v>-0.418</v>
+        <v>-0.352</v>
       </c>
       <c r="E33" s="1">
-        <v>-0.55</v>
+        <v>-0.443</v>
       </c>
       <c r="F33" s="1">
-        <v>-0.654</v>
+        <v>-0.528</v>
       </c>
       <c r="G33" s="1">
-        <v>-0.671</v>
+        <v>-0.524</v>
       </c>
       <c r="H33" s="1">
-        <v>-0.607</v>
+        <v>-0.444</v>
       </c>
       <c r="I33" s="1">
-        <v>-0.506</v>
+        <v>-0.348</v>
       </c>
       <c r="J33" s="1">
-        <v>-0.413</v>
+        <v>-0.281</v>
       </c>
       <c r="K33" s="1">
-        <v>-0.347</v>
+        <v>-0.247</v>
       </c>
       <c r="L33" s="1">
-        <v>-0.304</v>
+        <v>-0.214</v>
       </c>
       <c r="M33" s="1">
-        <v>-0.277</v>
+        <v>-0.175</v>
       </c>
       <c r="N33" s="1">
-        <v>-0.261</v>
+        <v>-0.13</v>
       </c>
       <c r="O33" s="1">
-        <v>-0.249</v>
+        <v>-0.082</v>
       </c>
       <c r="P33" s="1">
-        <v>-0.252</v>
+        <v>-0.043</v>
       </c>
       <c r="Q33" s="1">
-        <v>-0.272</v>
+        <v>-0.029</v>
       </c>
       <c r="R33" s="1">
-        <v>-0.291</v>
+        <v>-0.038</v>
       </c>
       <c r="S33" s="1">
-        <v>-0.294</v>
+        <v>-0.045</v>
       </c>
       <c r="T33" s="1">
-        <v>-0.284</v>
+        <v>-0.035</v>
       </c>
       <c r="U33" s="1">
-        <v>-0.256</v>
+        <v>-0.029</v>
       </c>
     </row>
     <row r="34" spans="1:21">
       <c r="A34" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" s="1">
-        <v>-0.396</v>
+        <v>-0.422</v>
       </c>
       <c r="C34" s="1">
-        <v>-0.461</v>
+        <v>-0.463</v>
       </c>
       <c r="D34" s="1">
-        <v>-0.589</v>
+        <v>-0.556</v>
       </c>
       <c r="E34" s="1">
-        <v>-0.6919999999999999</v>
+        <v>-0.636</v>
       </c>
       <c r="F34" s="1">
-        <v>-0.716</v>
+        <v>-0.625</v>
       </c>
       <c r="G34" s="1">
-        <v>-0.657</v>
+        <v>-0.532</v>
       </c>
       <c r="H34" s="1">
-        <v>-0.551</v>
+        <v>-0.427</v>
       </c>
       <c r="I34" s="1">
-        <v>-0.444</v>
+        <v>-0.337</v>
       </c>
       <c r="J34" s="1">
-        <v>-0.361</v>
+        <v>-0.268</v>
       </c>
       <c r="K34" s="1">
-        <v>-0.301</v>
+        <v>-0.213</v>
       </c>
       <c r="L34" s="1">
-        <v>-0.266</v>
+        <v>-0.16</v>
       </c>
       <c r="M34" s="1">
-        <v>-0.247</v>
+        <v>-0.112</v>
       </c>
       <c r="N34" s="1">
-        <v>-0.235</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="O34" s="1">
-        <v>-0.233</v>
+        <v>-0.033</v>
       </c>
       <c r="P34" s="1">
-        <v>-0.246</v>
+        <v>-0.014</v>
       </c>
       <c r="Q34" s="1">
-        <v>-0.256</v>
+        <v>-0.015</v>
       </c>
       <c r="R34" s="1">
-        <v>-0.257</v>
+        <v>-0.026</v>
       </c>
       <c r="S34" s="1">
-        <v>-0.251</v>
+        <v>-0.032</v>
       </c>
       <c r="T34" s="1">
-        <v>-0.229</v>
+        <v>-0.028</v>
       </c>
       <c r="U34" s="1">
-        <v>-0.18</v>
+        <v>-0.026</v>
       </c>
     </row>
     <row r="35" spans="1:21">
       <c r="A35" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B35" s="1">
-        <v>-0.456</v>
+        <v>-0.482</v>
       </c>
       <c r="C35" s="1">
-        <v>-0.535</v>
+        <v>-0.554</v>
       </c>
       <c r="D35" s="1">
-        <v>-0.629</v>
+        <v>-0.627</v>
       </c>
       <c r="E35" s="1">
-        <v>-0.642</v>
+        <v>-0.601</v>
       </c>
       <c r="F35" s="1">
-        <v>-0.589</v>
+        <v>-0.504</v>
       </c>
       <c r="G35" s="1">
-        <v>-0.494</v>
+        <v>-0.396</v>
       </c>
       <c r="H35" s="1">
-        <v>-0.384</v>
+        <v>-0.305</v>
       </c>
       <c r="I35" s="1">
-        <v>-0.276</v>
+        <v>-0.213</v>
       </c>
       <c r="J35" s="1">
-        <v>-0.181</v>
+        <v>-0.118</v>
       </c>
       <c r="K35" s="1">
-        <v>-0.119</v>
+        <v>-0.043</v>
       </c>
       <c r="L35" s="1">
-        <v>-0.089</v>
+        <v>0.011</v>
       </c>
       <c r="M35" s="1">
-        <v>-0.07099999999999999</v>
+        <v>0.062</v>
       </c>
       <c r="N35" s="1">
-        <v>-0.052</v>
+        <v>0.111</v>
       </c>
       <c r="O35" s="1">
-        <v>-0.029</v>
+        <v>0.159</v>
       </c>
       <c r="P35" s="1">
-        <v>-0.005</v>
+        <v>0.192</v>
       </c>
       <c r="Q35" s="1">
-        <v>0.005</v>
+        <v>0.203</v>
       </c>
       <c r="R35" s="1">
-        <v>-0.008</v>
+        <v>0.195</v>
       </c>
       <c r="S35" s="1">
-        <v>-0.02</v>
+        <v>0.162</v>
       </c>
       <c r="T35" s="1">
-        <v>-0.006</v>
+        <v>0.123</v>
       </c>
       <c r="U35" s="1">
-        <v>0.031</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="36" spans="1:21">
       <c r="A36" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B36" s="1">
-        <v>-0.6929999999999999</v>
+        <v>-0.72</v>
       </c>
       <c r="C36" s="1">
-        <v>-0.713</v>
+        <v>-0.737</v>
       </c>
       <c r="D36" s="1">
-        <v>-0.701</v>
+        <v>-0.703</v>
       </c>
       <c r="E36" s="1">
-        <v>-0.633</v>
+        <v>-0.608</v>
       </c>
       <c r="F36" s="1">
-        <v>-0.532</v>
+        <v>-0.498</v>
       </c>
       <c r="G36" s="1">
-        <v>-0.412</v>
+        <v>-0.385</v>
       </c>
       <c r="H36" s="1">
-        <v>-0.282</v>
+        <v>-0.255</v>
       </c>
       <c r="I36" s="1">
-        <v>-0.159</v>
+        <v>-0.11</v>
       </c>
       <c r="J36" s="1">
-        <v>-0.074</v>
+        <v>0.023</v>
       </c>
       <c r="K36" s="1">
-        <v>-0.03</v>
+        <v>0.117</v>
       </c>
       <c r="L36" s="1">
-        <v>-0</v>
+        <v>0.196</v>
       </c>
       <c r="M36" s="1">
-        <v>0.038</v>
+        <v>0.274</v>
       </c>
       <c r="N36" s="1">
-        <v>0.09</v>
+        <v>0.348</v>
       </c>
       <c r="O36" s="1">
-        <v>0.141</v>
+        <v>0.411</v>
       </c>
       <c r="P36" s="1">
-        <v>0.162</v>
+        <v>0.437</v>
       </c>
       <c r="Q36" s="1">
-        <v>0.14</v>
+        <v>0.411</v>
       </c>
       <c r="R36" s="1">
-        <v>0.108</v>
+        <v>0.349</v>
       </c>
       <c r="S36" s="1">
-        <v>0.1</v>
+        <v>0.269</v>
       </c>
       <c r="T36" s="1">
-        <v>0.118</v>
+        <v>0.2</v>
       </c>
       <c r="U36" s="1">
-        <v>0.142</v>
+        <v>0.153</v>
       </c>
     </row>
     <row r="37" spans="1:21">
       <c r="A37" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B37" s="1">
-        <v>-0.612</v>
+        <v>-0.64</v>
       </c>
       <c r="C37" s="1">
-        <v>-0.5669999999999999</v>
+        <v>-0.58</v>
       </c>
       <c r="D37" s="1">
-        <v>-0.461</v>
+        <v>-0.452</v>
       </c>
       <c r="E37" s="1">
-        <v>-0.347</v>
+        <v>-0.332</v>
       </c>
       <c r="F37" s="1">
-        <v>-0.232</v>
+        <v>-0.222</v>
       </c>
       <c r="G37" s="1">
-        <v>-0.097</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="H37" s="1">
-        <v>0.044</v>
+        <v>0.08</v>
       </c>
       <c r="I37" s="1">
-        <v>0.152</v>
+        <v>0.232</v>
       </c>
       <c r="J37" s="1">
-        <v>0.217</v>
+        <v>0.351</v>
       </c>
       <c r="K37" s="1">
-        <v>0.265</v>
+        <v>0.453</v>
       </c>
       <c r="L37" s="1">
-        <v>0.337</v>
+        <v>0.574</v>
       </c>
       <c r="M37" s="1">
-        <v>0.447</v>
+        <v>0.72</v>
       </c>
       <c r="N37" s="1">
-        <v>0.549</v>
+        <v>0.832</v>
       </c>
       <c r="O37" s="1">
-        <v>0.583</v>
+        <v>0.857</v>
       </c>
       <c r="P37" s="1">
-        <v>0.54</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="Q37" s="1">
-        <v>0.46</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="R37" s="1">
-        <v>0.386</v>
+        <v>0.531</v>
       </c>
       <c r="S37" s="1">
-        <v>0.327</v>
+        <v>0.375</v>
       </c>
       <c r="T37" s="1">
-        <v>0.272</v>
+        <v>0.234</v>
       </c>
       <c r="U37" s="1">
-        <v>0.219</v>
+        <v>0.135</v>
       </c>
     </row>
     <row r="38" spans="1:21">
       <c r="A38" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B38" s="1">
-        <v>-0.5570000000000001</v>
+        <v>-0.585</v>
       </c>
       <c r="C38" s="1">
-        <v>-0.462</v>
+        <v>-0.484</v>
       </c>
       <c r="D38" s="1">
-        <v>-0.321</v>
+        <v>-0.344</v>
       </c>
       <c r="E38" s="1">
-        <v>-0.194</v>
+        <v>-0.229</v>
       </c>
       <c r="F38" s="1">
-        <v>-0.037</v>
+        <v>-0.08</v>
       </c>
       <c r="G38" s="1">
-        <v>0.134</v>
+        <v>0.112</v>
       </c>
       <c r="H38" s="1">
-        <v>0.266</v>
+        <v>0.305</v>
       </c>
       <c r="I38" s="1">
-        <v>0.343</v>
+        <v>0.462</v>
       </c>
       <c r="J38" s="1">
-        <v>0.403</v>
+        <v>0.603</v>
       </c>
       <c r="K38" s="1">
-        <v>0.505</v>
+        <v>0.779</v>
       </c>
       <c r="L38" s="1">
-        <v>0.665</v>
+        <v>0.982</v>
       </c>
       <c r="M38" s="1">
-        <v>0.8120000000000001</v>
+        <v>1.129</v>
       </c>
       <c r="N38" s="1">
-        <v>0.859</v>
+        <v>1.169</v>
       </c>
       <c r="O38" s="1">
-        <v>0.796</v>
+        <v>1.111</v>
       </c>
       <c r="P38" s="1">
-        <v>0.681</v>
+        <v>0.958</v>
       </c>
       <c r="Q38" s="1">
-        <v>0.571</v>
+        <v>0.744</v>
       </c>
       <c r="R38" s="1">
-        <v>0.475</v>
+        <v>0.533</v>
       </c>
       <c r="S38" s="1">
-        <v>0.383</v>
+        <v>0.359</v>
       </c>
       <c r="T38" s="1">
-        <v>0.297</v>
+        <v>0.237</v>
       </c>
       <c r="U38" s="1">
-        <v>0.222</v>
+        <v>0.185</v>
       </c>
     </row>
     <row r="39" spans="1:21">
       <c r="A39" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B39" s="1">
-        <v>-0.187</v>
+        <v>-0.215</v>
       </c>
       <c r="C39" s="1">
-        <v>-0.128</v>
+        <v>-0.174</v>
       </c>
       <c r="D39" s="1">
-        <v>0.006</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="E39" s="1">
-        <v>0.195</v>
+        <v>0.066</v>
       </c>
       <c r="F39" s="1">
-        <v>0.38</v>
+        <v>0.265</v>
       </c>
       <c r="G39" s="1">
-        <v>0.504</v>
+        <v>0.454</v>
       </c>
       <c r="H39" s="1">
-        <v>0.572</v>
+        <v>0.617</v>
       </c>
       <c r="I39" s="1">
-        <v>0.643</v>
+        <v>0.773</v>
       </c>
       <c r="J39" s="1">
-        <v>0.787</v>
+        <v>0.985</v>
       </c>
       <c r="K39" s="1">
-        <v>1.008</v>
+        <v>1.236</v>
       </c>
       <c r="L39" s="1">
-        <v>1.196</v>
+        <v>1.433</v>
       </c>
       <c r="M39" s="1">
-        <v>1.243</v>
+        <v>1.5</v>
       </c>
       <c r="N39" s="1">
-        <v>1.153</v>
+        <v>1.426</v>
       </c>
       <c r="O39" s="1">
-        <v>0.993</v>
+        <v>1.232</v>
       </c>
       <c r="P39" s="1">
-        <v>0.8159999999999999</v>
+        <v>0.952</v>
       </c>
       <c r="Q39" s="1">
-        <v>0.637</v>
+        <v>0.652</v>
       </c>
       <c r="R39" s="1">
-        <v>0.458</v>
+        <v>0.389</v>
       </c>
       <c r="S39" s="1">
-        <v>0.299</v>
+        <v>0.201</v>
       </c>
       <c r="T39" s="1">
-        <v>0.173</v>
+        <v>0.107</v>
       </c>
       <c r="U39" s="1">
-        <v>0.083</v>
+        <v>0.07099999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -3061,22 +3058,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update XRO plume and forecasts
</commit_message>
<xml_diff>
--- a/content/climate/XRO/XRO_ENSO_fcst.xlsx
+++ b/content/climate/XRO/XRO_ENSO_fcst.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>2023-01</t>
   </si>
@@ -135,6 +135,9 @@
   </si>
   <si>
     <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
   </si>
   <si>
     <t>Readme</t>
@@ -511,7 +514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U41"/>
+  <dimension ref="A1:U42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="21" width="10.7109375" style="1" customWidth="1"/>
@@ -519,7 +522,7 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B1" s="2">
         <v>0</v>
@@ -590,61 +593,61 @@
         <v>-0.699</v>
       </c>
       <c r="C2" s="1">
-        <v>-0.735</v>
+        <v>-0.731</v>
       </c>
       <c r="D2" s="1">
-        <v>-0.706</v>
+        <v>-0.703</v>
       </c>
       <c r="E2" s="1">
-        <v>-0.532</v>
+        <v>-0.53</v>
       </c>
       <c r="F2" s="1">
-        <v>-0.21</v>
+        <v>-0.211</v>
       </c>
       <c r="G2" s="1">
         <v>0.18</v>
       </c>
       <c r="H2" s="1">
-        <v>0.543</v>
+        <v>0.535</v>
       </c>
       <c r="I2" s="1">
-        <v>0.8129999999999999</v>
+        <v>0.805</v>
       </c>
       <c r="J2" s="1">
-        <v>1.059</v>
+        <v>1.053</v>
       </c>
       <c r="K2" s="1">
-        <v>1.395</v>
+        <v>1.37</v>
       </c>
       <c r="L2" s="1">
-        <v>1.751</v>
+        <v>1.738</v>
       </c>
       <c r="M2" s="1">
-        <v>1.983</v>
+        <v>1.993</v>
       </c>
       <c r="N2" s="1">
-        <v>2.032</v>
+        <v>2.05</v>
       </c>
       <c r="O2" s="1">
-        <v>1.924</v>
+        <v>1.931</v>
       </c>
       <c r="P2" s="1">
-        <v>1.652</v>
+        <v>1.666</v>
       </c>
       <c r="Q2" s="1">
-        <v>1.244</v>
+        <v>1.274</v>
       </c>
       <c r="R2" s="1">
-        <v>0.833</v>
+        <v>0.857</v>
       </c>
       <c r="S2" s="1">
-        <v>0.488</v>
+        <v>0.504</v>
       </c>
       <c r="T2" s="1">
-        <v>0.243</v>
+        <v>0.253</v>
       </c>
       <c r="U2" s="1">
-        <v>0.112</v>
+        <v>0.119</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -655,61 +658,61 @@
         <v>-0.492</v>
       </c>
       <c r="C3" s="1">
-        <v>-0.474</v>
+        <v>-0.476</v>
       </c>
       <c r="D3" s="1">
-        <v>-0.339</v>
+        <v>-0.345</v>
       </c>
       <c r="E3" s="1">
-        <v>-0.064</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="F3" s="1">
-        <v>0.269</v>
+        <v>0.262</v>
       </c>
       <c r="G3" s="1">
-        <v>0.5570000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="H3" s="1">
-        <v>0.78</v>
+        <v>0.754</v>
       </c>
       <c r="I3" s="1">
-        <v>0.981</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J3" s="1">
-        <v>1.22</v>
+        <v>1.172</v>
       </c>
       <c r="K3" s="1">
-        <v>1.462</v>
+        <v>1.414</v>
       </c>
       <c r="L3" s="1">
-        <v>1.602</v>
+        <v>1.552</v>
       </c>
       <c r="M3" s="1">
-        <v>1.617</v>
+        <v>1.552</v>
       </c>
       <c r="N3" s="1">
-        <v>1.522</v>
+        <v>1.446</v>
       </c>
       <c r="O3" s="1">
-        <v>1.297</v>
+        <v>1.24</v>
       </c>
       <c r="P3" s="1">
-        <v>0.972</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="Q3" s="1">
-        <v>0.628</v>
+        <v>0.617</v>
       </c>
       <c r="R3" s="1">
-        <v>0.32</v>
+        <v>0.335</v>
       </c>
       <c r="S3" s="1">
-        <v>0.096</v>
+        <v>0.119</v>
       </c>
       <c r="T3" s="1">
-        <v>-0.019</v>
+        <v>0.012</v>
       </c>
       <c r="U3" s="1">
-        <v>-0.067</v>
+        <v>-0.025</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -720,61 +723,61 @@
         <v>-0.039</v>
       </c>
       <c r="C4" s="1">
-        <v>0.025</v>
+        <v>0.02</v>
       </c>
       <c r="D4" s="1">
-        <v>0.203</v>
+        <v>0.19</v>
       </c>
       <c r="E4" s="1">
-        <v>0.43</v>
+        <v>0.414</v>
       </c>
       <c r="F4" s="1">
         <v>0.617</v>
       </c>
       <c r="G4" s="1">
-        <v>0.757</v>
+        <v>0.755</v>
       </c>
       <c r="H4" s="1">
-        <v>0.89</v>
+        <v>0.872</v>
       </c>
       <c r="I4" s="1">
-        <v>1.058</v>
+        <v>1.028</v>
       </c>
       <c r="J4" s="1">
-        <v>1.225</v>
+        <v>1.186</v>
       </c>
       <c r="K4" s="1">
-        <v>1.31</v>
+        <v>1.274</v>
       </c>
       <c r="L4" s="1">
-        <v>1.303</v>
+        <v>1.268</v>
       </c>
       <c r="M4" s="1">
-        <v>1.211</v>
+        <v>1.162</v>
       </c>
       <c r="N4" s="1">
-        <v>1.03</v>
+        <v>0.967</v>
       </c>
       <c r="O4" s="1">
-        <v>0.772</v>
+        <v>0.716</v>
       </c>
       <c r="P4" s="1">
-        <v>0.481</v>
+        <v>0.444</v>
       </c>
       <c r="Q4" s="1">
-        <v>0.203</v>
+        <v>0.185</v>
       </c>
       <c r="R4" s="1">
-        <v>-0.001</v>
+        <v>-0.014</v>
       </c>
       <c r="S4" s="1">
-        <v>-0.098</v>
+        <v>-0.113</v>
       </c>
       <c r="T4" s="1">
-        <v>-0.133</v>
+        <v>-0.141</v>
       </c>
       <c r="U4" s="1">
-        <v>-0.164</v>
+        <v>-0.174</v>
       </c>
     </row>
     <row r="5" spans="1:21">
@@ -785,61 +788,61 @@
         <v>0.162</v>
       </c>
       <c r="C5" s="1">
-        <v>0.252</v>
+        <v>0.26</v>
       </c>
       <c r="D5" s="1">
-        <v>0.44</v>
+        <v>0.457</v>
       </c>
       <c r="E5" s="1">
-        <v>0.66</v>
+        <v>0.669</v>
       </c>
       <c r="F5" s="1">
-        <v>0.861</v>
+        <v>0.867</v>
       </c>
       <c r="G5" s="1">
-        <v>1.039</v>
+        <v>1.037</v>
       </c>
       <c r="H5" s="1">
-        <v>1.213</v>
+        <v>1.197</v>
       </c>
       <c r="I5" s="1">
-        <v>1.342</v>
+        <v>1.323</v>
       </c>
       <c r="J5" s="1">
-        <v>1.388</v>
+        <v>1.366</v>
       </c>
       <c r="K5" s="1">
-        <v>1.351</v>
+        <v>1.327</v>
       </c>
       <c r="L5" s="1">
-        <v>1.242</v>
+        <v>1.208</v>
       </c>
       <c r="M5" s="1">
-        <v>1.043</v>
+        <v>1.019</v>
       </c>
       <c r="N5" s="1">
-        <v>0.756</v>
+        <v>0.75</v>
       </c>
       <c r="O5" s="1">
-        <v>0.427</v>
+        <v>0.434</v>
       </c>
       <c r="P5" s="1">
-        <v>0.112</v>
+        <v>0.122</v>
       </c>
       <c r="Q5" s="1">
-        <v>-0.137</v>
+        <v>-0.123</v>
       </c>
       <c r="R5" s="1">
-        <v>-0.261</v>
+        <v>-0.247</v>
       </c>
       <c r="S5" s="1">
-        <v>-0.305</v>
+        <v>-0.289</v>
       </c>
       <c r="T5" s="1">
-        <v>-0.359</v>
+        <v>-0.34</v>
       </c>
       <c r="U5" s="1">
-        <v>-0.448</v>
+        <v>-0.438</v>
       </c>
     </row>
     <row r="6" spans="1:21">
@@ -850,61 +853,61 @@
         <v>0.444</v>
       </c>
       <c r="C6" s="1">
-        <v>0.61</v>
+        <v>0.604</v>
       </c>
       <c r="D6" s="1">
-        <v>0.879</v>
+        <v>0.866</v>
       </c>
       <c r="E6" s="1">
-        <v>1.111</v>
+        <v>1.105</v>
       </c>
       <c r="F6" s="1">
-        <v>1.316</v>
+        <v>1.312</v>
       </c>
       <c r="G6" s="1">
-        <v>1.502</v>
+        <v>1.493</v>
       </c>
       <c r="H6" s="1">
-        <v>1.633</v>
+        <v>1.619</v>
       </c>
       <c r="I6" s="1">
-        <v>1.668</v>
+        <v>1.654</v>
       </c>
       <c r="J6" s="1">
-        <v>1.597</v>
+        <v>1.584</v>
       </c>
       <c r="K6" s="1">
-        <v>1.444</v>
+        <v>1.432</v>
       </c>
       <c r="L6" s="1">
-        <v>1.208</v>
+        <v>1.195</v>
       </c>
       <c r="M6" s="1">
-        <v>0.879</v>
+        <v>0.862</v>
       </c>
       <c r="N6" s="1">
-        <v>0.494</v>
+        <v>0.469</v>
       </c>
       <c r="O6" s="1">
-        <v>0.105</v>
+        <v>0.08</v>
       </c>
       <c r="P6" s="1">
-        <v>-0.204</v>
+        <v>-0.216</v>
       </c>
       <c r="Q6" s="1">
-        <v>-0.359</v>
+        <v>-0.356</v>
       </c>
       <c r="R6" s="1">
-        <v>-0.41</v>
+        <v>-0.397</v>
       </c>
       <c r="S6" s="1">
-        <v>-0.463</v>
+        <v>-0.453</v>
       </c>
       <c r="T6" s="1">
-        <v>-0.572</v>
+        <v>-0.5669999999999999</v>
       </c>
       <c r="U6" s="1">
-        <v>-0.697</v>
+        <v>-0.695</v>
       </c>
     </row>
     <row r="7" spans="1:21">
@@ -915,61 +918,61 @@
         <v>0.884</v>
       </c>
       <c r="C7" s="1">
-        <v>1.047</v>
+        <v>1.049</v>
       </c>
       <c r="D7" s="1">
-        <v>1.295</v>
+        <v>1.294</v>
       </c>
       <c r="E7" s="1">
-        <v>1.513</v>
+        <v>1.495</v>
       </c>
       <c r="F7" s="1">
-        <v>1.69</v>
+        <v>1.666</v>
       </c>
       <c r="G7" s="1">
-        <v>1.774</v>
+        <v>1.764</v>
       </c>
       <c r="H7" s="1">
-        <v>1.721</v>
+        <v>1.742</v>
       </c>
       <c r="I7" s="1">
-        <v>1.589</v>
+        <v>1.623</v>
       </c>
       <c r="J7" s="1">
-        <v>1.424</v>
+        <v>1.445</v>
       </c>
       <c r="K7" s="1">
-        <v>1.177</v>
+        <v>1.191</v>
       </c>
       <c r="L7" s="1">
-        <v>0.828</v>
+        <v>0.844</v>
       </c>
       <c r="M7" s="1">
-        <v>0.409</v>
+        <v>0.42</v>
       </c>
       <c r="N7" s="1">
-        <v>-0.025</v>
+        <v>-0.006</v>
       </c>
       <c r="O7" s="1">
-        <v>-0.369</v>
+        <v>-0.343</v>
       </c>
       <c r="P7" s="1">
-        <v>-0.537</v>
+        <v>-0.513</v>
       </c>
       <c r="Q7" s="1">
-        <v>-0.583</v>
+        <v>-0.5590000000000001</v>
       </c>
       <c r="R7" s="1">
-        <v>-0.643</v>
+        <v>-0.617</v>
       </c>
       <c r="S7" s="1">
-        <v>-0.786</v>
+        <v>-0.751</v>
       </c>
       <c r="T7" s="1">
-        <v>-0.954</v>
+        <v>-0.905</v>
       </c>
       <c r="U7" s="1">
-        <v>-1.002</v>
+        <v>-0.947</v>
       </c>
     </row>
     <row r="8" spans="1:21">
@@ -980,61 +983,61 @@
         <v>1.03</v>
       </c>
       <c r="C8" s="1">
-        <v>1.218</v>
+        <v>1.221</v>
       </c>
       <c r="D8" s="1">
-        <v>1.496</v>
+        <v>1.525</v>
       </c>
       <c r="E8" s="1">
-        <v>1.693</v>
+        <v>1.755</v>
       </c>
       <c r="F8" s="1">
-        <v>1.773</v>
+        <v>1.846</v>
       </c>
       <c r="G8" s="1">
-        <v>1.706</v>
+        <v>1.787</v>
       </c>
       <c r="H8" s="1">
-        <v>1.549</v>
+        <v>1.632</v>
       </c>
       <c r="I8" s="1">
-        <v>1.353</v>
+        <v>1.43</v>
       </c>
       <c r="J8" s="1">
-        <v>1.107</v>
+        <v>1.172</v>
       </c>
       <c r="K8" s="1">
-        <v>0.778</v>
+        <v>0.821</v>
       </c>
       <c r="L8" s="1">
-        <v>0.366</v>
+        <v>0.387</v>
       </c>
       <c r="M8" s="1">
-        <v>-0.074</v>
+        <v>-0.059</v>
       </c>
       <c r="N8" s="1">
-        <v>-0.424</v>
+        <v>-0.417</v>
       </c>
       <c r="O8" s="1">
-        <v>-0.588</v>
+        <v>-0.593</v>
       </c>
       <c r="P8" s="1">
-        <v>-0.622</v>
+        <v>-0.634</v>
       </c>
       <c r="Q8" s="1">
-        <v>-0.681</v>
+        <v>-0.694</v>
       </c>
       <c r="R8" s="1">
-        <v>-0.83</v>
+        <v>-0.844</v>
       </c>
       <c r="S8" s="1">
-        <v>-1.004</v>
+        <v>-1.022</v>
       </c>
       <c r="T8" s="1">
-        <v>-1.056</v>
+        <v>-1.079</v>
       </c>
       <c r="U8" s="1">
-        <v>-0.9360000000000001</v>
+        <v>-0.955</v>
       </c>
     </row>
     <row r="9" spans="1:21">
@@ -1045,61 +1048,61 @@
         <v>1.283</v>
       </c>
       <c r="C9" s="1">
-        <v>1.474</v>
+        <v>1.48</v>
       </c>
       <c r="D9" s="1">
-        <v>1.745</v>
+        <v>1.747</v>
       </c>
       <c r="E9" s="1">
-        <v>1.843</v>
+        <v>1.84</v>
       </c>
       <c r="F9" s="1">
-        <v>1.776</v>
+        <v>1.764</v>
       </c>
       <c r="G9" s="1">
-        <v>1.631</v>
+        <v>1.602</v>
       </c>
       <c r="H9" s="1">
-        <v>1.449</v>
+        <v>1.409</v>
       </c>
       <c r="I9" s="1">
-        <v>1.196</v>
+        <v>1.146</v>
       </c>
       <c r="J9" s="1">
-        <v>0.83</v>
+        <v>0.788</v>
       </c>
       <c r="K9" s="1">
-        <v>0.372</v>
+        <v>0.347</v>
       </c>
       <c r="L9" s="1">
-        <v>-0.106</v>
+        <v>-0.117</v>
       </c>
       <c r="M9" s="1">
-        <v>-0.482</v>
+        <v>-0.487</v>
       </c>
       <c r="N9" s="1">
-        <v>-0.651</v>
+        <v>-0.655</v>
       </c>
       <c r="O9" s="1">
-        <v>-0.6850000000000001</v>
+        <v>-0.6860000000000001</v>
       </c>
       <c r="P9" s="1">
-        <v>-0.744</v>
+        <v>-0.746</v>
       </c>
       <c r="Q9" s="1">
-        <v>-0.905</v>
+        <v>-0.906</v>
       </c>
       <c r="R9" s="1">
-        <v>-1.099</v>
+        <v>-1.1</v>
       </c>
       <c r="S9" s="1">
-        <v>-1.156</v>
+        <v>-1.16</v>
       </c>
       <c r="T9" s="1">
-        <v>-1.025</v>
+        <v>-1.03</v>
       </c>
       <c r="U9" s="1">
-        <v>-0.833</v>
+        <v>-0.841</v>
       </c>
     </row>
     <row r="10" spans="1:21">
@@ -1110,61 +1113,61 @@
         <v>1.534</v>
       </c>
       <c r="C10" s="1">
-        <v>1.7</v>
+        <v>1.688</v>
       </c>
       <c r="D10" s="1">
-        <v>1.887</v>
+        <v>1.845</v>
       </c>
       <c r="E10" s="1">
-        <v>1.878</v>
+        <v>1.828</v>
       </c>
       <c r="F10" s="1">
-        <v>1.73</v>
+        <v>1.695</v>
       </c>
       <c r="G10" s="1">
-        <v>1.521</v>
+        <v>1.489</v>
       </c>
       <c r="H10" s="1">
-        <v>1.25</v>
+        <v>1.213</v>
       </c>
       <c r="I10" s="1">
-        <v>0.881</v>
+        <v>0.85</v>
       </c>
       <c r="J10" s="1">
-        <v>0.432</v>
+        <v>0.413</v>
       </c>
       <c r="K10" s="1">
-        <v>-0.027</v>
+        <v>-0.04</v>
       </c>
       <c r="L10" s="1">
-        <v>-0.391</v>
+        <v>-0.398</v>
       </c>
       <c r="M10" s="1">
-        <v>-0.5669999999999999</v>
+        <v>-0.576</v>
       </c>
       <c r="N10" s="1">
-        <v>-0.612</v>
+        <v>-0.623</v>
       </c>
       <c r="O10" s="1">
-        <v>-0.68</v>
+        <v>-0.6860000000000001</v>
       </c>
       <c r="P10" s="1">
         <v>-0.837</v>
       </c>
       <c r="Q10" s="1">
-        <v>-1.011</v>
+        <v>-1.016</v>
       </c>
       <c r="R10" s="1">
-        <v>-1.061</v>
+        <v>-1.072</v>
       </c>
       <c r="S10" s="1">
-        <v>-0.9399999999999999</v>
+        <v>-0.949</v>
       </c>
       <c r="T10" s="1">
-        <v>-0.76</v>
+        <v>-0.769</v>
       </c>
       <c r="U10" s="1">
-        <v>-0.635</v>
+        <v>-0.647</v>
       </c>
     </row>
     <row r="11" spans="1:21">
@@ -1175,58 +1178,58 @@
         <v>1.574</v>
       </c>
       <c r="C11" s="1">
-        <v>1.702</v>
+        <v>1.688</v>
       </c>
       <c r="D11" s="1">
-        <v>1.793</v>
+        <v>1.757</v>
       </c>
       <c r="E11" s="1">
-        <v>1.698</v>
+        <v>1.662</v>
       </c>
       <c r="F11" s="1">
-        <v>1.51</v>
+        <v>1.474</v>
       </c>
       <c r="G11" s="1">
-        <v>1.238</v>
+        <v>1.205</v>
       </c>
       <c r="H11" s="1">
-        <v>0.886</v>
+        <v>0.87</v>
       </c>
       <c r="I11" s="1">
-        <v>0.478</v>
+        <v>0.471</v>
       </c>
       <c r="J11" s="1">
-        <v>0.067</v>
+        <v>0.054</v>
       </c>
       <c r="K11" s="1">
-        <v>-0.255</v>
+        <v>-0.273</v>
       </c>
       <c r="L11" s="1">
-        <v>-0.427</v>
+        <v>-0.434</v>
       </c>
       <c r="M11" s="1">
-        <v>-0.487</v>
+        <v>-0.49</v>
       </c>
       <c r="N11" s="1">
-        <v>-0.544</v>
+        <v>-0.548</v>
       </c>
       <c r="O11" s="1">
-        <v>-0.662</v>
+        <v>-0.667</v>
       </c>
       <c r="P11" s="1">
-        <v>-0.795</v>
+        <v>-0.804</v>
       </c>
       <c r="Q11" s="1">
-        <v>-0.833</v>
+        <v>-0.844</v>
       </c>
       <c r="R11" s="1">
-        <v>-0.738</v>
+        <v>-0.747</v>
       </c>
       <c r="S11" s="1">
-        <v>-0.596</v>
+        <v>-0.602</v>
       </c>
       <c r="T11" s="1">
-        <v>-0.501</v>
+        <v>-0.503</v>
       </c>
       <c r="U11" s="1">
         <v>-0.47</v>
@@ -1240,61 +1243,61 @@
         <v>1.867</v>
       </c>
       <c r="C12" s="1">
-        <v>1.845</v>
+        <v>1.841</v>
       </c>
       <c r="D12" s="1">
-        <v>1.718</v>
+        <v>1.707</v>
       </c>
       <c r="E12" s="1">
-        <v>1.528</v>
+        <v>1.499</v>
       </c>
       <c r="F12" s="1">
-        <v>1.264</v>
+        <v>1.223</v>
       </c>
       <c r="G12" s="1">
-        <v>0.883</v>
+        <v>0.858</v>
       </c>
       <c r="H12" s="1">
-        <v>0.424</v>
+        <v>0.413</v>
       </c>
       <c r="I12" s="1">
-        <v>-0.042</v>
+        <v>-0.043</v>
       </c>
       <c r="J12" s="1">
-        <v>-0.407</v>
+        <v>-0.402</v>
       </c>
       <c r="K12" s="1">
-        <v>-0.581</v>
+        <v>-0.574</v>
       </c>
       <c r="L12" s="1">
-        <v>-0.629</v>
+        <v>-0.622</v>
       </c>
       <c r="M12" s="1">
-        <v>-0.696</v>
+        <v>-0.6850000000000001</v>
       </c>
       <c r="N12" s="1">
-        <v>-0.847</v>
+        <v>-0.832</v>
       </c>
       <c r="O12" s="1">
-        <v>-1.018</v>
+        <v>-1.001</v>
       </c>
       <c r="P12" s="1">
-        <v>-1.067</v>
+        <v>-1.051</v>
       </c>
       <c r="Q12" s="1">
-        <v>-0.948</v>
+        <v>-0.9330000000000001</v>
       </c>
       <c r="R12" s="1">
-        <v>-0.772</v>
+        <v>-0.76</v>
       </c>
       <c r="S12" s="1">
-        <v>-0.647</v>
+        <v>-0.635</v>
       </c>
       <c r="T12" s="1">
-        <v>-0.589</v>
+        <v>-0.573</v>
       </c>
       <c r="U12" s="1">
-        <v>-0.5639999999999999</v>
+        <v>-0.548</v>
       </c>
     </row>
     <row r="13" spans="1:21">
@@ -1305,61 +1308,61 @@
         <v>1.952</v>
       </c>
       <c r="C13" s="1">
-        <v>1.872</v>
+        <v>1.873</v>
       </c>
       <c r="D13" s="1">
-        <v>1.653</v>
+        <v>1.658</v>
       </c>
       <c r="E13" s="1">
-        <v>1.332</v>
+        <v>1.35</v>
       </c>
       <c r="F13" s="1">
-        <v>0.906</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="G13" s="1">
-        <v>0.401</v>
+        <v>0.426</v>
       </c>
       <c r="H13" s="1">
-        <v>-0.114</v>
+        <v>-0.1</v>
       </c>
       <c r="I13" s="1">
-        <v>-0.522</v>
+        <v>-0.508</v>
       </c>
       <c r="J13" s="1">
-        <v>-0.726</v>
+        <v>-0.702</v>
       </c>
       <c r="K13" s="1">
-        <v>-0.785</v>
+        <v>-0.758</v>
       </c>
       <c r="L13" s="1">
-        <v>-0.866</v>
+        <v>-0.837</v>
       </c>
       <c r="M13" s="1">
-        <v>-1.046</v>
+        <v>-1.008</v>
       </c>
       <c r="N13" s="1">
-        <v>-1.243</v>
+        <v>-1.199</v>
       </c>
       <c r="O13" s="1">
-        <v>-1.297</v>
+        <v>-1.253</v>
       </c>
       <c r="P13" s="1">
-        <v>-1.154</v>
+        <v>-1.112</v>
       </c>
       <c r="Q13" s="1">
-        <v>-0.944</v>
+        <v>-0.907</v>
       </c>
       <c r="R13" s="1">
-        <v>-0.79</v>
+        <v>-0.757</v>
       </c>
       <c r="S13" s="1">
-        <v>-0.704</v>
+        <v>-0.679</v>
       </c>
       <c r="T13" s="1">
-        <v>-0.656</v>
+        <v>-0.642</v>
       </c>
       <c r="U13" s="1">
-        <v>-0.61</v>
+        <v>-0.603</v>
       </c>
     </row>
     <row r="14" spans="1:21">
@@ -1370,19 +1373,19 @@
         <v>1.757</v>
       </c>
       <c r="C14" s="1">
-        <v>1.656</v>
+        <v>1.654</v>
       </c>
       <c r="D14" s="1">
-        <v>1.369</v>
+        <v>1.363</v>
       </c>
       <c r="E14" s="1">
-        <v>0.924</v>
+        <v>0.922</v>
       </c>
       <c r="F14" s="1">
-        <v>0.368</v>
+        <v>0.38</v>
       </c>
       <c r="G14" s="1">
-        <v>-0.197</v>
+        <v>-0.186</v>
       </c>
       <c r="H14" s="1">
         <v>-0.639</v>
@@ -1391,40 +1394,40 @@
         <v>-0.844</v>
       </c>
       <c r="J14" s="1">
-        <v>-0.882</v>
+        <v>-0.88</v>
       </c>
       <c r="K14" s="1">
-        <v>-0.947</v>
+        <v>-0.948</v>
       </c>
       <c r="L14" s="1">
         <v>-1.126</v>
       </c>
       <c r="M14" s="1">
-        <v>-1.339</v>
+        <v>-1.334</v>
       </c>
       <c r="N14" s="1">
-        <v>-1.397</v>
+        <v>-1.387</v>
       </c>
       <c r="O14" s="1">
-        <v>-1.236</v>
+        <v>-1.226</v>
       </c>
       <c r="P14" s="1">
-        <v>-1.007</v>
+        <v>-0.998</v>
       </c>
       <c r="Q14" s="1">
-        <v>-0.843</v>
+        <v>-0.833</v>
       </c>
       <c r="R14" s="1">
-        <v>-0.763</v>
+        <v>-0.75</v>
       </c>
       <c r="S14" s="1">
-        <v>-0.724</v>
+        <v>-0.71</v>
       </c>
       <c r="T14" s="1">
-        <v>-0.6840000000000001</v>
+        <v>-0.667</v>
       </c>
       <c r="U14" s="1">
-        <v>-0.612</v>
+        <v>-0.592</v>
       </c>
     </row>
     <row r="15" spans="1:21">
@@ -1435,61 +1438,61 @@
         <v>1.514</v>
       </c>
       <c r="C15" s="1">
-        <v>1.318</v>
+        <v>1.306</v>
       </c>
       <c r="D15" s="1">
-        <v>0.895</v>
+        <v>0.873</v>
       </c>
       <c r="E15" s="1">
-        <v>0.354</v>
+        <v>0.328</v>
       </c>
       <c r="F15" s="1">
-        <v>-0.228</v>
+        <v>-0.252</v>
       </c>
       <c r="G15" s="1">
-        <v>-0.698</v>
+        <v>-0.712</v>
       </c>
       <c r="H15" s="1">
-        <v>-0.912</v>
+        <v>-0.911</v>
       </c>
       <c r="I15" s="1">
-        <v>-0.944</v>
+        <v>-0.9360000000000001</v>
       </c>
       <c r="J15" s="1">
-        <v>-1.007</v>
+        <v>-1.003</v>
       </c>
       <c r="K15" s="1">
-        <v>-1.196</v>
+        <v>-1.195</v>
       </c>
       <c r="L15" s="1">
-        <v>-1.417</v>
+        <v>-1.421</v>
       </c>
       <c r="M15" s="1">
-        <v>-1.478</v>
+        <v>-1.487</v>
       </c>
       <c r="N15" s="1">
-        <v>-1.313</v>
+        <v>-1.323</v>
       </c>
       <c r="O15" s="1">
-        <v>-1.073</v>
+        <v>-1.082</v>
       </c>
       <c r="P15" s="1">
-        <v>-0.894</v>
+        <v>-0.904</v>
       </c>
       <c r="Q15" s="1">
-        <v>-0.801</v>
+        <v>-0.8169999999999999</v>
       </c>
       <c r="R15" s="1">
-        <v>-0.755</v>
+        <v>-0.779</v>
       </c>
       <c r="S15" s="1">
-        <v>-0.709</v>
+        <v>-0.737</v>
       </c>
       <c r="T15" s="1">
-        <v>-0.636</v>
+        <v>-0.666</v>
       </c>
       <c r="U15" s="1">
-        <v>-0.5590000000000001</v>
+        <v>-0.582</v>
       </c>
     </row>
     <row r="16" spans="1:21">
@@ -1500,61 +1503,61 @@
         <v>1.204</v>
       </c>
       <c r="C16" s="1">
-        <v>0.922</v>
+        <v>0.92</v>
       </c>
       <c r="D16" s="1">
-        <v>0.399</v>
+        <v>0.392</v>
       </c>
       <c r="E16" s="1">
-        <v>-0.141</v>
+        <v>-0.148</v>
       </c>
       <c r="F16" s="1">
-        <v>-0.571</v>
+        <v>-0.575</v>
       </c>
       <c r="G16" s="1">
-        <v>-0.76</v>
+        <v>-0.768</v>
       </c>
       <c r="H16" s="1">
-        <v>-0.795</v>
+        <v>-0.8</v>
       </c>
       <c r="I16" s="1">
-        <v>-0.853</v>
+        <v>-0.862</v>
       </c>
       <c r="J16" s="1">
-        <v>-1.008</v>
+        <v>-1.029</v>
       </c>
       <c r="K16" s="1">
-        <v>-1.192</v>
+        <v>-1.225</v>
       </c>
       <c r="L16" s="1">
-        <v>-1.248</v>
+        <v>-1.281</v>
       </c>
       <c r="M16" s="1">
-        <v>-1.115</v>
+        <v>-1.139</v>
       </c>
       <c r="N16" s="1">
-        <v>-0.916</v>
+        <v>-0.9320000000000001</v>
       </c>
       <c r="O16" s="1">
-        <v>-0.766</v>
+        <v>-0.783</v>
       </c>
       <c r="P16" s="1">
-        <v>-0.695</v>
+        <v>-0.707</v>
       </c>
       <c r="Q16" s="1">
-        <v>-0.665</v>
+        <v>-0.67</v>
       </c>
       <c r="R16" s="1">
-        <v>-0.626</v>
+        <v>-0.631</v>
       </c>
       <c r="S16" s="1">
-        <v>-0.5570000000000001</v>
+        <v>-0.5629999999999999</v>
       </c>
       <c r="T16" s="1">
-        <v>-0.482</v>
+        <v>-0.487</v>
       </c>
       <c r="U16" s="1">
-        <v>-0.444</v>
+        <v>-0.449</v>
       </c>
     </row>
     <row r="17" spans="1:21">
@@ -1565,61 +1568,61 @@
         <v>0.823</v>
       </c>
       <c r="C17" s="1">
-        <v>0.499</v>
+        <v>0.496</v>
       </c>
       <c r="D17" s="1">
-        <v>-0.056</v>
+        <v>-0.054</v>
       </c>
       <c r="E17" s="1">
-        <v>-0.492</v>
+        <v>-0.485</v>
       </c>
       <c r="F17" s="1">
-        <v>-0.6919999999999999</v>
+        <v>-0.6850000000000001</v>
       </c>
       <c r="G17" s="1">
-        <v>-0.735</v>
+        <v>-0.728</v>
       </c>
       <c r="H17" s="1">
-        <v>-0.806</v>
+        <v>-0.798</v>
       </c>
       <c r="I17" s="1">
-        <v>-0.978</v>
+        <v>-0.97</v>
       </c>
       <c r="J17" s="1">
-        <v>-1.17</v>
+        <v>-1.167</v>
       </c>
       <c r="K17" s="1">
-        <v>-1.221</v>
+        <v>-1.222</v>
       </c>
       <c r="L17" s="1">
-        <v>-1.082</v>
+        <v>-1.084</v>
       </c>
       <c r="M17" s="1">
-        <v>-0.887</v>
+        <v>-0.885</v>
       </c>
       <c r="N17" s="1">
-        <v>-0.747</v>
+        <v>-0.743</v>
       </c>
       <c r="O17" s="1">
-        <v>-0.681</v>
+        <v>-0.6830000000000001</v>
       </c>
       <c r="P17" s="1">
-        <v>-0.659</v>
+        <v>-0.665</v>
       </c>
       <c r="Q17" s="1">
-        <v>-0.622</v>
+        <v>-0.636</v>
       </c>
       <c r="R17" s="1">
-        <v>-0.555</v>
+        <v>-0.573</v>
       </c>
       <c r="S17" s="1">
-        <v>-0.482</v>
+        <v>-0.507</v>
       </c>
       <c r="T17" s="1">
-        <v>-0.45</v>
+        <v>-0.479</v>
       </c>
       <c r="U17" s="1">
-        <v>-0.472</v>
+        <v>-0.502</v>
       </c>
     </row>
     <row r="18" spans="1:21">
@@ -1630,61 +1633,61 @@
         <v>0.29</v>
       </c>
       <c r="C18" s="1">
-        <v>-0.007</v>
+        <v>-0.015</v>
       </c>
       <c r="D18" s="1">
-        <v>-0.446</v>
+        <v>-0.456</v>
       </c>
       <c r="E18" s="1">
-        <v>-0.675</v>
+        <v>-0.677</v>
       </c>
       <c r="F18" s="1">
-        <v>-0.744</v>
+        <v>-0.746</v>
       </c>
       <c r="G18" s="1">
-        <v>-0.827</v>
+        <v>-0.823</v>
       </c>
       <c r="H18" s="1">
-        <v>-1.001</v>
+        <v>-0.988</v>
       </c>
       <c r="I18" s="1">
-        <v>-1.189</v>
+        <v>-1.168</v>
       </c>
       <c r="J18" s="1">
-        <v>-1.236</v>
+        <v>-1.214</v>
       </c>
       <c r="K18" s="1">
-        <v>-1.101</v>
+        <v>-1.08</v>
       </c>
       <c r="L18" s="1">
-        <v>-0.903</v>
+        <v>-0.886</v>
       </c>
       <c r="M18" s="1">
-        <v>-0.757</v>
+        <v>-0.745</v>
       </c>
       <c r="N18" s="1">
-        <v>-0.6860000000000001</v>
+        <v>-0.676</v>
       </c>
       <c r="O18" s="1">
-        <v>-0.649</v>
+        <v>-0.651</v>
       </c>
       <c r="P18" s="1">
-        <v>-0.603</v>
+        <v>-0.622</v>
       </c>
       <c r="Q18" s="1">
-        <v>-0.533</v>
+        <v>-0.556</v>
       </c>
       <c r="R18" s="1">
-        <v>-0.458</v>
+        <v>-0.481</v>
       </c>
       <c r="S18" s="1">
-        <v>-0.423</v>
+        <v>-0.438</v>
       </c>
       <c r="T18" s="1">
-        <v>-0.437</v>
+        <v>-0.454</v>
       </c>
       <c r="U18" s="1">
-        <v>-0.477</v>
+        <v>-0.501</v>
       </c>
     </row>
     <row r="19" spans="1:21">
@@ -1695,61 +1698,61 @@
         <v>0.228</v>
       </c>
       <c r="C19" s="1">
-        <v>0.051</v>
+        <v>0.037</v>
       </c>
       <c r="D19" s="1">
-        <v>-0.188</v>
+        <v>-0.199</v>
       </c>
       <c r="E19" s="1">
-        <v>-0.321</v>
+        <v>-0.314</v>
       </c>
       <c r="F19" s="1">
-        <v>-0.451</v>
+        <v>-0.438</v>
       </c>
       <c r="G19" s="1">
-        <v>-0.624</v>
+        <v>-0.614</v>
       </c>
       <c r="H19" s="1">
-        <v>-0.785</v>
+        <v>-0.779</v>
       </c>
       <c r="I19" s="1">
-        <v>-0.826</v>
+        <v>-0.82</v>
       </c>
       <c r="J19" s="1">
-        <v>-0.722</v>
+        <v>-0.712</v>
       </c>
       <c r="K19" s="1">
-        <v>-0.579</v>
+        <v>-0.5659999999999999</v>
       </c>
       <c r="L19" s="1">
-        <v>-0.499</v>
+        <v>-0.486</v>
       </c>
       <c r="M19" s="1">
-        <v>-0.503</v>
+        <v>-0.495</v>
       </c>
       <c r="N19" s="1">
-        <v>-0.556</v>
+        <v>-0.552</v>
       </c>
       <c r="O19" s="1">
-        <v>-0.596</v>
+        <v>-0.592</v>
       </c>
       <c r="P19" s="1">
-        <v>-0.579</v>
+        <v>-0.57</v>
       </c>
       <c r="Q19" s="1">
-        <v>-0.526</v>
+        <v>-0.521</v>
       </c>
       <c r="R19" s="1">
-        <v>-0.515</v>
+        <v>-0.51</v>
       </c>
       <c r="S19" s="1">
-        <v>-0.5620000000000001</v>
+        <v>-0.548</v>
       </c>
       <c r="T19" s="1">
-        <v>-0.624</v>
+        <v>-0.611</v>
       </c>
       <c r="U19" s="1">
-        <v>-0.641</v>
+        <v>-0.635</v>
       </c>
     </row>
     <row r="20" spans="1:21">
@@ -1760,61 +1763,61 @@
         <v>0.167</v>
       </c>
       <c r="C20" s="1">
-        <v>0.091</v>
+        <v>0.099</v>
       </c>
       <c r="D20" s="1">
-        <v>-0.032</v>
+        <v>-0.019</v>
       </c>
       <c r="E20" s="1">
-        <v>-0.173</v>
+        <v>-0.149</v>
       </c>
       <c r="F20" s="1">
-        <v>-0.337</v>
+        <v>-0.302</v>
       </c>
       <c r="G20" s="1">
-        <v>-0.461</v>
+        <v>-0.416</v>
       </c>
       <c r="H20" s="1">
-        <v>-0.476</v>
+        <v>-0.425</v>
       </c>
       <c r="I20" s="1">
-        <v>-0.388</v>
+        <v>-0.34</v>
       </c>
       <c r="J20" s="1">
-        <v>-0.291</v>
+        <v>-0.25</v>
       </c>
       <c r="K20" s="1">
-        <v>-0.263</v>
+        <v>-0.228</v>
       </c>
       <c r="L20" s="1">
-        <v>-0.313</v>
+        <v>-0.287</v>
       </c>
       <c r="M20" s="1">
-        <v>-0.409</v>
+        <v>-0.384</v>
       </c>
       <c r="N20" s="1">
-        <v>-0.486</v>
+        <v>-0.456</v>
       </c>
       <c r="O20" s="1">
-        <v>-0.492</v>
+        <v>-0.462</v>
       </c>
       <c r="P20" s="1">
-        <v>-0.46</v>
+        <v>-0.433</v>
       </c>
       <c r="Q20" s="1">
-        <v>-0.46</v>
+        <v>-0.423</v>
       </c>
       <c r="R20" s="1">
-        <v>-0.51</v>
+        <v>-0.468</v>
       </c>
       <c r="S20" s="1">
-        <v>-0.575</v>
+        <v>-0.536</v>
       </c>
       <c r="T20" s="1">
-        <v>-0.588</v>
+        <v>-0.5590000000000001</v>
       </c>
       <c r="U20" s="1">
-        <v>-0.533</v>
+        <v>-0.514</v>
       </c>
     </row>
     <row r="21" spans="1:21">
@@ -1825,61 +1828,61 @@
         <v>-0.076</v>
       </c>
       <c r="C21" s="1">
-        <v>-0.101</v>
+        <v>-0.096</v>
       </c>
       <c r="D21" s="1">
-        <v>-0.178</v>
+        <v>-0.173</v>
       </c>
       <c r="E21" s="1">
-        <v>-0.3</v>
+        <v>-0.298</v>
       </c>
       <c r="F21" s="1">
-        <v>-0.415</v>
+        <v>-0.42</v>
       </c>
       <c r="G21" s="1">
-        <v>-0.436</v>
+        <v>-0.447</v>
       </c>
       <c r="H21" s="1">
-        <v>-0.354</v>
+        <v>-0.363</v>
       </c>
       <c r="I21" s="1">
-        <v>-0.26</v>
+        <v>-0.269</v>
       </c>
       <c r="J21" s="1">
-        <v>-0.238</v>
+        <v>-0.248</v>
       </c>
       <c r="K21" s="1">
-        <v>-0.3</v>
+        <v>-0.315</v>
       </c>
       <c r="L21" s="1">
-        <v>-0.411</v>
+        <v>-0.425</v>
       </c>
       <c r="M21" s="1">
-        <v>-0.503</v>
+        <v>-0.511</v>
       </c>
       <c r="N21" s="1">
-        <v>-0.519</v>
+        <v>-0.527</v>
       </c>
       <c r="O21" s="1">
-        <v>-0.492</v>
+        <v>-0.501</v>
       </c>
       <c r="P21" s="1">
-        <v>-0.49</v>
+        <v>-0.507</v>
       </c>
       <c r="Q21" s="1">
-        <v>-0.547</v>
+        <v>-0.5669999999999999</v>
       </c>
       <c r="R21" s="1">
-        <v>-0.63</v>
+        <v>-0.642</v>
       </c>
       <c r="S21" s="1">
-        <v>-0.655</v>
+        <v>-0.664</v>
       </c>
       <c r="T21" s="1">
-        <v>-0.595</v>
+        <v>-0.613</v>
       </c>
       <c r="U21" s="1">
-        <v>-0.499</v>
+        <v>-0.523</v>
       </c>
     </row>
     <row r="22" spans="1:21">
@@ -1890,61 +1893,61 @@
         <v>-0.242</v>
       </c>
       <c r="C22" s="1">
-        <v>-0.29</v>
+        <v>-0.296</v>
       </c>
       <c r="D22" s="1">
-        <v>-0.414</v>
+        <v>-0.42</v>
       </c>
       <c r="E22" s="1">
-        <v>-0.536</v>
+        <v>-0.542</v>
       </c>
       <c r="F22" s="1">
-        <v>-0.5629999999999999</v>
+        <v>-0.5620000000000001</v>
       </c>
       <c r="G22" s="1">
-        <v>-0.482</v>
+        <v>-0.471</v>
       </c>
       <c r="H22" s="1">
-        <v>-0.381</v>
+        <v>-0.367</v>
       </c>
       <c r="I22" s="1">
-        <v>-0.348</v>
+        <v>-0.331</v>
       </c>
       <c r="J22" s="1">
-        <v>-0.403</v>
+        <v>-0.387</v>
       </c>
       <c r="K22" s="1">
-        <v>-0.505</v>
+        <v>-0.493</v>
       </c>
       <c r="L22" s="1">
-        <v>-0.576</v>
+        <v>-0.572</v>
       </c>
       <c r="M22" s="1">
-        <v>-0.575</v>
+        <v>-0.577</v>
       </c>
       <c r="N22" s="1">
-        <v>-0.536</v>
+        <v>-0.541</v>
       </c>
       <c r="O22" s="1">
-        <v>-0.531</v>
+        <v>-0.544</v>
       </c>
       <c r="P22" s="1">
-        <v>-0.586</v>
+        <v>-0.612</v>
       </c>
       <c r="Q22" s="1">
-        <v>-0.663</v>
+        <v>-0.699</v>
       </c>
       <c r="R22" s="1">
-        <v>-0.6820000000000001</v>
+        <v>-0.72</v>
       </c>
       <c r="S22" s="1">
-        <v>-0.617</v>
+        <v>-0.655</v>
       </c>
       <c r="T22" s="1">
-        <v>-0.523</v>
+        <v>-0.5590000000000001</v>
       </c>
       <c r="U22" s="1">
-        <v>-0.43</v>
+        <v>-0.46</v>
       </c>
     </row>
     <row r="23" spans="1:21">
@@ -1955,61 +1958,61 @@
         <v>-0.311</v>
       </c>
       <c r="C23" s="1">
-        <v>-0.429</v>
+        <v>-0.425</v>
       </c>
       <c r="D23" s="1">
-        <v>-0.5649999999999999</v>
+        <v>-0.5580000000000001</v>
       </c>
       <c r="E23" s="1">
-        <v>-0.551</v>
+        <v>-0.548</v>
       </c>
       <c r="F23" s="1">
         <v>-0.418</v>
       </c>
       <c r="G23" s="1">
-        <v>-0.296</v>
+        <v>-0.293</v>
       </c>
       <c r="H23" s="1">
-        <v>-0.269</v>
+        <v>-0.265</v>
       </c>
       <c r="I23" s="1">
-        <v>-0.343</v>
+        <v>-0.334</v>
       </c>
       <c r="J23" s="1">
-        <v>-0.464</v>
+        <v>-0.458</v>
       </c>
       <c r="K23" s="1">
-        <v>-0.554</v>
+        <v>-0.5590000000000001</v>
       </c>
       <c r="L23" s="1">
-        <v>-0.5620000000000001</v>
+        <v>-0.575</v>
       </c>
       <c r="M23" s="1">
-        <v>-0.526</v>
+        <v>-0.541</v>
       </c>
       <c r="N23" s="1">
-        <v>-0.524</v>
+        <v>-0.535</v>
       </c>
       <c r="O23" s="1">
-        <v>-0.585</v>
+        <v>-0.593</v>
       </c>
       <c r="P23" s="1">
-        <v>-0.658</v>
+        <v>-0.667</v>
       </c>
       <c r="Q23" s="1">
-        <v>-0.67</v>
+        <v>-0.681</v>
       </c>
       <c r="R23" s="1">
-        <v>-0.606</v>
+        <v>-0.612</v>
       </c>
       <c r="S23" s="1">
-        <v>-0.511</v>
+        <v>-0.513</v>
       </c>
       <c r="T23" s="1">
         <v>-0.419</v>
       </c>
       <c r="U23" s="1">
-        <v>-0.326</v>
+        <v>-0.324</v>
       </c>
     </row>
     <row r="24" spans="1:21">
@@ -2020,61 +2023,61 @@
         <v>-0.122</v>
       </c>
       <c r="C24" s="1">
-        <v>-0.193</v>
+        <v>-0.183</v>
       </c>
       <c r="D24" s="1">
-        <v>-0.229</v>
+        <v>-0.212</v>
       </c>
       <c r="E24" s="1">
-        <v>-0.165</v>
+        <v>-0.152</v>
       </c>
       <c r="F24" s="1">
-        <v>-0.097</v>
+        <v>-0.091</v>
       </c>
       <c r="G24" s="1">
-        <v>-0.107</v>
+        <v>-0.102</v>
       </c>
       <c r="H24" s="1">
-        <v>-0.197</v>
+        <v>-0.194</v>
       </c>
       <c r="I24" s="1">
-        <v>-0.33</v>
+        <v>-0.332</v>
       </c>
       <c r="J24" s="1">
-        <v>-0.441</v>
+        <v>-0.445</v>
       </c>
       <c r="K24" s="1">
         <v>-0.473</v>
       </c>
       <c r="L24" s="1">
-        <v>-0.457</v>
+        <v>-0.452</v>
       </c>
       <c r="M24" s="1">
-        <v>-0.47</v>
+        <v>-0.463</v>
       </c>
       <c r="N24" s="1">
-        <v>-0.54</v>
+        <v>-0.529</v>
       </c>
       <c r="O24" s="1">
-        <v>-0.625</v>
+        <v>-0.608</v>
       </c>
       <c r="P24" s="1">
-        <v>-0.648</v>
+        <v>-0.629</v>
       </c>
       <c r="Q24" s="1">
-        <v>-0.581</v>
+        <v>-0.569</v>
       </c>
       <c r="R24" s="1">
-        <v>-0.479</v>
+        <v>-0.473</v>
       </c>
       <c r="S24" s="1">
-        <v>-0.395</v>
+        <v>-0.39</v>
       </c>
       <c r="T24" s="1">
-        <v>-0.327</v>
+        <v>-0.321</v>
       </c>
       <c r="U24" s="1">
-        <v>-0.256</v>
+        <v>-0.245</v>
       </c>
     </row>
     <row r="25" spans="1:21">
@@ -2085,61 +2088,61 @@
         <v>-0.617</v>
       </c>
       <c r="C25" s="1">
-        <v>-0.589</v>
+        <v>-0.596</v>
       </c>
       <c r="D25" s="1">
-        <v>-0.492</v>
+        <v>-0.5</v>
       </c>
       <c r="E25" s="1">
-        <v>-0.379</v>
+        <v>-0.382</v>
       </c>
       <c r="F25" s="1">
         <v>-0.327</v>
       </c>
       <c r="G25" s="1">
+        <v>-0.335</v>
+      </c>
+      <c r="H25" s="1">
+        <v>-0.366</v>
+      </c>
+      <c r="I25" s="1">
+        <v>-0.385</v>
+      </c>
+      <c r="J25" s="1">
+        <v>-0.368</v>
+      </c>
+      <c r="K25" s="1">
         <v>-0.337</v>
       </c>
-      <c r="H25" s="1">
-        <v>-0.379</v>
-      </c>
-      <c r="I25" s="1">
-        <v>-0.413</v>
-      </c>
-      <c r="J25" s="1">
-        <v>-0.412</v>
-      </c>
-      <c r="K25" s="1">
-        <v>-0.381</v>
-      </c>
       <c r="L25" s="1">
+        <v>-0.327</v>
+      </c>
+      <c r="M25" s="1">
+        <v>-0.339</v>
+      </c>
+      <c r="N25" s="1">
+        <v>-0.362</v>
+      </c>
+      <c r="O25" s="1">
         <v>-0.36</v>
       </c>
-      <c r="M25" s="1">
-        <v>-0.369</v>
-      </c>
-      <c r="N25" s="1">
-        <v>-0.39</v>
-      </c>
-      <c r="O25" s="1">
-        <v>-0.387</v>
-      </c>
       <c r="P25" s="1">
-        <v>-0.35</v>
+        <v>-0.325</v>
       </c>
       <c r="Q25" s="1">
-        <v>-0.297</v>
+        <v>-0.28</v>
       </c>
       <c r="R25" s="1">
-        <v>-0.239</v>
+        <v>-0.226</v>
       </c>
       <c r="S25" s="1">
-        <v>-0.168</v>
+        <v>-0.155</v>
       </c>
       <c r="T25" s="1">
-        <v>-0.08599999999999999</v>
+        <v>-0.065</v>
       </c>
       <c r="U25" s="1">
-        <v>-0.002</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="26" spans="1:21">
@@ -2150,61 +2153,61 @@
         <v>-0.752</v>
       </c>
       <c r="C26" s="1">
-        <v>-0.647</v>
+        <v>-0.653</v>
       </c>
       <c r="D26" s="1">
-        <v>-0.491</v>
+        <v>-0.499</v>
       </c>
       <c r="E26" s="1">
-        <v>-0.412</v>
+        <v>-0.421</v>
       </c>
       <c r="F26" s="1">
-        <v>-0.419</v>
+        <v>-0.432</v>
       </c>
       <c r="G26" s="1">
-        <v>-0.475</v>
+        <v>-0.493</v>
       </c>
       <c r="H26" s="1">
-        <v>-0.526</v>
+        <v>-0.54</v>
       </c>
       <c r="I26" s="1">
-        <v>-0.519</v>
+        <v>-0.53</v>
       </c>
       <c r="J26" s="1">
-        <v>-0.474</v>
+        <v>-0.484</v>
       </c>
       <c r="K26" s="1">
-        <v>-0.455</v>
+        <v>-0.468</v>
       </c>
       <c r="L26" s="1">
-        <v>-0.482</v>
+        <v>-0.497</v>
       </c>
       <c r="M26" s="1">
-        <v>-0.524</v>
+        <v>-0.545</v>
       </c>
       <c r="N26" s="1">
-        <v>-0.529</v>
+        <v>-0.555</v>
       </c>
       <c r="O26" s="1">
-        <v>-0.476</v>
+        <v>-0.504</v>
       </c>
       <c r="P26" s="1">
-        <v>-0.401</v>
+        <v>-0.428</v>
       </c>
       <c r="Q26" s="1">
-        <v>-0.319</v>
+        <v>-0.342</v>
       </c>
       <c r="R26" s="1">
-        <v>-0.227</v>
+        <v>-0.239</v>
       </c>
       <c r="S26" s="1">
-        <v>-0.122</v>
+        <v>-0.116</v>
       </c>
       <c r="T26" s="1">
-        <v>-0.018</v>
+        <v>-0.003</v>
       </c>
       <c r="U26" s="1">
-        <v>0.066</v>
+        <v>0.077</v>
       </c>
     </row>
     <row r="27" spans="1:21">
@@ -2215,61 +2218,61 @@
         <v>-0.371</v>
       </c>
       <c r="C27" s="1">
-        <v>-0.287</v>
+        <v>-0.288</v>
       </c>
       <c r="D27" s="1">
-        <v>-0.226</v>
+        <v>-0.23</v>
       </c>
       <c r="E27" s="1">
-        <v>-0.274</v>
+        <v>-0.277</v>
       </c>
       <c r="F27" s="1">
+        <v>-0.373</v>
+      </c>
+      <c r="G27" s="1">
+        <v>-0.437</v>
+      </c>
+      <c r="H27" s="1">
+        <v>-0.424</v>
+      </c>
+      <c r="I27" s="1">
+        <v>-0.376</v>
+      </c>
+      <c r="J27" s="1">
+        <v>-0.345</v>
+      </c>
+      <c r="K27" s="1">
+        <v>-0.363</v>
+      </c>
+      <c r="L27" s="1">
+        <v>-0.408</v>
+      </c>
+      <c r="M27" s="1">
+        <v>-0.416</v>
+      </c>
+      <c r="N27" s="1">
         <v>-0.374</v>
       </c>
-      <c r="G27" s="1">
-        <v>-0.446</v>
-      </c>
-      <c r="H27" s="1">
-        <v>-0.43</v>
-      </c>
-      <c r="I27" s="1">
-        <v>-0.375</v>
-      </c>
-      <c r="J27" s="1">
-        <v>-0.359</v>
-      </c>
-      <c r="K27" s="1">
-        <v>-0.395</v>
-      </c>
-      <c r="L27" s="1">
-        <v>-0.434</v>
-      </c>
-      <c r="M27" s="1">
-        <v>-0.432</v>
-      </c>
-      <c r="N27" s="1">
-        <v>-0.382</v>
-      </c>
       <c r="O27" s="1">
-        <v>-0.317</v>
+        <v>-0.306</v>
       </c>
       <c r="P27" s="1">
-        <v>-0.257</v>
+        <v>-0.239</v>
       </c>
       <c r="Q27" s="1">
-        <v>-0.194</v>
+        <v>-0.182</v>
       </c>
       <c r="R27" s="1">
-        <v>-0.122</v>
+        <v>-0.121</v>
       </c>
       <c r="S27" s="1">
         <v>-0.054</v>
       </c>
       <c r="T27" s="1">
-        <v>0.004</v>
+        <v>0.006</v>
       </c>
       <c r="U27" s="1">
-        <v>0.058</v>
+        <v>0.064</v>
       </c>
     </row>
     <row r="28" spans="1:21">
@@ -2280,61 +2283,61 @@
         <v>0.101</v>
       </c>
       <c r="C28" s="1">
-        <v>0.077</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="D28" s="1">
-        <v>0.022</v>
+        <v>0.031</v>
       </c>
       <c r="E28" s="1">
         <v>-0.048</v>
       </c>
       <c r="F28" s="1">
+        <v>-0.097</v>
+      </c>
+      <c r="G28" s="1">
+        <v>-0.1</v>
+      </c>
+      <c r="H28" s="1">
+        <v>-0.08400000000000001</v>
+      </c>
+      <c r="I28" s="1">
+        <v>-0.07099999999999999</v>
+      </c>
+      <c r="J28" s="1">
+        <v>-0.073</v>
+      </c>
+      <c r="K28" s="1">
+        <v>-0.098</v>
+      </c>
+      <c r="L28" s="1">
+        <v>-0.114</v>
+      </c>
+      <c r="M28" s="1">
         <v>-0.101</v>
       </c>
-      <c r="G28" s="1">
-        <v>-0.11</v>
-      </c>
-      <c r="H28" s="1">
-        <v>-0.095</v>
-      </c>
-      <c r="I28" s="1">
-        <v>-0.08799999999999999</v>
-      </c>
-      <c r="J28" s="1">
-        <v>-0.099</v>
-      </c>
-      <c r="K28" s="1">
-        <v>-0.124</v>
-      </c>
-      <c r="L28" s="1">
-        <v>-0.141</v>
-      </c>
-      <c r="M28" s="1">
-        <v>-0.128</v>
-      </c>
       <c r="N28" s="1">
-        <v>-0.104</v>
+        <v>-0.082</v>
       </c>
       <c r="O28" s="1">
-        <v>-0.098</v>
+        <v>-0.076</v>
       </c>
       <c r="P28" s="1">
-        <v>-0.105</v>
+        <v>-0.079</v>
       </c>
       <c r="Q28" s="1">
-        <v>-0.108</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="R28" s="1">
-        <v>-0.099</v>
+        <v>-0.089</v>
       </c>
       <c r="S28" s="1">
-        <v>-0.067</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="T28" s="1">
-        <v>-0.022</v>
+        <v>-0.033</v>
       </c>
       <c r="U28" s="1">
-        <v>0.02</v>
+        <v>-0.001</v>
       </c>
     </row>
     <row r="29" spans="1:21">
@@ -2348,58 +2351,58 @@
         <v>-0.152</v>
       </c>
       <c r="D29" s="1">
-        <v>-0.165</v>
+        <v>-0.161</v>
       </c>
       <c r="E29" s="1">
-        <v>-0.152</v>
+        <v>-0.138</v>
       </c>
       <c r="F29" s="1">
-        <v>-0.097</v>
+        <v>-0.081</v>
       </c>
       <c r="G29" s="1">
-        <v>-0.045</v>
+        <v>-0.019</v>
       </c>
       <c r="H29" s="1">
-        <v>-0.013</v>
+        <v>0.027</v>
       </c>
       <c r="I29" s="1">
+        <v>0.052</v>
+      </c>
+      <c r="J29" s="1">
+        <v>0.066</v>
+      </c>
+      <c r="K29" s="1">
+        <v>0.074</v>
+      </c>
+      <c r="L29" s="1">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="M29" s="1">
+        <v>0.094</v>
+      </c>
+      <c r="N29" s="1">
+        <v>0.076</v>
+      </c>
+      <c r="O29" s="1">
+        <v>0.038</v>
+      </c>
+      <c r="P29" s="1">
         <v>0.006</v>
       </c>
-      <c r="J29" s="1">
-        <v>0.006</v>
-      </c>
-      <c r="K29" s="1">
-        <v>0.012</v>
-      </c>
-      <c r="L29" s="1">
-        <v>0.039</v>
-      </c>
-      <c r="M29" s="1">
-        <v>0.046</v>
-      </c>
-      <c r="N29" s="1">
-        <v>0.028</v>
-      </c>
-      <c r="O29" s="1">
-        <v>0.004</v>
-      </c>
-      <c r="P29" s="1">
-        <v>-0.012</v>
-      </c>
       <c r="Q29" s="1">
-        <v>-0.015</v>
+        <v>-0.007</v>
       </c>
       <c r="R29" s="1">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="S29" s="1">
-        <v>0.029</v>
+        <v>0.023</v>
       </c>
       <c r="T29" s="1">
-        <v>0.056</v>
+        <v>0.044</v>
       </c>
       <c r="U29" s="1">
-        <v>0.073</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="30" spans="1:21">
@@ -2410,61 +2413,61 @@
         <v>-0.054</v>
       </c>
       <c r="C30" s="1">
-        <v>-0.054</v>
+        <v>-0.062</v>
       </c>
       <c r="D30" s="1">
-        <v>-0.042</v>
+        <v>-0.055</v>
       </c>
       <c r="E30" s="1">
-        <v>-0.005</v>
+        <v>-0.017</v>
       </c>
       <c r="F30" s="1">
-        <v>0.026</v>
+        <v>0.018</v>
       </c>
       <c r="G30" s="1">
         <v>0.032</v>
       </c>
       <c r="H30" s="1">
-        <v>0.022</v>
+        <v>0.016</v>
       </c>
       <c r="I30" s="1">
-        <v>-0.001</v>
+        <v>-0.031</v>
       </c>
       <c r="J30" s="1">
-        <v>-0.018</v>
+        <v>-0.053</v>
       </c>
       <c r="K30" s="1">
-        <v>-0.014</v>
+        <v>-0.039</v>
       </c>
       <c r="L30" s="1">
-        <v>-0.006</v>
+        <v>-0.023</v>
       </c>
       <c r="M30" s="1">
-        <v>-0.021</v>
+        <v>-0.031</v>
       </c>
       <c r="N30" s="1">
-        <v>-0.06</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="O30" s="1">
-        <v>-0.108</v>
+        <v>-0.126</v>
       </c>
       <c r="P30" s="1">
-        <v>-0.143</v>
+        <v>-0.168</v>
       </c>
       <c r="Q30" s="1">
-        <v>-0.148</v>
+        <v>-0.171</v>
       </c>
       <c r="R30" s="1">
-        <v>-0.122</v>
+        <v>-0.153</v>
       </c>
       <c r="S30" s="1">
-        <v>-0.102</v>
+        <v>-0.141</v>
       </c>
       <c r="T30" s="1">
-        <v>-0.108</v>
+        <v>-0.152</v>
       </c>
       <c r="U30" s="1">
-        <v>-0.12</v>
+        <v>-0.175</v>
       </c>
     </row>
     <row r="31" spans="1:21">
@@ -2475,61 +2478,61 @@
         <v>-0.005</v>
       </c>
       <c r="C31" s="1">
-        <v>0.01</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="D31" s="1">
-        <v>0.038</v>
+        <v>0.027</v>
       </c>
       <c r="E31" s="1">
-        <v>0.057</v>
+        <v>0.036</v>
       </c>
       <c r="F31" s="1">
-        <v>0.05</v>
+        <v>0.026</v>
       </c>
       <c r="G31" s="1">
-        <v>0.012</v>
+        <v>-0.02</v>
       </c>
       <c r="H31" s="1">
-        <v>-0.048</v>
+        <v>-0.08799999999999999</v>
       </c>
       <c r="I31" s="1">
-        <v>-0.096</v>
+        <v>-0.133</v>
       </c>
       <c r="J31" s="1">
-        <v>-0.1</v>
+        <v>-0.13</v>
       </c>
       <c r="K31" s="1">
-        <v>-0.075</v>
+        <v>-0.101</v>
       </c>
       <c r="L31" s="1">
-        <v>-0.078</v>
+        <v>-0.099</v>
       </c>
       <c r="M31" s="1">
-        <v>-0.137</v>
+        <v>-0.144</v>
       </c>
       <c r="N31" s="1">
-        <v>-0.217</v>
+        <v>-0.207</v>
       </c>
       <c r="O31" s="1">
+        <v>-0.251</v>
+      </c>
+      <c r="P31" s="1">
+        <v>-0.252</v>
+      </c>
+      <c r="Q31" s="1">
+        <v>-0.233</v>
+      </c>
+      <c r="R31" s="1">
+        <v>-0.227</v>
+      </c>
+      <c r="S31" s="1">
         <v>-0.269</v>
       </c>
-      <c r="P31" s="1">
-        <v>-0.271</v>
-      </c>
-      <c r="Q31" s="1">
-        <v>-0.248</v>
-      </c>
-      <c r="R31" s="1">
-        <v>-0.244</v>
-      </c>
-      <c r="S31" s="1">
-        <v>-0.283</v>
-      </c>
       <c r="T31" s="1">
-        <v>-0.343</v>
+        <v>-0.327</v>
       </c>
       <c r="U31" s="1">
-        <v>-0.37</v>
+        <v>-0.348</v>
       </c>
     </row>
     <row r="32" spans="1:21">
@@ -2540,61 +2543,61 @@
         <v>-0.091</v>
       </c>
       <c r="C32" s="1">
-        <v>-0.081</v>
+        <v>-0.083</v>
       </c>
       <c r="D32" s="1">
-        <v>-0.074</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="E32" s="1">
-        <v>-0.102</v>
+        <v>-0.128</v>
       </c>
       <c r="F32" s="1">
-        <v>-0.177</v>
+        <v>-0.21</v>
       </c>
       <c r="G32" s="1">
+        <v>-0.301</v>
+      </c>
+      <c r="H32" s="1">
+        <v>-0.34</v>
+      </c>
+      <c r="I32" s="1">
+        <v>-0.309</v>
+      </c>
+      <c r="J32" s="1">
+        <v>-0.252</v>
+      </c>
+      <c r="K32" s="1">
+        <v>-0.22</v>
+      </c>
+      <c r="L32" s="1">
+        <v>-0.223</v>
+      </c>
+      <c r="M32" s="1">
+        <v>-0.248</v>
+      </c>
+      <c r="N32" s="1">
         <v>-0.272</v>
       </c>
-      <c r="H32" s="1">
-        <v>-0.319</v>
-      </c>
-      <c r="I32" s="1">
-        <v>-0.294</v>
-      </c>
-      <c r="J32" s="1">
-        <v>-0.234</v>
-      </c>
-      <c r="K32" s="1">
-        <v>-0.197</v>
-      </c>
-      <c r="L32" s="1">
-        <v>-0.209</v>
-      </c>
-      <c r="M32" s="1">
-        <v>-0.25</v>
-      </c>
-      <c r="N32" s="1">
-        <v>-0.28</v>
-      </c>
       <c r="O32" s="1">
-        <v>-0.27</v>
+        <v>-0.273</v>
       </c>
       <c r="P32" s="1">
-        <v>-0.244</v>
+        <v>-0.254</v>
       </c>
       <c r="Q32" s="1">
-        <v>-0.239</v>
+        <v>-0.243</v>
       </c>
       <c r="R32" s="1">
-        <v>-0.272</v>
+        <v>-0.265</v>
       </c>
       <c r="S32" s="1">
-        <v>-0.327</v>
+        <v>-0.307</v>
       </c>
       <c r="T32" s="1">
-        <v>-0.353</v>
+        <v>-0.329</v>
       </c>
       <c r="U32" s="1">
-        <v>-0.322</v>
+        <v>-0.304</v>
       </c>
     </row>
     <row r="33" spans="1:21">
@@ -2605,61 +2608,61 @@
         <v>-0.336</v>
       </c>
       <c r="C33" s="1">
-        <v>-0.323</v>
+        <v>-0.324</v>
       </c>
       <c r="D33" s="1">
-        <v>-0.35</v>
+        <v>-0.363</v>
       </c>
       <c r="E33" s="1">
-        <v>-0.447</v>
+        <v>-0.465</v>
       </c>
       <c r="F33" s="1">
-        <v>-0.54</v>
+        <v>-0.5570000000000001</v>
       </c>
       <c r="G33" s="1">
-        <v>-0.544</v>
+        <v>-0.5620000000000001</v>
       </c>
       <c r="H33" s="1">
-        <v>-0.462</v>
+        <v>-0.48</v>
       </c>
       <c r="I33" s="1">
-        <v>-0.365</v>
+        <v>-0.381</v>
       </c>
       <c r="J33" s="1">
-        <v>-0.295</v>
+        <v>-0.309</v>
       </c>
       <c r="K33" s="1">
-        <v>-0.252</v>
+        <v>-0.266</v>
       </c>
       <c r="L33" s="1">
-        <v>-0.217</v>
+        <v>-0.232</v>
       </c>
       <c r="M33" s="1">
-        <v>-0.181</v>
+        <v>-0.199</v>
       </c>
       <c r="N33" s="1">
-        <v>-0.142</v>
+        <v>-0.155</v>
       </c>
       <c r="O33" s="1">
-        <v>-0.106</v>
+        <v>-0.108</v>
       </c>
       <c r="P33" s="1">
-        <v>-0.077</v>
+        <v>-0.074</v>
       </c>
       <c r="Q33" s="1">
-        <v>-0.07000000000000001</v>
+        <v>-0.062</v>
       </c>
       <c r="R33" s="1">
+        <v>-0.074</v>
+      </c>
+      <c r="S33" s="1">
         <v>-0.08799999999999999</v>
       </c>
-      <c r="S33" s="1">
-        <v>-0.103</v>
-      </c>
       <c r="T33" s="1">
-        <v>-0.096</v>
+        <v>-0.083</v>
       </c>
       <c r="U33" s="1">
-        <v>-0.08500000000000001</v>
+        <v>-0.079</v>
       </c>
     </row>
     <row r="34" spans="1:21">
@@ -2670,61 +2673,61 @@
         <v>-0.425</v>
       </c>
       <c r="C34" s="1">
-        <v>-0.465</v>
+        <v>-0.472</v>
       </c>
       <c r="D34" s="1">
-        <v>-0.5639999999999999</v>
+        <v>-0.577</v>
       </c>
       <c r="E34" s="1">
-        <v>-0.652</v>
+        <v>-0.664</v>
       </c>
       <c r="F34" s="1">
-        <v>-0.647</v>
+        <v>-0.654</v>
       </c>
       <c r="G34" s="1">
-        <v>-0.552</v>
+        <v>-0.5590000000000001</v>
       </c>
       <c r="H34" s="1">
-        <v>-0.44</v>
+        <v>-0.443</v>
       </c>
       <c r="I34" s="1">
-        <v>-0.351</v>
+        <v>-0.355</v>
       </c>
       <c r="J34" s="1">
-        <v>-0.276</v>
+        <v>-0.293</v>
       </c>
       <c r="K34" s="1">
-        <v>-0.208</v>
+        <v>-0.239</v>
       </c>
       <c r="L34" s="1">
-        <v>-0.15</v>
+        <v>-0.189</v>
       </c>
       <c r="M34" s="1">
-        <v>-0.106</v>
+        <v>-0.141</v>
       </c>
       <c r="N34" s="1">
-        <v>-0.074</v>
+        <v>-0.092</v>
       </c>
       <c r="O34" s="1">
-        <v>-0.041</v>
+        <v>-0.047</v>
       </c>
       <c r="P34" s="1">
-        <v>-0.019</v>
+        <v>-0.032</v>
       </c>
       <c r="Q34" s="1">
-        <v>-0.013</v>
+        <v>-0.04</v>
       </c>
       <c r="R34" s="1">
-        <v>-0.014</v>
+        <v>-0.043</v>
       </c>
       <c r="S34" s="1">
-        <v>-0.01</v>
+        <v>-0.04</v>
       </c>
       <c r="T34" s="1">
-        <v>-0.008999999999999999</v>
+        <v>-0.036</v>
       </c>
       <c r="U34" s="1">
-        <v>-0.011</v>
+        <v>-0.039</v>
       </c>
     </row>
     <row r="35" spans="1:21">
@@ -2735,61 +2738,61 @@
         <v>-0.485</v>
       </c>
       <c r="C35" s="1">
-        <v>-0.553</v>
+        <v>-0.556</v>
       </c>
       <c r="D35" s="1">
-        <v>-0.624</v>
+        <v>-0.627</v>
       </c>
       <c r="E35" s="1">
-        <v>-0.601</v>
+        <v>-0.599</v>
       </c>
       <c r="F35" s="1">
-        <v>-0.507</v>
+        <v>-0.503</v>
       </c>
       <c r="G35" s="1">
-        <v>-0.404</v>
+        <v>-0.401</v>
       </c>
       <c r="H35" s="1">
-        <v>-0.315</v>
+        <v>-0.311</v>
       </c>
       <c r="I35" s="1">
-        <v>-0.224</v>
+        <v>-0.226</v>
       </c>
       <c r="J35" s="1">
-        <v>-0.139</v>
+        <v>-0.144</v>
       </c>
       <c r="K35" s="1">
-        <v>-0.067</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="L35" s="1">
-        <v>-0.006</v>
+        <v>-0.001</v>
       </c>
       <c r="M35" s="1">
-        <v>0.05</v>
+        <v>0.066</v>
       </c>
       <c r="N35" s="1">
-        <v>0.106</v>
+        <v>0.123</v>
       </c>
       <c r="O35" s="1">
-        <v>0.153</v>
+        <v>0.164</v>
       </c>
       <c r="P35" s="1">
-        <v>0.179</v>
+        <v>0.186</v>
       </c>
       <c r="Q35" s="1">
-        <v>0.185</v>
+        <v>0.187</v>
       </c>
       <c r="R35" s="1">
-        <v>0.176</v>
+        <v>0.175</v>
       </c>
       <c r="S35" s="1">
-        <v>0.151</v>
+        <v>0.141</v>
       </c>
       <c r="T35" s="1">
-        <v>0.111</v>
+        <v>0.099</v>
       </c>
       <c r="U35" s="1">
-        <v>0.077</v>
+        <v>0.067</v>
       </c>
     </row>
     <row r="36" spans="1:21">
@@ -2800,61 +2803,61 @@
         <v>-0.723</v>
       </c>
       <c r="C36" s="1">
-        <v>-0.735</v>
+        <v>-0.739</v>
       </c>
       <c r="D36" s="1">
-        <v>-0.697</v>
+        <v>-0.708</v>
       </c>
       <c r="E36" s="1">
-        <v>-0.593</v>
+        <v>-0.608</v>
       </c>
       <c r="F36" s="1">
-        <v>-0.474</v>
+        <v>-0.492</v>
       </c>
       <c r="G36" s="1">
-        <v>-0.363</v>
+        <v>-0.382</v>
       </c>
       <c r="H36" s="1">
-        <v>-0.243</v>
+        <v>-0.26</v>
       </c>
       <c r="I36" s="1">
-        <v>-0.117</v>
+        <v>-0.122</v>
       </c>
       <c r="J36" s="1">
-        <v>-0.002</v>
+        <v>-0.01</v>
       </c>
       <c r="K36" s="1">
-        <v>0.079</v>
+        <v>0.066</v>
       </c>
       <c r="L36" s="1">
-        <v>0.141</v>
+        <v>0.136</v>
       </c>
       <c r="M36" s="1">
-        <v>0.213</v>
+        <v>0.221</v>
       </c>
       <c r="N36" s="1">
-        <v>0.297</v>
+        <v>0.317</v>
       </c>
       <c r="O36" s="1">
-        <v>0.347</v>
+        <v>0.39</v>
       </c>
       <c r="P36" s="1">
-        <v>0.362</v>
+        <v>0.413</v>
       </c>
       <c r="Q36" s="1">
-        <v>0.347</v>
+        <v>0.384</v>
       </c>
       <c r="R36" s="1">
-        <v>0.292</v>
+        <v>0.324</v>
       </c>
       <c r="S36" s="1">
-        <v>0.225</v>
+        <v>0.253</v>
       </c>
       <c r="T36" s="1">
-        <v>0.172</v>
+        <v>0.183</v>
       </c>
       <c r="U36" s="1">
-        <v>0.139</v>
+        <v>0.136</v>
       </c>
     </row>
     <row r="37" spans="1:21">
@@ -2865,61 +2868,61 @@
         <v>-0.643</v>
       </c>
       <c r="C37" s="1">
-        <v>-0.581</v>
+        <v>-0.583</v>
       </c>
       <c r="D37" s="1">
-        <v>-0.45</v>
+        <v>-0.455</v>
       </c>
       <c r="E37" s="1">
-        <v>-0.333</v>
+        <v>-0.331</v>
       </c>
       <c r="F37" s="1">
-        <v>-0.231</v>
+        <v>-0.221</v>
       </c>
       <c r="G37" s="1">
-        <v>-0.106</v>
+        <v>-0.08699999999999999</v>
       </c>
       <c r="H37" s="1">
-        <v>0.047</v>
+        <v>0.073</v>
       </c>
       <c r="I37" s="1">
-        <v>0.197</v>
+        <v>0.217</v>
       </c>
       <c r="J37" s="1">
-        <v>0.313</v>
+        <v>0.335</v>
       </c>
       <c r="K37" s="1">
-        <v>0.408</v>
+        <v>0.44</v>
       </c>
       <c r="L37" s="1">
-        <v>0.52</v>
+        <v>0.575</v>
       </c>
       <c r="M37" s="1">
-        <v>0.653</v>
+        <v>0.738</v>
       </c>
       <c r="N37" s="1">
-        <v>0.759</v>
+        <v>0.85</v>
       </c>
       <c r="O37" s="1">
-        <v>0.786</v>
+        <v>0.869</v>
       </c>
       <c r="P37" s="1">
-        <v>0.739</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="Q37" s="1">
-        <v>0.639</v>
+        <v>0.707</v>
       </c>
       <c r="R37" s="1">
-        <v>0.499</v>
+        <v>0.546</v>
       </c>
       <c r="S37" s="1">
-        <v>0.348</v>
+        <v>0.389</v>
       </c>
       <c r="T37" s="1">
-        <v>0.225</v>
+        <v>0.267</v>
       </c>
       <c r="U37" s="1">
-        <v>0.145</v>
+        <v>0.178</v>
       </c>
     </row>
     <row r="38" spans="1:21">
@@ -2927,64 +2930,64 @@
         <v>36</v>
       </c>
       <c r="B38" s="1">
-        <v>-0.588</v>
+        <v>-0.5590000000000001</v>
       </c>
       <c r="C38" s="1">
-        <v>-0.484</v>
+        <v>-0.439</v>
       </c>
       <c r="D38" s="1">
-        <v>-0.344</v>
+        <v>-0.285</v>
       </c>
       <c r="E38" s="1">
-        <v>-0.238</v>
+        <v>-0.19</v>
       </c>
       <c r="F38" s="1">
-        <v>-0.099</v>
+        <v>-0.074</v>
       </c>
       <c r="G38" s="1">
-        <v>0.092</v>
+        <v>0.098</v>
       </c>
       <c r="H38" s="1">
-        <v>0.28</v>
+        <v>0.293</v>
       </c>
       <c r="I38" s="1">
-        <v>0.426</v>
+        <v>0.471</v>
       </c>
       <c r="J38" s="1">
-        <v>0.541</v>
+        <v>0.622</v>
       </c>
       <c r="K38" s="1">
-        <v>0.695</v>
+        <v>0.76</v>
       </c>
       <c r="L38" s="1">
-        <v>0.888</v>
+        <v>0.929</v>
       </c>
       <c r="M38" s="1">
-        <v>1.051</v>
+        <v>1.091</v>
       </c>
       <c r="N38" s="1">
-        <v>1.115</v>
+        <v>1.15</v>
       </c>
       <c r="O38" s="1">
-        <v>1.052</v>
+        <v>1.069</v>
       </c>
       <c r="P38" s="1">
-        <v>0.892</v>
+        <v>0.889</v>
       </c>
       <c r="Q38" s="1">
         <v>0.6889999999999999</v>
       </c>
       <c r="R38" s="1">
-        <v>0.489</v>
+        <v>0.523</v>
       </c>
       <c r="S38" s="1">
-        <v>0.331</v>
+        <v>0.363</v>
       </c>
       <c r="T38" s="1">
-        <v>0.238</v>
+        <v>0.212</v>
       </c>
       <c r="U38" s="1">
-        <v>0.201</v>
+        <v>0.108</v>
       </c>
     </row>
     <row r="39" spans="1:21">
@@ -2992,64 +2995,64 @@
         <v>37</v>
       </c>
       <c r="B39" s="1">
-        <v>-0.215</v>
+        <v>-0.273</v>
       </c>
       <c r="C39" s="1">
-        <v>-0.172</v>
+        <v>-0.205</v>
       </c>
       <c r="D39" s="1">
-        <v>-0.08400000000000001</v>
+        <v>-0.08699999999999999</v>
       </c>
       <c r="E39" s="1">
-        <v>0.057</v>
+        <v>0.068</v>
       </c>
       <c r="F39" s="1">
-        <v>0.248</v>
+        <v>0.275</v>
       </c>
       <c r="G39" s="1">
-        <v>0.445</v>
+        <v>0.514</v>
       </c>
       <c r="H39" s="1">
-        <v>0.617</v>
+        <v>0.737</v>
       </c>
       <c r="I39" s="1">
-        <v>0.779</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="J39" s="1">
-        <v>0.975</v>
+        <v>1.147</v>
       </c>
       <c r="K39" s="1">
-        <v>1.211</v>
+        <v>1.353</v>
       </c>
       <c r="L39" s="1">
-        <v>1.398</v>
+        <v>1.507</v>
       </c>
       <c r="M39" s="1">
-        <v>1.46</v>
+        <v>1.532</v>
       </c>
       <c r="N39" s="1">
         <v>1.393</v>
       </c>
       <c r="O39" s="1">
-        <v>1.214</v>
+        <v>1.151</v>
       </c>
       <c r="P39" s="1">
-        <v>0.9379999999999999</v>
+        <v>0.876</v>
       </c>
       <c r="Q39" s="1">
-        <v>0.643</v>
+        <v>0.586</v>
       </c>
       <c r="R39" s="1">
-        <v>0.396</v>
+        <v>0.312</v>
       </c>
       <c r="S39" s="1">
-        <v>0.231</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="T39" s="1">
-        <v>0.151</v>
+        <v>-0.081</v>
       </c>
       <c r="U39" s="1">
-        <v>0.124</v>
+        <v>-0.172</v>
       </c>
     </row>
     <row r="40" spans="1:21">
@@ -3057,64 +3060,64 @@
         <v>38</v>
       </c>
       <c r="B40" s="1">
-        <v>-0.007</v>
+        <v>-0.008</v>
       </c>
       <c r="C40" s="1">
-        <v>0.077</v>
+        <v>0.068</v>
       </c>
       <c r="D40" s="1">
-        <v>0.272</v>
+        <v>0.27</v>
       </c>
       <c r="E40" s="1">
-        <v>0.507</v>
+        <v>0.53</v>
       </c>
       <c r="F40" s="1">
-        <v>0.723</v>
+        <v>0.803</v>
       </c>
       <c r="G40" s="1">
-        <v>0.918</v>
+        <v>1.082</v>
       </c>
       <c r="H40" s="1">
-        <v>1.137</v>
+        <v>1.326</v>
       </c>
       <c r="I40" s="1">
-        <v>1.435</v>
+        <v>1.591</v>
       </c>
       <c r="J40" s="1">
-        <v>1.775</v>
+        <v>1.874</v>
       </c>
       <c r="K40" s="1">
-        <v>2.001</v>
+        <v>2.08</v>
       </c>
       <c r="L40" s="1">
-        <v>2.055</v>
+        <v>2.121</v>
       </c>
       <c r="M40" s="1">
-        <v>1.971</v>
+        <v>1.966</v>
       </c>
       <c r="N40" s="1">
-        <v>1.723</v>
+        <v>1.658</v>
       </c>
       <c r="O40" s="1">
-        <v>1.311</v>
+        <v>1.258</v>
       </c>
       <c r="P40" s="1">
-        <v>0.863</v>
+        <v>0.841</v>
       </c>
       <c r="Q40" s="1">
-        <v>0.478</v>
+        <v>0.452</v>
       </c>
       <c r="R40" s="1">
-        <v>0.211</v>
+        <v>0.139</v>
       </c>
       <c r="S40" s="1">
-        <v>0.067</v>
+        <v>-0.037</v>
       </c>
       <c r="T40" s="1">
-        <v>0.002</v>
+        <v>-0.11</v>
       </c>
       <c r="U40" s="1">
-        <v>-0.051</v>
+        <v>-0.168</v>
       </c>
     </row>
     <row r="41" spans="1:21">
@@ -3122,64 +3125,129 @@
         <v>39</v>
       </c>
       <c r="B41" s="1">
-        <v>0.433</v>
+        <v>0.452</v>
       </c>
       <c r="C41" s="1">
-        <v>0.582</v>
+        <v>0.602</v>
       </c>
       <c r="D41" s="1">
-        <v>0.871</v>
+        <v>0.917</v>
       </c>
       <c r="E41" s="1">
-        <v>1.199</v>
+        <v>1.29</v>
       </c>
       <c r="F41" s="1">
-        <v>1.557</v>
+        <v>1.693</v>
       </c>
       <c r="G41" s="1">
-        <v>2</v>
+        <v>2.11</v>
       </c>
       <c r="H41" s="1">
-        <v>2.569</v>
+        <v>2.498</v>
       </c>
       <c r="I41" s="1">
-        <v>3.112</v>
+        <v>2.819</v>
       </c>
       <c r="J41" s="1">
-        <v>3.388</v>
+        <v>3.015</v>
       </c>
       <c r="K41" s="1">
-        <v>3.417</v>
+        <v>3.017</v>
       </c>
       <c r="L41" s="1">
-        <v>3.285</v>
+        <v>2.784</v>
       </c>
       <c r="M41" s="1">
-        <v>2.85</v>
+        <v>2.313</v>
       </c>
       <c r="N41" s="1">
-        <v>2.08</v>
+        <v>1.715</v>
       </c>
       <c r="O41" s="1">
-        <v>1.252</v>
+        <v>1.114</v>
       </c>
       <c r="P41" s="1">
-        <v>0.57</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="Q41" s="1">
-        <v>0.097</v>
+        <v>0.132</v>
       </c>
       <c r="R41" s="1">
-        <v>-0.139</v>
+        <v>-0.119</v>
       </c>
       <c r="S41" s="1">
-        <v>-0.236</v>
+        <v>-0.221</v>
       </c>
       <c r="T41" s="1">
-        <v>-0.314</v>
+        <v>-0.289</v>
       </c>
       <c r="U41" s="1">
-        <v>-0.418</v>
+        <v>-0.379</v>
+      </c>
+    </row>
+    <row r="42" spans="1:21">
+      <c r="A42" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B42" s="1">
+        <v>1.04</v>
+      </c>
+      <c r="C42" s="1">
+        <v>1.224</v>
+      </c>
+      <c r="D42" s="1">
+        <v>1.618</v>
+      </c>
+      <c r="E42" s="1">
+        <v>2.089</v>
+      </c>
+      <c r="F42" s="1">
+        <v>2.577</v>
+      </c>
+      <c r="G42" s="1">
+        <v>2.986</v>
+      </c>
+      <c r="H42" s="1">
+        <v>3.221</v>
+      </c>
+      <c r="I42" s="1">
+        <v>3.293</v>
+      </c>
+      <c r="J42" s="1">
+        <v>3.209</v>
+      </c>
+      <c r="K42" s="1">
+        <v>2.939</v>
+      </c>
+      <c r="L42" s="1">
+        <v>2.43</v>
+      </c>
+      <c r="M42" s="1">
+        <v>1.782</v>
+      </c>
+      <c r="N42" s="1">
+        <v>1.115</v>
+      </c>
+      <c r="O42" s="1">
+        <v>0.459</v>
+      </c>
+      <c r="P42" s="1">
+        <v>-0.046</v>
+      </c>
+      <c r="Q42" s="1">
+        <v>-0.315</v>
+      </c>
+      <c r="R42" s="1">
+        <v>-0.42</v>
+      </c>
+      <c r="S42" s="1">
+        <v>-0.475</v>
+      </c>
+      <c r="T42" s="1">
+        <v>-0.59</v>
+      </c>
+      <c r="U42" s="1">
+        <v>-0.724</v>
       </c>
     </row>
   </sheetData>
@@ -3194,22 +3262,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>